<commit_message>
excel notes for backend workflow updated
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECDF416C-9436-46B5-B2AE-62EC14C96726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96B3E298-3216-4265-9916-49120E16CE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="4725" yWindow="5895" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
-    <sheet name="PROCEDURES" sheetId="2" r:id="rId1"/>
+    <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
+    <sheet name="OPERATIONS" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="163">
   <si>
     <t>MediaID</t>
   </si>
@@ -389,12 +391,423 @@
   <si>
     <t>--</t>
   </si>
+  <si>
+    <t>addMedia</t>
+  </si>
+  <si>
+    <t>if title.exists(): throw err;   else: return title</t>
+  </si>
+  <si>
+    <t>operation.name</t>
+  </si>
+  <si>
+    <t>operation.function</t>
+  </si>
+  <si>
+    <t>operation.parameters</t>
+  </si>
+  <si>
+    <t>media_title, media_type, media_genre, media_date</t>
+  </si>
+  <si>
+    <t>parameters.contraints</t>
+  </si>
+  <si>
+    <t>title/type/genre not text; date not date</t>
+  </si>
+  <si>
+    <t>Typ błędu</t>
+  </si>
+  <si>
+    <t>Gdzie</t>
+  </si>
+  <si>
+    <t>Przykład</t>
+  </si>
+  <si>
+    <t>Zły JSON / typ</t>
+  </si>
+  <si>
+    <t>schemas.py</t>
+  </si>
+  <si>
+    <t>title: int</t>
+  </si>
+  <si>
+    <t>Zły zakres</t>
+  </si>
+  <si>
+    <t>price &lt;= 0</t>
+  </si>
+  <si>
+    <t>Złamana reguła biznesowa</t>
+  </si>
+  <si>
+    <t>domain/exceptions.py</t>
+  </si>
+  <si>
+    <t>MediaAlreadyExistsError</t>
+  </si>
+  <si>
+    <t>Stan logicznie niemożliwy</t>
+  </si>
+  <si>
+    <t>CannotDeleteMediaWithCopiesError</t>
+  </si>
+  <si>
+    <t>Enum = zamknięty zbiór dozwolonych stanów / typów</t>
+  </si>
+  <si>
+    <t>Podział błędów</t>
+  </si>
+  <si>
+    <t>Czym jest enum?</t>
+  </si>
+  <si>
+    <t>MediaType = BOOK | GAME | MOVIE</t>
+  </si>
+  <si>
+    <t>CopyStatus = AVAILABLE | SOLD</t>
+  </si>
+  <si>
+    <t>EmployeeStatus = ACTIVE | INACTIVE</t>
+  </si>
+  <si>
+    <t>Czym jest Service?</t>
+  </si>
+  <si>
+    <t>Service:</t>
+  </si>
+  <si>
+    <t>NIE waliduje typów</t>
+  </si>
+  <si>
+    <t>NIE waliduje JSON</t>
+  </si>
+  <si>
+    <t>NIE sprawdza czy string jest stringiem</t>
+  </si>
+  <si>
+    <t>Service sprawdza:</t>
+  </si>
+  <si>
+    <t>istnienie / brak</t>
+  </si>
+  <si>
+    <t>relacje między bytami</t>
+  </si>
+  <si>
+    <t>reguły biznesowe</t>
+  </si>
+  <si>
+    <t>Przykład:</t>
+  </si>
+  <si>
+    <t>✔️ „Media o takim tytule już istnieje”</t>
+  </si>
+  <si>
+    <t>❌ „title nie jest stringiem”</t>
+  </si>
+  <si>
+    <t>Zero wyników w query</t>
+  </si>
+  <si>
+    <t>repositories/media_repo.py</t>
+  </si>
+  <si>
+    <t>SQL returned 0: RecordNotFound</t>
+  </si>
+  <si>
+    <t>„Jak wygląda mapowanie na HTTPS?”</t>
+  </si>
+  <si>
+    <t>Mechanicznie:</t>
+  </si>
+  <si>
+    <t>FastAPI łapie wyjątek</t>
+  </si>
+  <si>
+    <t>Twój handler:</t>
+  </si>
+  <si>
+    <t>wybiera kod HTTP</t>
+  </si>
+  <si>
+    <t>buduje JSON odpowiedzi</t>
+  </si>
+  <si>
+    <t>Domena NIE ZNA HTTP.</t>
+  </si>
+  <si>
+    <t>HTTP NIE ZNA DOMENY (poza mapowaniem).</t>
+  </si>
+  <si>
+    <t>Repository robi SQL, które rzuca:</t>
+  </si>
+  <si>
+    <t>RecordNotFound</t>
+  </si>
+  <si>
+    <t>IntegrityError</t>
+  </si>
+  <si>
+    <t>sqlite3.Error</t>
+  </si>
+  <si>
+    <t>Service decyduje:</t>
+  </si>
+  <si>
+    <t>„co to ZNACZY w domenie”</t>
+  </si>
+  <si>
+    <t>zamienia to na:</t>
+  </si>
+  <si>
+    <t>MediaNotFoundError</t>
+  </si>
+  <si>
+    <t>API mapuje:</t>
+  </si>
+  <si>
+    <t>MediaAlreadyExistsError → HTTP 409</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Weźmy przypadek </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>POST /media</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>duplikat tytułu</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HTTP 409</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>0. Założenia</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Endpoint: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>POST /media</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Procedura: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>add_media</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reguła domenowa: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">nie można dodać drugiego Media o tym samym </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>(title, media_type)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Błąd domenowy: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>MediaAlreadyExistsError</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">DB: ma UNIQUE constraint </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>(title, media_type)</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Request HTTP</t>
+  </si>
+  <si>
+    <t>Klient wysyła POST /media; Content-Type: application/json;</t>
+  </si>
+  <si>
+    <t>JSON: {"title":"Wiedźmin 3", "media_type":"GAME", "release_year":2015}</t>
+  </si>
+  <si>
+    <t>2. FastAPI - parsing + schemas</t>
+  </si>
+  <si>
+    <t>Schema sprawdza: [czy title jest str], [czy media_type pasuje do definicji w enums.py], [czy release_year to int]</t>
+  </si>
+  <si>
+    <t>FastAPI: [Odczytuje body (json)], [przekazuje je do Pydantic schema wewnątrz schemas.py]</t>
+  </si>
+  <si>
+    <t>Jeśli tu jest błąd: FastAPI zwraca 422 Unprocessable Entity, nic dalej się nie wykonuje</t>
+  </si>
+  <si>
+    <t>3. Endpoint API</t>
+  </si>
+  <si>
+    <t>Endpoint wywołuje service po otrzymaniu poprawnych danych</t>
+  </si>
+  <si>
+    <t>try:
+    result = add_media(...)
+    return 201 + response
+except DomainError:
+    (nie tutaj)</t>
+  </si>
+  <si>
+    <t>4. Service (add_media) - centrum decyzyjne</t>
+  </si>
+  <si>
+    <t>Service otrzymuje sensowne dane (schemas):</t>
+  </si>
+  <si>
+    <t>title = "Wiedźmin 3"</t>
+  </si>
+  <si>
+    <t>media_type = GAME</t>
+  </si>
+  <si>
+    <t>release_year = 2015</t>
+  </si>
+  <si>
+    <t>Sprawdza istnienie tytułu za pomocą get_by_title_type()</t>
+  </si>
+  <si>
+    <t>5. Repository - SQL</t>
+  </si>
+  <si>
+    <t>Repository wykonuje na SQL INSERT</t>
+  </si>
+  <si>
+    <t>Wyrzuca błąd techniczny w stylu IntegrityError/sqlite3.Error</t>
+  </si>
+  <si>
+    <t>6. Service - mapowanie techniczne do domenowego</t>
+  </si>
+  <si>
+    <t>Service łapie wyjątek repozytorium</t>
+  </si>
+  <si>
+    <t>except IntegrityError:
+    raise MediaAlreadyExistsError(...)</t>
+  </si>
+  <si>
+    <t>MediaAlreadyExistsError nie jest łapane w Endpointzie, tylko FastAPI(2)</t>
+  </si>
+  <si>
+    <t>7. Propagacja wyjątku do FastAPI</t>
+  </si>
+  <si>
+    <t>Handler w FastAPI konstruuje response JSON</t>
+  </si>
+  <si>
+    <t>{ "error": "MEDIA_ALREADY_EXISTS", "message": "Media with given title and type already exists"}</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +847,33 @@
       <color theme="3" tint="0.249977111117893"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -585,7 +1025,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -603,10 +1043,62 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -617,53 +1109,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1000,7 +1458,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16D3FA07-1889-4EEB-80C7-3AA9DEAD6859}">
   <dimension ref="A1:R28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.140625" style="1" bestFit="1" customWidth="1"/>
@@ -1015,23 +1473,23 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18">
       <c r="A1" s="21" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
       <c r="R1" s="2"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18">
       <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
@@ -1059,12 +1517,12 @@
       </c>
       <c r="R2" s="4"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:18">
+      <c r="A3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="4"/>
@@ -1085,14 +1543,14 @@
       </c>
       <c r="R3" s="4"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:18">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="4"/>
@@ -1105,44 +1563,44 @@
       <c r="J4" s="3"/>
       <c r="R4" s="4"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:18">
+      <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7" t="s">
+      <c r="B5" s="6"/>
+      <c r="C5" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:18" ht="15" customHeight="1">
+      <c r="A6" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="28"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="25" t="s">
+      <c r="K6" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="19" t="s">
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+    </row>
+    <row r="7" spans="1:18">
+      <c r="A7" s="24"/>
+      <c r="B7" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="8" t="s">
         <v>34</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -1158,16 +1616,16 @@
         <v>6</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="19" t="s">
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+    </row>
+    <row r="8" spans="1:18">
+      <c r="A8" s="24"/>
+      <c r="B8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -1183,16 +1641,16 @@
         <v>21</v>
       </c>
       <c r="J8" s="4"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
-      <c r="M8" s="25"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20" t="s">
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+    </row>
+    <row r="9" spans="1:18">
+      <c r="A9" s="25"/>
+      <c r="B9" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="9" t="s">
         <v>36</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -1204,26 +1662,25 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="20"/>
+    </row>
+    <row r="11" spans="1:18">
+      <c r="A11" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="F11" s="8" t="s">
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="F11" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="11"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+    </row>
+    <row r="12" spans="1:18">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
@@ -1249,14 +1706,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+    <row r="13" spans="1:18">
+      <c r="A13" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="13" t="s">
         <v>52</v>
       </c>
       <c r="F13" s="3" t="s">
@@ -1275,12 +1732,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
-      <c r="B14" s="19" t="s">
+    <row r="14" spans="1:18">
+      <c r="A14" s="24"/>
+      <c r="B14" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="14" t="s">
         <v>54</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -1295,38 +1752,38 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="19" t="s">
+    <row r="15" spans="1:18">
+      <c r="A15" s="24"/>
+      <c r="B15" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="14" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="20" t="s">
+    <row r="16" spans="1:18">
+      <c r="A16" s="25"/>
+      <c r="B16" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="28"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="13" t="s">
         <v>56</v>
       </c>
       <c r="F17" s="3" t="s">
@@ -1342,12 +1799,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
-      <c r="B18" s="19" t="s">
+    <row r="18" spans="1:9">
+      <c r="A18" s="24"/>
+      <c r="B18" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="14" t="s">
         <v>57</v>
       </c>
       <c r="F18" s="3" t="s">
@@ -1363,12 +1820,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="19" t="s">
+    <row r="19" spans="1:9">
+      <c r="A19" s="24"/>
+      <c r="B19" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="14" t="s">
         <v>67</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -1378,88 +1835,88 @@
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20" t="s">
+    <row r="20" spans="1:9">
+      <c r="A20" s="25"/>
+      <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:9">
+      <c r="A21" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="19" t="s">
+    <row r="22" spans="1:9">
+      <c r="A22" s="24"/>
+      <c r="B22" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="14" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="19" t="s">
+    <row r="23" spans="1:9">
+      <c r="A23" s="24"/>
+      <c r="B23" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="14" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20" t="s">
+    <row r="24" spans="1:9">
+      <c r="A24" s="25"/>
+      <c r="B24" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="15" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+    <row r="25" spans="1:9">
+      <c r="A25" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
-      <c r="B26" s="19" t="s">
+    <row r="26" spans="1:9">
+      <c r="A26" s="24"/>
+      <c r="B26" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
-      <c r="B27" s="19" t="s">
+    <row r="27" spans="1:9">
+      <c r="A27" s="24"/>
+      <c r="B27" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="16" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="20" t="s">
+    <row r="28" spans="1:9">
+      <c r="A28" s="25"/>
+      <c r="B28" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="15" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1480,4 +1937,1023 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{183FBF69-F40B-4D82-939D-3AFD7BBD6803}">
+  <dimension ref="A1:K72"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="4"/>
+      <c r="H2" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="28"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="E21" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="30"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="C28" s="18"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" s="33"/>
+      <c r="C29" s="33"/>
+      <c r="E29" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="E30" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="E31" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="32"/>
+      <c r="C33" s="32"/>
+      <c r="E33" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="E34" s="30" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="30"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="E35" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="E36" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B38" s="32"/>
+      <c r="C38" s="32"/>
+      <c r="E38" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="E39" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="30"/>
+    </row>
+    <row r="40" spans="1:9" ht="15" customHeight="1">
+      <c r="A40" s="19"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="E40" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="F40" s="31"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="31"/>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" s="32"/>
+      <c r="C41" s="32"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="31"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="32"/>
+      <c r="C42" s="32"/>
+      <c r="E42" s="31"/>
+      <c r="F42" s="31"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="31"/>
+      <c r="I42" s="31"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="32"/>
+      <c r="C43" s="32"/>
+      <c r="E43" s="31"/>
+      <c r="F43" s="31"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="31"/>
+      <c r="I43" s="31"/>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="32" t="s">
+        <v>105</v>
+      </c>
+      <c r="B44" s="32"/>
+      <c r="C44" s="32"/>
+      <c r="E44" s="31"/>
+      <c r="F44" s="31"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="31"/>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="19"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="29"/>
+      <c r="H45" s="29"/>
+      <c r="I45" s="29"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="B46" s="32"/>
+      <c r="C46" s="32"/>
+      <c r="E46" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="B47" s="32"/>
+      <c r="C47" s="32"/>
+      <c r="E47" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="F47" s="30"/>
+      <c r="G47" s="30"/>
+      <c r="H47" s="30"/>
+      <c r="I47" s="30"/>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B48" s="32"/>
+      <c r="C48" s="32"/>
+      <c r="E48" s="30" t="s">
+        <v>149</v>
+      </c>
+      <c r="F48" s="30"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="30"/>
+      <c r="I48" s="30"/>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="19"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="E49" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="F49" s="30"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="30"/>
+      <c r="I49" s="30"/>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="B50" s="32"/>
+      <c r="C50" s="32"/>
+      <c r="E50" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="F50" s="30"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="30"/>
+      <c r="I50" s="30"/>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="B51" s="32"/>
+      <c r="C51" s="32"/>
+      <c r="E51" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
+      <c r="I51" s="30"/>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="B52" s="32"/>
+      <c r="C52" s="32"/>
+      <c r="E52" s="29"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="29"/>
+      <c r="H52" s="29"/>
+      <c r="I52" s="29"/>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" s="32"/>
+      <c r="C53" s="32"/>
+      <c r="E53" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="29"/>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="32"/>
+      <c r="B54" s="32"/>
+      <c r="C54" s="32"/>
+      <c r="E54" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="F54" s="30"/>
+      <c r="G54" s="30"/>
+      <c r="H54" s="30"/>
+      <c r="I54" s="30"/>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="B55" s="32"/>
+      <c r="C55" s="32"/>
+      <c r="E55" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="F55" s="30"/>
+      <c r="G55" s="30"/>
+      <c r="H55" s="30"/>
+      <c r="I55" s="30"/>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="B56" s="32"/>
+      <c r="C56" s="32"/>
+      <c r="E56" s="29"/>
+      <c r="F56" s="29"/>
+      <c r="G56" s="29"/>
+      <c r="H56" s="29"/>
+      <c r="I56" s="29"/>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="B57" s="32"/>
+      <c r="C57" s="32"/>
+      <c r="E57" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="F57" s="29"/>
+      <c r="G57" s="29"/>
+      <c r="H57" s="29"/>
+      <c r="I57" s="29"/>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B58" s="32"/>
+      <c r="C58" s="32"/>
+      <c r="E58" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="F58" s="30"/>
+      <c r="G58" s="30"/>
+      <c r="H58" s="30"/>
+      <c r="I58" s="30"/>
+    </row>
+    <row r="59" spans="1:9" ht="15" customHeight="1">
+      <c r="A59" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="B59" s="32"/>
+      <c r="C59" s="32"/>
+      <c r="E59" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="F59" s="31"/>
+      <c r="G59" s="31"/>
+      <c r="H59" s="31"/>
+      <c r="I59" s="31"/>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="32"/>
+      <c r="B60" s="32"/>
+      <c r="C60" s="32"/>
+      <c r="E60" s="31"/>
+      <c r="F60" s="31"/>
+      <c r="G60" s="31"/>
+      <c r="H60" s="31"/>
+      <c r="I60" s="31"/>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B61" s="32"/>
+      <c r="C61" s="32"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="29"/>
+      <c r="G61" s="29"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="29"/>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="B62" s="32"/>
+      <c r="C62" s="32"/>
+      <c r="E62" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F62" s="29"/>
+      <c r="G62" s="29"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="29"/>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="E63" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="F63" s="30"/>
+      <c r="G63" s="30"/>
+      <c r="H63" s="30"/>
+      <c r="I63" s="30"/>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="B64" s="33"/>
+      <c r="C64" s="33"/>
+      <c r="E64" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="F64" s="30"/>
+      <c r="G64" s="30"/>
+      <c r="H64" s="30"/>
+      <c r="I64" s="30"/>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B65" s="32"/>
+      <c r="C65" s="32"/>
+      <c r="E65" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="F65" s="30"/>
+      <c r="G65" s="30"/>
+      <c r="H65" s="30"/>
+      <c r="I65" s="30"/>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="B66" s="32"/>
+      <c r="C66" s="32"/>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" s="19"/>
+      <c r="B67" s="19"/>
+      <c r="C67" s="19"/>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="B68" s="32"/>
+      <c r="C68" s="32"/>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="B69" s="32"/>
+      <c r="C69" s="32"/>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="B70" s="32"/>
+      <c r="C70" s="32"/>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="B71" s="32"/>
+      <c r="C71" s="32"/>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="B72" s="32"/>
+      <c r="C72" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="83">
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="E35:I35"/>
+    <mergeCell ref="E40:I44"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="E55:I55"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="E46:I46"/>
+    <mergeCell ref="E47:I47"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="E49:I49"/>
+    <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="E52:I52"/>
+    <mergeCell ref="E53:I53"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="E63:I63"/>
+    <mergeCell ref="E64:I64"/>
+    <mergeCell ref="E65:I65"/>
+    <mergeCell ref="E56:I56"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="E61:I61"/>
+    <mergeCell ref="E59:I60"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update media schema, API, and app version to 0.6.7
- Renamed media table columns and made release_year/publisher required
- Updated models, repositories, and schemas to match new schema
- API now enforces required fields and validation for media
- Services require release_year and publisher for media creation
- Added root endpoint and bumped FastAPI app version to 0.6.7
- Removed database file from project content; updated Excel file
- Cleaned up documentation and comments in schemas.py
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96B3E298-3216-4265-9916-49120E16CE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{244E2E4C-8291-4A02-A4D3-01E50CE28B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4725" yWindow="5895" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="43050" yWindow="540" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
     <sheet name="OPERATIONS" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="178">
   <si>
     <t>MediaID</t>
   </si>
@@ -802,12 +801,60 @@
   <si>
     <t>{ "error": "MEDIA_ALREADY_EXISTS", "message": "Media with given title and type already exists"}</t>
   </si>
+  <si>
+    <t>ITEMS</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>Publisher</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Wiedzmin</t>
+  </si>
+  <si>
+    <t>GAME</t>
+  </si>
+  <si>
+    <t>CDPR</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>COUNT(*)</t>
+  </si>
+  <si>
+    <t>GET /copies</t>
+  </si>
+  <si>
+    <t>AVAILABLE</t>
+  </si>
+  <si>
+    <t>SOLD</t>
+  </si>
+  <si>
+    <t>Cyberpunk</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -875,16 +922,40 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1021,11 +1092,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1109,22 +1272,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="10" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1941,45 +2131,47 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{183FBF69-F40B-4D82-939D-3AFD7BBD6803}">
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:M72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
       <c r="H1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:13">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>28</v>
+      <c r="B2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E2" t="s">
+        <v>167</v>
       </c>
       <c r="F2" s="4"/>
       <c r="H2" s="17" t="s">
@@ -1995,7 +2187,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -2024,7 +2216,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:13">
       <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
@@ -2033,23 +2225,31 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:13">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="26" t="s">
+    <row r="6" spans="1:13" ht="15.75" thickBot="1">
+      <c r="A6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="28"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="49"/>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="H6" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -2063,8 +2263,26 @@
         <v>6</v>
       </c>
       <c r="E7" s="4"/>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="H7" s="36" t="s">
+        <v>164</v>
+      </c>
+      <c r="I7" s="37" t="s">
+        <v>165</v>
+      </c>
+      <c r="J7" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="K7" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="L7" s="42" t="s">
+        <v>168</v>
+      </c>
+      <c r="M7" s="43" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -2078,8 +2296,26 @@
         <v>21</v>
       </c>
       <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="H8" s="39" t="s">
+        <v>169</v>
+      </c>
+      <c r="I8" s="40" t="s">
+        <v>170</v>
+      </c>
+      <c r="J8" s="40">
+        <v>2015</v>
+      </c>
+      <c r="K8" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="L8" s="44">
+        <v>5</v>
+      </c>
+      <c r="M8" s="45">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -2089,15 +2325,33 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="H9" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="I9" s="40" t="s">
+        <v>170</v>
+      </c>
+      <c r="J9" s="40">
+        <v>2020</v>
+      </c>
+      <c r="K9" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="L9" s="44">
+        <v>10</v>
+      </c>
+      <c r="M9" s="45">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11" s="26" t="s">
         <v>7</v>
       </c>
@@ -2105,8 +2359,20 @@
       <c r="C11" s="27"/>
       <c r="D11" s="27"/>
       <c r="E11" s="28"/>
-    </row>
-    <row r="12" spans="1:11">
+      <c r="J11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1">
       <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
@@ -2122,8 +2388,23 @@
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:11">
+      <c r="I12" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="L12" t="s">
+        <v>175</v>
+      </c>
+      <c r="M12">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -2139,8 +2420,20 @@
       <c r="E13" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" spans="1:11">
+      <c r="J13">
+        <v>2</v>
+      </c>
+      <c r="K13" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="L13" t="s">
+        <v>175</v>
+      </c>
+      <c r="M13">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
@@ -2152,15 +2445,39 @@
       <c r="E14" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" spans="1:11">
+      <c r="J14">
+        <v>3</v>
+      </c>
+      <c r="K14" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="L14" t="s">
+        <v>176</v>
+      </c>
+      <c r="M14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" thickBot="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="J15">
+        <v>4</v>
+      </c>
+      <c r="K15" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="L15" t="s">
+        <v>175</v>
+      </c>
+      <c r="M15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1">
       <c r="A16" s="26" t="s">
         <v>12</v>
       </c>
@@ -2168,8 +2485,20 @@
       <c r="C16" s="27"/>
       <c r="D16" s="28"/>
       <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="J16">
+        <v>5</v>
+      </c>
+      <c r="K16" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="L16" t="s">
+        <v>175</v>
+      </c>
+      <c r="M16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
@@ -2183,8 +2512,15 @@
         <v>15</v>
       </c>
       <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="J17" t="s">
+        <v>173</v>
+      </c>
+      <c r="L17">
+        <f>COUNTIF(L12:L16, "AVAILABLE")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
@@ -2199,7 +2535,7 @@
       </c>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:12">
       <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
@@ -2208,28 +2544,28 @@
       <c r="D19" s="3"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:12">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="34" t="s">
+    <row r="21" spans="1:12">
+      <c r="A21" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="E21" s="29" t="s">
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="E21" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="29"/>
-      <c r="I21" s="29"/>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="30"/>
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22" t="s">
         <v>78</v>
       </c>
@@ -2239,15 +2575,15 @@
       <c r="C22" t="s">
         <v>80</v>
       </c>
-      <c r="E22" s="29" t="s">
+      <c r="E22" s="30" t="s">
         <v>131</v>
       </c>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="29"/>
-    </row>
-    <row r="23" spans="1:9">
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="30"/>
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23" s="18" t="s">
         <v>81</v>
       </c>
@@ -2257,15 +2593,15 @@
       <c r="C23" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E23" s="30" t="s">
+      <c r="E23" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-    </row>
-    <row r="24" spans="1:9">
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" s="18" t="s">
         <v>84</v>
       </c>
@@ -2275,15 +2611,15 @@
       <c r="C24" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="30" t="s">
+      <c r="E24" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-    </row>
-    <row r="25" spans="1:9">
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" s="18" t="s">
         <v>86</v>
       </c>
@@ -2293,15 +2629,15 @@
       <c r="C25" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="30" t="s">
+      <c r="E25" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-    </row>
-    <row r="26" spans="1:9">
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" s="18" t="s">
         <v>89</v>
       </c>
@@ -2311,15 +2647,15 @@
       <c r="C26" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="30" t="s">
+      <c r="E26" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-    </row>
-    <row r="27" spans="1:9">
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" s="18" t="s">
         <v>109</v>
       </c>
@@ -2329,75 +2665,75 @@
       <c r="C27" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="E27" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
-    </row>
-    <row r="28" spans="1:9">
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+    </row>
+    <row r="28" spans="1:12">
       <c r="C28" s="18"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29"/>
-      <c r="I28" s="29"/>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" s="33" t="s">
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="B29" s="33"/>
-      <c r="C29" s="33"/>
-      <c r="E29" s="29" t="s">
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="E29" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="29"/>
-      <c r="I29" s="29"/>
-    </row>
-    <row r="30" spans="1:9">
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30" s="32" t="s">
         <v>91</v>
       </c>
       <c r="B30" s="32"/>
       <c r="C30" s="32"/>
-      <c r="E30" s="30" t="s">
+      <c r="E30" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-    </row>
-    <row r="31" spans="1:9">
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" s="32" t="s">
         <v>94</v>
       </c>
       <c r="B31" s="32"/>
       <c r="C31" s="32"/>
-      <c r="E31" s="30" t="s">
+      <c r="E31" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-    </row>
-    <row r="32" spans="1:9">
+      <c r="F31" s="33"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" s="32" t="s">
         <v>95</v>
       </c>
       <c r="B32" s="32"/>
       <c r="C32" s="32"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="32" t="s">
@@ -2405,36 +2741,36 @@
       </c>
       <c r="B33" s="32"/>
       <c r="C33" s="32"/>
-      <c r="E33" s="29" t="s">
+      <c r="E33" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="F33" s="29"/>
-      <c r="G33" s="29"/>
-      <c r="H33" s="29"/>
-      <c r="I33" s="29"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
     </row>
     <row r="34" spans="1:9">
-      <c r="E34" s="30" t="s">
+      <c r="E34" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-      <c r="I34" s="30"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="33"/>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="B35" s="33"/>
-      <c r="C35" s="33"/>
-      <c r="E35" s="30" t="s">
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="E35" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="F35" s="30"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
-      <c r="I35" s="30"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="33"/>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="32" t="s">
@@ -2442,13 +2778,13 @@
       </c>
       <c r="B36" s="32"/>
       <c r="C36" s="32"/>
-      <c r="E36" s="30" t="s">
+      <c r="E36" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="32" t="s">
@@ -2456,11 +2792,11 @@
       </c>
       <c r="B37" s="32"/>
       <c r="C37" s="32"/>
-      <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="29"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="29"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="32" t="s">
@@ -2468,13 +2804,13 @@
       </c>
       <c r="B38" s="32"/>
       <c r="C38" s="32"/>
-      <c r="E38" s="29" t="s">
+      <c r="E38" s="30" t="s">
         <v>144</v>
       </c>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="32" t="s">
@@ -2482,25 +2818,25 @@
       </c>
       <c r="B39" s="32"/>
       <c r="C39" s="32"/>
-      <c r="E39" s="30" t="s">
+      <c r="E39" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="30"/>
-      <c r="I39" s="30"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
     </row>
     <row r="40" spans="1:9" ht="15" customHeight="1">
       <c r="A40" s="19"/>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="F40" s="31"/>
-      <c r="G40" s="31"/>
-      <c r="H40" s="31"/>
-      <c r="I40" s="31"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="34"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="34"/>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="32" t="s">
@@ -2508,11 +2844,11 @@
       </c>
       <c r="B41" s="32"/>
       <c r="C41" s="32"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="31"/>
+      <c r="E41" s="34"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="34"/>
+      <c r="H41" s="34"/>
+      <c r="I41" s="34"/>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="32" t="s">
@@ -2520,11 +2856,11 @@
       </c>
       <c r="B42" s="32"/>
       <c r="C42" s="32"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="34"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="34"/>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="32" t="s">
@@ -2532,11 +2868,11 @@
       </c>
       <c r="B43" s="32"/>
       <c r="C43" s="32"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="31"/>
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="34"/>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="32" t="s">
@@ -2544,21 +2880,21 @@
       </c>
       <c r="B44" s="32"/>
       <c r="C44" s="32"/>
-      <c r="E44" s="31"/>
-      <c r="F44" s="31"/>
-      <c r="G44" s="31"/>
-      <c r="H44" s="31"/>
-      <c r="I44" s="31"/>
+      <c r="E44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="34"/>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" s="19"/>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="29"/>
-      <c r="H45" s="29"/>
-      <c r="I45" s="29"/>
+      <c r="E45" s="30"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="32" t="s">
@@ -2566,13 +2902,13 @@
       </c>
       <c r="B46" s="32"/>
       <c r="C46" s="32"/>
-      <c r="E46" s="29" t="s">
+      <c r="E46" s="30" t="s">
         <v>147</v>
       </c>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="29"/>
-      <c r="I46" s="29"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="30"/>
+      <c r="H46" s="30"/>
+      <c r="I46" s="30"/>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="32" t="s">
@@ -2580,13 +2916,13 @@
       </c>
       <c r="B47" s="32"/>
       <c r="C47" s="32"/>
-      <c r="E47" s="30" t="s">
+      <c r="E47" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="30"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="32" t="s">
@@ -2594,25 +2930,25 @@
       </c>
       <c r="B48" s="32"/>
       <c r="C48" s="32"/>
-      <c r="E48" s="30" t="s">
+      <c r="E48" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
-      <c r="I48" s="30"/>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="33"/>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" s="19"/>
       <c r="B49" s="19"/>
       <c r="C49" s="19"/>
-      <c r="E49" s="30" t="s">
+      <c r="E49" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="F49" s="30"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="30"/>
-      <c r="I49" s="30"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="33"/>
+      <c r="I49" s="33"/>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" s="32" t="s">
@@ -2620,13 +2956,13 @@
       </c>
       <c r="B50" s="32"/>
       <c r="C50" s="32"/>
-      <c r="E50" s="30" t="s">
+      <c r="E50" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="F50" s="30"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="30"/>
-      <c r="I50" s="30"/>
+      <c r="F50" s="33"/>
+      <c r="G50" s="33"/>
+      <c r="H50" s="33"/>
+      <c r="I50" s="33"/>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" s="32" t="s">
@@ -2634,13 +2970,13 @@
       </c>
       <c r="B51" s="32"/>
       <c r="C51" s="32"/>
-      <c r="E51" s="30" t="s">
+      <c r="E51" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
-      <c r="I51" s="30"/>
+      <c r="F51" s="33"/>
+      <c r="G51" s="33"/>
+      <c r="H51" s="33"/>
+      <c r="I51" s="33"/>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="32" t="s">
@@ -2648,11 +2984,11 @@
       </c>
       <c r="B52" s="32"/>
       <c r="C52" s="32"/>
-      <c r="E52" s="29"/>
-      <c r="F52" s="29"/>
-      <c r="G52" s="29"/>
-      <c r="H52" s="29"/>
-      <c r="I52" s="29"/>
+      <c r="E52" s="30"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="30"/>
+      <c r="H52" s="30"/>
+      <c r="I52" s="30"/>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" s="32" t="s">
@@ -2660,25 +2996,25 @@
       </c>
       <c r="B53" s="32"/>
       <c r="C53" s="32"/>
-      <c r="E53" s="29" t="s">
+      <c r="E53" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="F53" s="29"/>
-      <c r="G53" s="29"/>
-      <c r="H53" s="29"/>
-      <c r="I53" s="29"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="30"/>
+      <c r="H53" s="30"/>
+      <c r="I53" s="30"/>
     </row>
     <row r="54" spans="1:9">
       <c r="A54" s="32"/>
       <c r="B54" s="32"/>
       <c r="C54" s="32"/>
-      <c r="E54" s="30" t="s">
+      <c r="E54" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="F54" s="30"/>
-      <c r="G54" s="30"/>
-      <c r="H54" s="30"/>
-      <c r="I54" s="30"/>
+      <c r="F54" s="33"/>
+      <c r="G54" s="33"/>
+      <c r="H54" s="33"/>
+      <c r="I54" s="33"/>
     </row>
     <row r="55" spans="1:9">
       <c r="A55" s="32" t="s">
@@ -2686,13 +3022,13 @@
       </c>
       <c r="B55" s="32"/>
       <c r="C55" s="32"/>
-      <c r="E55" s="30" t="s">
+      <c r="E55" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="F55" s="30"/>
-      <c r="G55" s="30"/>
-      <c r="H55" s="30"/>
-      <c r="I55" s="30"/>
+      <c r="F55" s="33"/>
+      <c r="G55" s="33"/>
+      <c r="H55" s="33"/>
+      <c r="I55" s="33"/>
     </row>
     <row r="56" spans="1:9">
       <c r="A56" s="32" t="s">
@@ -2700,11 +3036,11 @@
       </c>
       <c r="B56" s="32"/>
       <c r="C56" s="32"/>
-      <c r="E56" s="29"/>
-      <c r="F56" s="29"/>
-      <c r="G56" s="29"/>
-      <c r="H56" s="29"/>
-      <c r="I56" s="29"/>
+      <c r="E56" s="30"/>
+      <c r="F56" s="30"/>
+      <c r="G56" s="30"/>
+      <c r="H56" s="30"/>
+      <c r="I56" s="30"/>
     </row>
     <row r="57" spans="1:9">
       <c r="A57" s="32" t="s">
@@ -2712,13 +3048,13 @@
       </c>
       <c r="B57" s="32"/>
       <c r="C57" s="32"/>
-      <c r="E57" s="29" t="s">
+      <c r="E57" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="F57" s="29"/>
-      <c r="G57" s="29"/>
-      <c r="H57" s="29"/>
-      <c r="I57" s="29"/>
+      <c r="F57" s="30"/>
+      <c r="G57" s="30"/>
+      <c r="H57" s="30"/>
+      <c r="I57" s="30"/>
     </row>
     <row r="58" spans="1:9">
       <c r="A58" s="32" t="s">
@@ -2726,13 +3062,13 @@
       </c>
       <c r="B58" s="32"/>
       <c r="C58" s="32"/>
-      <c r="E58" s="30" t="s">
+      <c r="E58" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="F58" s="30"/>
-      <c r="G58" s="30"/>
-      <c r="H58" s="30"/>
-      <c r="I58" s="30"/>
+      <c r="F58" s="33"/>
+      <c r="G58" s="33"/>
+      <c r="H58" s="33"/>
+      <c r="I58" s="33"/>
     </row>
     <row r="59" spans="1:9" ht="15" customHeight="1">
       <c r="A59" s="32" t="s">
@@ -2740,23 +3076,23 @@
       </c>
       <c r="B59" s="32"/>
       <c r="C59" s="32"/>
-      <c r="E59" s="31" t="s">
+      <c r="E59" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="F59" s="31"/>
-      <c r="G59" s="31"/>
-      <c r="H59" s="31"/>
-      <c r="I59" s="31"/>
+      <c r="F59" s="34"/>
+      <c r="G59" s="34"/>
+      <c r="H59" s="34"/>
+      <c r="I59" s="34"/>
     </row>
     <row r="60" spans="1:9">
       <c r="A60" s="32"/>
       <c r="B60" s="32"/>
       <c r="C60" s="32"/>
-      <c r="E60" s="31"/>
-      <c r="F60" s="31"/>
-      <c r="G60" s="31"/>
-      <c r="H60" s="31"/>
-      <c r="I60" s="31"/>
+      <c r="E60" s="34"/>
+      <c r="F60" s="34"/>
+      <c r="G60" s="34"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="34"/>
     </row>
     <row r="61" spans="1:9">
       <c r="A61" s="32" t="s">
@@ -2764,11 +3100,11 @@
       </c>
       <c r="B61" s="32"/>
       <c r="C61" s="32"/>
-      <c r="E61" s="29"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="29"/>
-      <c r="H61" s="29"/>
-      <c r="I61" s="29"/>
+      <c r="E61" s="30"/>
+      <c r="F61" s="30"/>
+      <c r="G61" s="30"/>
+      <c r="H61" s="30"/>
+      <c r="I61" s="30"/>
     </row>
     <row r="62" spans="1:9">
       <c r="A62" s="32" t="s">
@@ -2776,36 +3112,36 @@
       </c>
       <c r="B62" s="32"/>
       <c r="C62" s="32"/>
-      <c r="E62" s="29" t="s">
+      <c r="E62" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="F62" s="29"/>
-      <c r="G62" s="29"/>
-      <c r="H62" s="29"/>
-      <c r="I62" s="29"/>
+      <c r="F62" s="30"/>
+      <c r="G62" s="30"/>
+      <c r="H62" s="30"/>
+      <c r="I62" s="30"/>
     </row>
     <row r="63" spans="1:9">
-      <c r="E63" s="30" t="s">
+      <c r="E63" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="F63" s="30"/>
-      <c r="G63" s="30"/>
-      <c r="H63" s="30"/>
-      <c r="I63" s="30"/>
+      <c r="F63" s="33"/>
+      <c r="G63" s="33"/>
+      <c r="H63" s="33"/>
+      <c r="I63" s="33"/>
     </row>
     <row r="64" spans="1:9">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B64" s="33"/>
-      <c r="C64" s="33"/>
-      <c r="E64" s="30" t="s">
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="E64" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="F64" s="30"/>
-      <c r="G64" s="30"/>
-      <c r="H64" s="30"/>
-      <c r="I64" s="30"/>
+      <c r="F64" s="33"/>
+      <c r="G64" s="33"/>
+      <c r="H64" s="33"/>
+      <c r="I64" s="33"/>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" s="32" t="s">
@@ -2813,13 +3149,13 @@
       </c>
       <c r="B65" s="32"/>
       <c r="C65" s="32"/>
-      <c r="E65" s="30" t="s">
+      <c r="E65" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="F65" s="30"/>
-      <c r="G65" s="30"/>
-      <c r="H65" s="30"/>
-      <c r="I65" s="30"/>
+      <c r="F65" s="33"/>
+      <c r="G65" s="33"/>
+      <c r="H65" s="33"/>
+      <c r="I65" s="33"/>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" s="32" t="s">
@@ -2869,31 +3205,42 @@
       <c r="C72" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="83">
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A43:C43"/>
+  <mergeCells count="84">
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="E63:I63"/>
+    <mergeCell ref="E64:I64"/>
+    <mergeCell ref="E65:I65"/>
+    <mergeCell ref="E56:I56"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="E61:I61"/>
+    <mergeCell ref="E59:I60"/>
+    <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="E52:I52"/>
+    <mergeCell ref="E53:I53"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="E35:I35"/>
+    <mergeCell ref="E40:I44"/>
+    <mergeCell ref="E55:I55"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="E38:I38"/>
+    <mergeCell ref="E39:I39"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="E46:I46"/>
+    <mergeCell ref="E47:I47"/>
+    <mergeCell ref="E48:I48"/>
+    <mergeCell ref="E49:I49"/>
     <mergeCell ref="A42:C42"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A66:C66"/>
@@ -2910,12 +3257,30 @@
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="A56:C56"/>
     <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="E35:I35"/>
-    <mergeCell ref="E40:I44"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E22:I22"/>
     <mergeCell ref="E23:I23"/>
@@ -2924,35 +3289,7 @@
     <mergeCell ref="E26:I26"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E28:I28"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="E34:I34"/>
-    <mergeCell ref="E55:I55"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="E38:I38"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="E45:I45"/>
-    <mergeCell ref="E46:I46"/>
-    <mergeCell ref="E47:I47"/>
-    <mergeCell ref="E48:I48"/>
-    <mergeCell ref="E49:I49"/>
-    <mergeCell ref="E50:I50"/>
-    <mergeCell ref="E51:I51"/>
-    <mergeCell ref="E52:I52"/>
-    <mergeCell ref="E53:I53"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="E63:I63"/>
-    <mergeCell ref="E64:I64"/>
-    <mergeCell ref="E65:I65"/>
-    <mergeCell ref="E56:I56"/>
-    <mergeCell ref="E57:I57"/>
-    <mergeCell ref="E58:I58"/>
-    <mergeCell ref="E61:I61"/>
-    <mergeCell ref="E59:I60"/>
+    <mergeCell ref="H6:M6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add media copies support: API, models, DB, services
Implemented full support for managing media copies, including:
- New /copies API route and router registration
- CopyCreateSchema and CopyResponseSchema for validation/serialization
- CopyStatus enum and MediaCopy dataclass
- Repository for tblMediaCopies CRUD operations
- Business logic for adding copies with media validation
- Database schema changes: tblMediaCopies table with FK to tblMediaTitles
- Project file and documentation updates
- Updated DB_DRAFT.xlsx to reflect schema changes
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{244E2E4C-8291-4A02-A4D3-01E50CE28B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12E6B6F-D0E5-4D98-A091-50B2C0B318C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43050" yWindow="540" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="81495" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
@@ -1245,50 +1245,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="2" applyBorder="1"/>
@@ -1299,6 +1255,44 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="1" applyBorder="1"/>
     <xf numFmtId="6" fontId="10" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1310,6 +1304,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1664,19 +1664,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
       <c r="R1" s="2"/>
     </row>
     <row r="2" spans="1:18">
@@ -1763,7 +1763,7 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="33" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="10" t="s">
@@ -1772,21 +1772,21 @@
       <c r="C6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="38"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
     </row>
     <row r="7" spans="1:18">
-      <c r="A7" s="24"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="11" t="s">
         <v>38</v>
       </c>
@@ -1806,12 +1806,12 @@
         <v>6</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
     </row>
     <row r="8" spans="1:18">
-      <c r="A8" s="24"/>
+      <c r="A8" s="34"/>
       <c r="B8" s="11" t="s">
         <v>39</v>
       </c>
@@ -1831,12 +1831,12 @@
         <v>21</v>
       </c>
       <c r="J8" s="4"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
     </row>
     <row r="9" spans="1:18">
-      <c r="A9" s="25"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="12" t="s">
         <v>40</v>
       </c>
@@ -1852,23 +1852,23 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
     </row>
     <row r="11" spans="1:18">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="F11" s="26" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="F11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="28"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="38"/>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="5" t="s">
@@ -1897,7 +1897,7 @@
       </c>
     </row>
     <row r="13" spans="1:18">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="33" t="s">
         <v>24</v>
       </c>
       <c r="B13" s="10" t="s">
@@ -1923,7 +1923,7 @@
       </c>
     </row>
     <row r="14" spans="1:18">
-      <c r="A14" s="24"/>
+      <c r="A14" s="34"/>
       <c r="B14" s="11" t="s">
         <v>46</v>
       </c>
@@ -1943,7 +1943,7 @@
       </c>
     </row>
     <row r="15" spans="1:18">
-      <c r="A15" s="24"/>
+      <c r="A15" s="34"/>
       <c r="B15" s="11" t="s">
         <v>47</v>
       </c>
@@ -1952,22 +1952,22 @@
       </c>
     </row>
     <row r="16" spans="1:18">
-      <c r="A16" s="25"/>
+      <c r="A16" s="35"/>
       <c r="B16" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="28"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="38"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="33" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="10" t="s">
@@ -1990,7 +1990,7 @@
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="24"/>
+      <c r="A18" s="34"/>
       <c r="B18" s="11" t="s">
         <v>46</v>
       </c>
@@ -2011,7 +2011,7 @@
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="24"/>
+      <c r="A19" s="34"/>
       <c r="B19" s="11" t="s">
         <v>50</v>
       </c>
@@ -2026,7 +2026,7 @@
       <c r="I19" s="3"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="25"/>
+      <c r="A20" s="35"/>
       <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
@@ -2035,7 +2035,7 @@
       </c>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="33" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="10" t="s">
@@ -2046,7 +2046,7 @@
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="24"/>
+      <c r="A22" s="34"/>
       <c r="B22" s="11" t="s">
         <v>46</v>
       </c>
@@ -2055,7 +2055,7 @@
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="24"/>
+      <c r="A23" s="34"/>
       <c r="B23" s="11" t="s">
         <v>47</v>
       </c>
@@ -2064,7 +2064,7 @@
       </c>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="25"/>
+      <c r="A24" s="35"/>
       <c r="B24" s="12" t="s">
         <v>48</v>
       </c>
@@ -2073,7 +2073,7 @@
       </c>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="33" t="s">
         <v>7</v>
       </c>
       <c r="B25" s="10" t="s">
@@ -2084,7 +2084,7 @@
       </c>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" s="24"/>
+      <c r="A26" s="34"/>
       <c r="B26" s="11" t="s">
         <v>46</v>
       </c>
@@ -2093,7 +2093,7 @@
       </c>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="24"/>
+      <c r="A27" s="34"/>
       <c r="B27" s="11" t="s">
         <v>68</v>
       </c>
@@ -2102,7 +2102,7 @@
       </c>
     </row>
     <row r="28" spans="1:9">
-      <c r="A28" s="25"/>
+      <c r="A28" s="35"/>
       <c r="B28" s="12" t="s">
         <v>48</v>
       </c>
@@ -2146,13 +2146,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
       <c r="H1" t="s">
         <v>24</v>
       </c>
@@ -2233,21 +2233,21 @@
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="49"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="47"/>
       <c r="E6" s="2"/>
-      <c r="H6" s="35" t="s">
+      <c r="H6" s="49" t="s">
         <v>163</v>
       </c>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="3" t="s">
@@ -2257,28 +2257,28 @@
         <v>0</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>6</v>
-      </c>
       <c r="E7" s="4"/>
-      <c r="H7" s="36" t="s">
+      <c r="H7" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="I7" s="37" t="s">
+      <c r="I7" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="J7" s="37" t="s">
+      <c r="J7" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="K7" s="38" t="s">
+      <c r="K7" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="L7" s="42" t="s">
+      <c r="L7" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="M7" s="43" t="s">
+      <c r="M7" s="27" t="s">
         <v>172</v>
       </c>
     </row>
@@ -2290,28 +2290,28 @@
         <v>17</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="E8" s="4"/>
-      <c r="H8" s="39" t="s">
+      <c r="H8" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="I8" s="40" t="s">
+      <c r="I8" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="J8" s="40">
+      <c r="J8" s="24">
         <v>2015</v>
       </c>
-      <c r="K8" s="41" t="s">
+      <c r="K8" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="L8" s="44">
+      <c r="L8" s="28">
         <v>5</v>
       </c>
-      <c r="M8" s="45">
+      <c r="M8" s="29">
         <v>50</v>
       </c>
     </row>
@@ -2325,22 +2325,22 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
-      <c r="H9" s="39" t="s">
+      <c r="H9" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="I9" s="40" t="s">
+      <c r="I9" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="J9" s="40">
+      <c r="J9" s="24">
         <v>2020</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K9" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="L9" s="44">
+      <c r="L9" s="28">
         <v>10</v>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="29">
         <v>70</v>
       </c>
     </row>
@@ -2352,13 +2352,13 @@
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="28"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="38"/>
       <c r="J11" s="3" t="s">
         <v>4</v>
       </c>
@@ -2394,7 +2394,7 @@
       <c r="J12">
         <v>1</v>
       </c>
-      <c r="K12" s="39" t="s">
+      <c r="K12" s="23" t="s">
         <v>177</v>
       </c>
       <c r="L12" t="s">
@@ -2423,7 +2423,7 @@
       <c r="J13">
         <v>2</v>
       </c>
-      <c r="K13" s="39" t="s">
+      <c r="K13" s="23" t="s">
         <v>177</v>
       </c>
       <c r="L13" t="s">
@@ -2448,7 +2448,7 @@
       <c r="J14">
         <v>3</v>
       </c>
-      <c r="K14" s="39" t="s">
+      <c r="K14" s="23" t="s">
         <v>177</v>
       </c>
       <c r="L14" t="s">
@@ -2467,7 +2467,7 @@
       <c r="J15">
         <v>4</v>
       </c>
-      <c r="K15" s="39" t="s">
+      <c r="K15" s="23" t="s">
         <v>177</v>
       </c>
       <c r="L15" t="s">
@@ -2478,17 +2478,17 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="28"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38"/>
       <c r="E16" s="1"/>
       <c r="J16">
         <v>5</v>
       </c>
-      <c r="K16" s="39" t="s">
+      <c r="K16" s="23" t="s">
         <v>177</v>
       </c>
       <c r="L16" t="s">
@@ -2552,18 +2552,18 @@
       <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:12">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="48" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="E21" s="30" t="s">
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="E21" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="39"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
@@ -2575,13 +2575,13 @@
       <c r="C22" t="s">
         <v>80</v>
       </c>
-      <c r="E22" s="30" t="s">
+      <c r="E22" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="18" t="s">
@@ -2593,13 +2593,13 @@
       <c r="C23" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E23" s="33" t="s">
+      <c r="E23" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="33"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40"/>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="18" t="s">
@@ -2611,13 +2611,13 @@
       <c r="C24" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="33" t="s">
+      <c r="E24" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="18" t="s">
@@ -2629,13 +2629,13 @@
       <c r="C25" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="33" t="s">
+      <c r="E25" s="40" t="s">
         <v>134</v>
       </c>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="33"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="18" t="s">
@@ -2647,13 +2647,13 @@
       <c r="C26" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="33" t="s">
+      <c r="E26" s="40" t="s">
         <v>135</v>
       </c>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
+      <c r="I26" s="40"/>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="18" t="s">
@@ -2665,504 +2665,504 @@
       <c r="C27" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E27" s="33" t="s">
+      <c r="E27" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
     </row>
     <row r="28" spans="1:12">
       <c r="C28" s="18"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="E29" s="30" t="s">
+      <c r="B29" s="43"/>
+      <c r="C29" s="43"/>
+      <c r="E29" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
     </row>
     <row r="30" spans="1:12">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="E30" s="33" t="s">
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="E30" s="40" t="s">
         <v>138</v>
       </c>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="40"/>
     </row>
     <row r="31" spans="1:12">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="E31" s="33" t="s">
+      <c r="B31" s="42"/>
+      <c r="C31" s="42"/>
+      <c r="E31" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="40"/>
+      <c r="I31" s="40"/>
     </row>
     <row r="32" spans="1:12">
-      <c r="A32" s="32" t="s">
+      <c r="A32" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="30"/>
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="39"/>
     </row>
     <row r="33" spans="1:9">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="E33" s="30" t="s">
+      <c r="B33" s="42"/>
+      <c r="C33" s="42"/>
+      <c r="E33" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-      <c r="I33" s="30"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="39"/>
+      <c r="I33" s="39"/>
     </row>
     <row r="34" spans="1:9">
-      <c r="E34" s="33" t="s">
+      <c r="E34" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="33"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="40"/>
+      <c r="H34" s="40"/>
+      <c r="I34" s="40"/>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" s="29" t="s">
+      <c r="A35" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="B35" s="29"/>
-      <c r="C35" s="29"/>
-      <c r="E35" s="33" t="s">
+      <c r="B35" s="43"/>
+      <c r="C35" s="43"/>
+      <c r="E35" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="F35" s="33"/>
-      <c r="G35" s="33"/>
-      <c r="H35" s="33"/>
-      <c r="I35" s="33"/>
+      <c r="F35" s="40"/>
+      <c r="G35" s="40"/>
+      <c r="H35" s="40"/>
+      <c r="I35" s="40"/>
     </row>
     <row r="36" spans="1:9">
-      <c r="A36" s="32" t="s">
+      <c r="A36" s="42" t="s">
         <v>98</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="E36" s="33" t="s">
+      <c r="B36" s="42"/>
+      <c r="C36" s="42"/>
+      <c r="E36" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
+      <c r="F36" s="40"/>
+      <c r="G36" s="40"/>
+      <c r="H36" s="40"/>
+      <c r="I36" s="40"/>
     </row>
     <row r="37" spans="1:9">
-      <c r="A37" s="32" t="s">
+      <c r="A37" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="30"/>
-      <c r="I37" s="30"/>
+      <c r="B37" s="42"/>
+      <c r="C37" s="42"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
     </row>
     <row r="38" spans="1:9">
-      <c r="A38" s="32" t="s">
+      <c r="A38" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="E38" s="30" t="s">
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
+      <c r="E38" s="39" t="s">
         <v>144</v>
       </c>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
     </row>
     <row r="39" spans="1:9">
-      <c r="A39" s="32" t="s">
+      <c r="A39" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="E39" s="33" t="s">
+      <c r="B39" s="42"/>
+      <c r="C39" s="42"/>
+      <c r="E39" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="F39" s="33"/>
-      <c r="G39" s="33"/>
-      <c r="H39" s="33"/>
-      <c r="I39" s="33"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="40"/>
     </row>
     <row r="40" spans="1:9" ht="15" customHeight="1">
       <c r="A40" s="19"/>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
-      <c r="E40" s="34" t="s">
+      <c r="E40" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="F40" s="34"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="34"/>
+      <c r="F40" s="41"/>
+      <c r="G40" s="41"/>
+      <c r="H40" s="41"/>
+      <c r="I40" s="41"/>
     </row>
     <row r="41" spans="1:9">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="34"/>
+      <c r="B41" s="42"/>
+      <c r="C41" s="42"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="41"/>
+      <c r="I41" s="41"/>
     </row>
     <row r="42" spans="1:9">
-      <c r="A42" s="32" t="s">
+      <c r="A42" s="42" t="s">
         <v>103</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="34"/>
+      <c r="B42" s="42"/>
+      <c r="C42" s="42"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="41"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="41"/>
+      <c r="I42" s="41"/>
     </row>
     <row r="43" spans="1:9">
-      <c r="A43" s="32" t="s">
+      <c r="A43" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="32"/>
-      <c r="C43" s="32"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="34"/>
+      <c r="B43" s="42"/>
+      <c r="C43" s="42"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="41"/>
     </row>
     <row r="44" spans="1:9">
-      <c r="A44" s="32" t="s">
+      <c r="A44" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="E44" s="34"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="34"/>
+      <c r="B44" s="42"/>
+      <c r="C44" s="42"/>
+      <c r="E44" s="41"/>
+      <c r="F44" s="41"/>
+      <c r="G44" s="41"/>
+      <c r="H44" s="41"/>
+      <c r="I44" s="41"/>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" s="19"/>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
-      <c r="I45" s="30"/>
+      <c r="E45" s="39"/>
+      <c r="F45" s="39"/>
+      <c r="G45" s="39"/>
+      <c r="H45" s="39"/>
+      <c r="I45" s="39"/>
     </row>
     <row r="46" spans="1:9">
-      <c r="A46" s="32" t="s">
+      <c r="A46" s="42" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-      <c r="E46" s="30" t="s">
+      <c r="B46" s="42"/>
+      <c r="C46" s="42"/>
+      <c r="E46" s="39" t="s">
         <v>147</v>
       </c>
-      <c r="F46" s="30"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="30"/>
-      <c r="I46" s="30"/>
+      <c r="F46" s="39"/>
+      <c r="G46" s="39"/>
+      <c r="H46" s="39"/>
+      <c r="I46" s="39"/>
     </row>
     <row r="47" spans="1:9">
-      <c r="A47" s="32" t="s">
+      <c r="A47" s="42" t="s">
         <v>107</v>
       </c>
-      <c r="B47" s="32"/>
-      <c r="C47" s="32"/>
-      <c r="E47" s="33" t="s">
+      <c r="B47" s="42"/>
+      <c r="C47" s="42"/>
+      <c r="E47" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="F47" s="33"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="33"/>
-      <c r="I47" s="33"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="40"/>
+      <c r="I47" s="40"/>
     </row>
     <row r="48" spans="1:9">
-      <c r="A48" s="32" t="s">
+      <c r="A48" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B48" s="32"/>
-      <c r="C48" s="32"/>
-      <c r="E48" s="33" t="s">
+      <c r="B48" s="42"/>
+      <c r="C48" s="42"/>
+      <c r="E48" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="33"/>
+      <c r="F48" s="40"/>
+      <c r="G48" s="40"/>
+      <c r="H48" s="40"/>
+      <c r="I48" s="40"/>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" s="19"/>
       <c r="B49" s="19"/>
       <c r="C49" s="19"/>
-      <c r="E49" s="33" t="s">
+      <c r="E49" s="40" t="s">
         <v>150</v>
       </c>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
+      <c r="F49" s="40"/>
+      <c r="G49" s="40"/>
+      <c r="H49" s="40"/>
+      <c r="I49" s="40"/>
     </row>
     <row r="50" spans="1:9">
-      <c r="A50" s="32" t="s">
+      <c r="A50" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="B50" s="32"/>
-      <c r="C50" s="32"/>
-      <c r="E50" s="33" t="s">
+      <c r="B50" s="42"/>
+      <c r="C50" s="42"/>
+      <c r="E50" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="33"/>
-      <c r="I50" s="33"/>
+      <c r="F50" s="40"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="40"/>
+      <c r="I50" s="40"/>
     </row>
     <row r="51" spans="1:9">
-      <c r="A51" s="32" t="s">
+      <c r="A51" s="42" t="s">
         <v>121</v>
       </c>
-      <c r="B51" s="32"/>
-      <c r="C51" s="32"/>
-      <c r="E51" s="33" t="s">
+      <c r="B51" s="42"/>
+      <c r="C51" s="42"/>
+      <c r="E51" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="F51" s="33"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="33"/>
-      <c r="I51" s="33"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="40"/>
+      <c r="I51" s="40"/>
     </row>
     <row r="52" spans="1:9">
-      <c r="A52" s="32" t="s">
+      <c r="A52" s="42" t="s">
         <v>122</v>
       </c>
-      <c r="B52" s="32"/>
-      <c r="C52" s="32"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
-      <c r="I52" s="30"/>
+      <c r="B52" s="42"/>
+      <c r="C52" s="42"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="39"/>
+      <c r="I52" s="39"/>
     </row>
     <row r="53" spans="1:9">
-      <c r="A53" s="32" t="s">
+      <c r="A53" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="B53" s="32"/>
-      <c r="C53" s="32"/>
-      <c r="E53" s="30" t="s">
+      <c r="B53" s="42"/>
+      <c r="C53" s="42"/>
+      <c r="E53" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="F53" s="30"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="30"/>
-      <c r="I53" s="30"/>
+      <c r="F53" s="39"/>
+      <c r="G53" s="39"/>
+      <c r="H53" s="39"/>
+      <c r="I53" s="39"/>
     </row>
     <row r="54" spans="1:9">
-      <c r="A54" s="32"/>
-      <c r="B54" s="32"/>
-      <c r="C54" s="32"/>
-      <c r="E54" s="33" t="s">
+      <c r="A54" s="42"/>
+      <c r="B54" s="42"/>
+      <c r="C54" s="42"/>
+      <c r="E54" s="40" t="s">
         <v>154</v>
       </c>
-      <c r="F54" s="33"/>
-      <c r="G54" s="33"/>
-      <c r="H54" s="33"/>
-      <c r="I54" s="33"/>
+      <c r="F54" s="40"/>
+      <c r="G54" s="40"/>
+      <c r="H54" s="40"/>
+      <c r="I54" s="40"/>
     </row>
     <row r="55" spans="1:9">
-      <c r="A55" s="32" t="s">
+      <c r="A55" s="42" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="32"/>
-      <c r="C55" s="32"/>
-      <c r="E55" s="33" t="s">
+      <c r="B55" s="42"/>
+      <c r="C55" s="42"/>
+      <c r="E55" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="F55" s="33"/>
-      <c r="G55" s="33"/>
-      <c r="H55" s="33"/>
-      <c r="I55" s="33"/>
+      <c r="F55" s="40"/>
+      <c r="G55" s="40"/>
+      <c r="H55" s="40"/>
+      <c r="I55" s="40"/>
     </row>
     <row r="56" spans="1:9">
-      <c r="A56" s="32" t="s">
+      <c r="A56" s="42" t="s">
         <v>125</v>
       </c>
-      <c r="B56" s="32"/>
-      <c r="C56" s="32"/>
-      <c r="E56" s="30"/>
-      <c r="F56" s="30"/>
-      <c r="G56" s="30"/>
-      <c r="H56" s="30"/>
-      <c r="I56" s="30"/>
+      <c r="B56" s="42"/>
+      <c r="C56" s="42"/>
+      <c r="E56" s="39"/>
+      <c r="F56" s="39"/>
+      <c r="G56" s="39"/>
+      <c r="H56" s="39"/>
+      <c r="I56" s="39"/>
     </row>
     <row r="57" spans="1:9">
-      <c r="A57" s="32" t="s">
+      <c r="A57" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="B57" s="32"/>
-      <c r="C57" s="32"/>
-      <c r="E57" s="30" t="s">
+      <c r="B57" s="42"/>
+      <c r="C57" s="42"/>
+      <c r="E57" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="F57" s="30"/>
-      <c r="G57" s="30"/>
-      <c r="H57" s="30"/>
-      <c r="I57" s="30"/>
+      <c r="F57" s="39"/>
+      <c r="G57" s="39"/>
+      <c r="H57" s="39"/>
+      <c r="I57" s="39"/>
     </row>
     <row r="58" spans="1:9">
-      <c r="A58" s="32" t="s">
+      <c r="A58" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="B58" s="32"/>
-      <c r="C58" s="32"/>
-      <c r="E58" s="33" t="s">
+      <c r="B58" s="42"/>
+      <c r="C58" s="42"/>
+      <c r="E58" s="40" t="s">
         <v>157</v>
       </c>
-      <c r="F58" s="33"/>
-      <c r="G58" s="33"/>
-      <c r="H58" s="33"/>
-      <c r="I58" s="33"/>
+      <c r="F58" s="40"/>
+      <c r="G58" s="40"/>
+      <c r="H58" s="40"/>
+      <c r="I58" s="40"/>
     </row>
     <row r="59" spans="1:9" ht="15" customHeight="1">
-      <c r="A59" s="32" t="s">
+      <c r="A59" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="B59" s="32"/>
-      <c r="C59" s="32"/>
-      <c r="E59" s="34" t="s">
+      <c r="B59" s="42"/>
+      <c r="C59" s="42"/>
+      <c r="E59" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="F59" s="34"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="34"/>
-      <c r="I59" s="34"/>
+      <c r="F59" s="41"/>
+      <c r="G59" s="41"/>
+      <c r="H59" s="41"/>
+      <c r="I59" s="41"/>
     </row>
     <row r="60" spans="1:9">
-      <c r="A60" s="32"/>
-      <c r="B60" s="32"/>
-      <c r="C60" s="32"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
+      <c r="A60" s="42"/>
+      <c r="B60" s="42"/>
+      <c r="C60" s="42"/>
+      <c r="E60" s="41"/>
+      <c r="F60" s="41"/>
+      <c r="G60" s="41"/>
+      <c r="H60" s="41"/>
+      <c r="I60" s="41"/>
     </row>
     <row r="61" spans="1:9">
-      <c r="A61" s="32" t="s">
+      <c r="A61" s="42" t="s">
         <v>128</v>
       </c>
-      <c r="B61" s="32"/>
-      <c r="C61" s="32"/>
-      <c r="E61" s="30"/>
-      <c r="F61" s="30"/>
-      <c r="G61" s="30"/>
-      <c r="H61" s="30"/>
-      <c r="I61" s="30"/>
+      <c r="B61" s="42"/>
+      <c r="C61" s="42"/>
+      <c r="E61" s="39"/>
+      <c r="F61" s="39"/>
+      <c r="G61" s="39"/>
+      <c r="H61" s="39"/>
+      <c r="I61" s="39"/>
     </row>
     <row r="62" spans="1:9">
-      <c r="A62" s="32" t="s">
+      <c r="A62" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="B62" s="32"/>
-      <c r="C62" s="32"/>
-      <c r="E62" s="30" t="s">
+      <c r="B62" s="42"/>
+      <c r="C62" s="42"/>
+      <c r="E62" s="39" t="s">
         <v>160</v>
       </c>
-      <c r="F62" s="30"/>
-      <c r="G62" s="30"/>
-      <c r="H62" s="30"/>
-      <c r="I62" s="30"/>
+      <c r="F62" s="39"/>
+      <c r="G62" s="39"/>
+      <c r="H62" s="39"/>
+      <c r="I62" s="39"/>
     </row>
     <row r="63" spans="1:9">
-      <c r="E63" s="33" t="s">
+      <c r="E63" s="40" t="s">
         <v>159</v>
       </c>
-      <c r="F63" s="33"/>
-      <c r="G63" s="33"/>
-      <c r="H63" s="33"/>
-      <c r="I63" s="33"/>
+      <c r="F63" s="40"/>
+      <c r="G63" s="40"/>
+      <c r="H63" s="40"/>
+      <c r="I63" s="40"/>
     </row>
     <row r="64" spans="1:9">
-      <c r="A64" s="29" t="s">
+      <c r="A64" s="43" t="s">
         <v>112</v>
       </c>
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-      <c r="E64" s="33" t="s">
+      <c r="B64" s="43"/>
+      <c r="C64" s="43"/>
+      <c r="E64" s="40" t="s">
         <v>161</v>
       </c>
-      <c r="F64" s="33"/>
-      <c r="G64" s="33"/>
-      <c r="H64" s="33"/>
-      <c r="I64" s="33"/>
+      <c r="F64" s="40"/>
+      <c r="G64" s="40"/>
+      <c r="H64" s="40"/>
+      <c r="I64" s="40"/>
     </row>
     <row r="65" spans="1:9">
-      <c r="A65" s="32" t="s">
+      <c r="A65" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="B65" s="32"/>
-      <c r="C65" s="32"/>
-      <c r="E65" s="33" t="s">
+      <c r="B65" s="42"/>
+      <c r="C65" s="42"/>
+      <c r="E65" s="40" t="s">
         <v>162</v>
       </c>
-      <c r="F65" s="33"/>
-      <c r="G65" s="33"/>
-      <c r="H65" s="33"/>
-      <c r="I65" s="33"/>
+      <c r="F65" s="40"/>
+      <c r="G65" s="40"/>
+      <c r="H65" s="40"/>
+      <c r="I65" s="40"/>
     </row>
     <row r="66" spans="1:9">
-      <c r="A66" s="32" t="s">
+      <c r="A66" s="42" t="s">
         <v>114</v>
       </c>
-      <c r="B66" s="32"/>
-      <c r="C66" s="32"/>
+      <c r="B66" s="42"/>
+      <c r="C66" s="42"/>
     </row>
     <row r="67" spans="1:9">
       <c r="A67" s="19"/>
@@ -3170,61 +3170,91 @@
       <c r="C67" s="19"/>
     </row>
     <row r="68" spans="1:9">
-      <c r="A68" s="32" t="s">
+      <c r="A68" s="42" t="s">
         <v>115</v>
       </c>
-      <c r="B68" s="32"/>
-      <c r="C68" s="32"/>
+      <c r="B68" s="42"/>
+      <c r="C68" s="42"/>
     </row>
     <row r="69" spans="1:9">
-      <c r="A69" s="32" t="s">
+      <c r="A69" s="42" t="s">
         <v>116</v>
       </c>
-      <c r="B69" s="32"/>
-      <c r="C69" s="32"/>
+      <c r="B69" s="42"/>
+      <c r="C69" s="42"/>
     </row>
     <row r="70" spans="1:9">
-      <c r="A70" s="32" t="s">
+      <c r="A70" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="B70" s="32"/>
-      <c r="C70" s="32"/>
+      <c r="B70" s="42"/>
+      <c r="C70" s="42"/>
     </row>
     <row r="71" spans="1:9">
-      <c r="A71" s="32" t="s">
+      <c r="A71" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="B71" s="32"/>
-      <c r="C71" s="32"/>
+      <c r="B71" s="42"/>
+      <c r="C71" s="42"/>
     </row>
     <row r="72" spans="1:9">
-      <c r="A72" s="32" t="s">
+      <c r="A72" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="B72" s="32"/>
-      <c r="C72" s="32"/>
+      <c r="B72" s="42"/>
+      <c r="C72" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="E63:I63"/>
-    <mergeCell ref="E64:I64"/>
-    <mergeCell ref="E65:I65"/>
-    <mergeCell ref="E56:I56"/>
-    <mergeCell ref="E57:I57"/>
-    <mergeCell ref="E58:I58"/>
-    <mergeCell ref="E61:I61"/>
-    <mergeCell ref="E59:I60"/>
-    <mergeCell ref="E50:I50"/>
-    <mergeCell ref="E51:I51"/>
-    <mergeCell ref="E52:I52"/>
-    <mergeCell ref="E53:I53"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="E29:I29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="E23:I23"/>
+    <mergeCell ref="E24:I24"/>
+    <mergeCell ref="E25:I25"/>
+    <mergeCell ref="E26:I26"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A59:C59"/>
     <mergeCell ref="A60:C60"/>
@@ -3241,55 +3271,25 @@
     <mergeCell ref="E47:I47"/>
     <mergeCell ref="E48:I48"/>
     <mergeCell ref="E49:I49"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="E21:I21"/>
-    <mergeCell ref="E22:I22"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="E30:I30"/>
+    <mergeCell ref="E31:I31"/>
+    <mergeCell ref="E32:I32"/>
+    <mergeCell ref="E33:I33"/>
+    <mergeCell ref="E34:I34"/>
+    <mergeCell ref="E50:I50"/>
+    <mergeCell ref="E51:I51"/>
+    <mergeCell ref="E52:I52"/>
+    <mergeCell ref="E53:I53"/>
+    <mergeCell ref="E54:I54"/>
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="E63:I63"/>
+    <mergeCell ref="E64:I64"/>
+    <mergeCell ref="E65:I65"/>
+    <mergeCell ref="E56:I56"/>
+    <mergeCell ref="E57:I57"/>
+    <mergeCell ref="E58:I58"/>
+    <mergeCell ref="E61:I61"/>
+    <mergeCell ref="E59:I60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add sales feature: sell copies and record sales
Introduces a new sales system with a tblSales table, Sale model, schemas, and repository. Adds a /sales API endpoint to sell media copies, updating their status and recording the sale. Implements error handling for not found and already sold copies. Updates main app to include sales routes and handlers.
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12E6B6F-D0E5-4D98-A091-50B2C0B318C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77217FD1-EB2F-485B-8689-21E035A8DA26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="81495" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="72720" yWindow="420" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="196">
   <si>
     <t>MediaID</t>
   </si>
@@ -846,6 +846,60 @@
   <si>
     <t>Cyberpunk</t>
   </si>
+  <si>
+    <t>Proces dodawania endpointu od zera</t>
+  </si>
+  <si>
+    <t>Error handlers for business logic errors</t>
+  </si>
+  <si>
+    <t>Schemas for API request validators</t>
+  </si>
+  <si>
+    <t>PATH = /backend/app/*</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>~/api/routes/[NAME].py</t>
+  </si>
+  <si>
+    <t>~/api/error_handlers.py</t>
+  </si>
+  <si>
+    <t>~/api/schemas.py</t>
+  </si>
+  <si>
+    <t>~/core/init_db.py</t>
+  </si>
+  <si>
+    <t>SQL script for intializing the table</t>
+  </si>
+  <si>
+    <t>~/domain/exceptions.py</t>
+  </si>
+  <si>
+    <t>Classes for domain errors (used in handlers)</t>
+  </si>
+  <si>
+    <t>~/repositories/[NAME]_repo.py</t>
+  </si>
+  <si>
+    <t>SQL script for CRUD operations</t>
+  </si>
+  <si>
+    <t>~/services/services.py</t>
+  </si>
+  <si>
+    <t>Business logic wrapper for CRUD operations (function/error invoker)</t>
+  </si>
+  <si>
+    <t>~/main.py</t>
+  </si>
+  <si>
+    <t>API endpoint invoker</t>
+  </si>
 </sst>
 </file>
 
@@ -854,7 +908,7 @@
   <numFmts count="1">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -936,6 +990,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1188,7 +1248,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1311,6 +1371,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -2141,7 +2207,7 @@
     <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2582,6 +2648,10 @@
       <c r="G22" s="39"/>
       <c r="H22" s="39"/>
       <c r="I22" s="39"/>
+      <c r="J22" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="K22" s="50"/>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="18" t="s">
@@ -2600,6 +2670,12 @@
       <c r="G23" s="40"/>
       <c r="H23" s="40"/>
       <c r="I23" s="40"/>
+      <c r="J23" s="52" t="s">
+        <v>181</v>
+      </c>
+      <c r="K23" s="51" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="18" t="s">
@@ -2618,6 +2694,12 @@
       <c r="G24" s="40"/>
       <c r="H24" s="40"/>
       <c r="I24" s="40"/>
+      <c r="J24" s="53" t="s">
+        <v>183</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="18" t="s">
@@ -2636,6 +2718,12 @@
       <c r="G25" s="40"/>
       <c r="H25" s="40"/>
       <c r="I25" s="40"/>
+      <c r="J25" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="18" t="s">
@@ -2654,6 +2742,12 @@
       <c r="G26" s="40"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
+      <c r="J26" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="18" t="s">
@@ -2672,6 +2766,12 @@
       <c r="G27" s="40"/>
       <c r="H27" s="40"/>
       <c r="I27" s="40"/>
+      <c r="J27" s="53" t="s">
+        <v>186</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="28" spans="1:12">
       <c r="C28" s="18"/>
@@ -2680,6 +2780,12 @@
       <c r="G28" s="39"/>
       <c r="H28" s="39"/>
       <c r="I28" s="39"/>
+      <c r="J28" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="43" t="s">
@@ -2694,6 +2800,12 @@
       <c r="G29" s="39"/>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
+      <c r="J29" s="53" t="s">
+        <v>190</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="42" t="s">
@@ -2708,6 +2820,12 @@
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
+      <c r="J30" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="42" t="s">
@@ -2722,6 +2840,12 @@
       <c r="G31" s="40"/>
       <c r="H31" s="40"/>
       <c r="I31" s="40"/>
+      <c r="J31" s="53" t="s">
+        <v>194</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="42" t="s">
@@ -3205,7 +3329,8 @@
       <c r="C72" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="85">
+    <mergeCell ref="J22:K22"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
Refactor sorting enums and expand copies API endpoints
Moved sorting enums to additional_queries.py and removed media_queries.py. Added CopiesSortField and list_filtered to copies_repo.py. Implemented GET /copies and GET /copies/{copy_id} endpoints with filtering, sorting, and pagination. Updated imports and project references accordingly. DB_DRAFT.xlsx was also updated.
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77217FD1-EB2F-485B-8689-21E035A8DA26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAE5F6A-4D04-4948-8731-28375022F735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="72720" yWindow="420" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
@@ -1248,7 +1248,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1371,12 +1371,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -2207,7 +2213,7 @@
     <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="49.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2648,10 +2654,10 @@
       <c r="G22" s="39"/>
       <c r="H22" s="39"/>
       <c r="I22" s="39"/>
-      <c r="J22" s="50" t="s">
+      <c r="J22" s="52" t="s">
         <v>178</v>
       </c>
-      <c r="K22" s="50"/>
+      <c r="K22" s="53"/>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="18" t="s">
@@ -2670,10 +2676,10 @@
       <c r="G23" s="40"/>
       <c r="H23" s="40"/>
       <c r="I23" s="40"/>
-      <c r="J23" s="52" t="s">
+      <c r="J23" s="56" t="s">
         <v>181</v>
       </c>
-      <c r="K23" s="51" t="s">
+      <c r="K23" s="57" t="s">
         <v>182</v>
       </c>
     </row>
@@ -2694,10 +2700,10 @@
       <c r="G24" s="40"/>
       <c r="H24" s="40"/>
       <c r="I24" s="40"/>
-      <c r="J24" s="53" t="s">
+      <c r="J24" s="54" t="s">
         <v>183</v>
       </c>
-      <c r="K24" s="18" t="s">
+      <c r="K24" s="50" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2718,10 +2724,10 @@
       <c r="G25" s="40"/>
       <c r="H25" s="40"/>
       <c r="I25" s="40"/>
-      <c r="J25" s="53" t="s">
+      <c r="J25" s="54" t="s">
         <v>184</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="K25" s="50" t="s">
         <v>179</v>
       </c>
     </row>
@@ -2742,10 +2748,10 @@
       <c r="G26" s="40"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
-      <c r="J26" s="53" t="s">
+      <c r="J26" s="54" t="s">
         <v>185</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="K26" s="50" t="s">
         <v>180</v>
       </c>
     </row>
@@ -2766,10 +2772,10 @@
       <c r="G27" s="40"/>
       <c r="H27" s="40"/>
       <c r="I27" s="40"/>
-      <c r="J27" s="53" t="s">
+      <c r="J27" s="54" t="s">
         <v>186</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="K27" s="50" t="s">
         <v>187</v>
       </c>
     </row>
@@ -2780,10 +2786,10 @@
       <c r="G28" s="39"/>
       <c r="H28" s="39"/>
       <c r="I28" s="39"/>
-      <c r="J28" s="53" t="s">
+      <c r="J28" s="54" t="s">
         <v>188</v>
       </c>
-      <c r="K28" s="18" t="s">
+      <c r="K28" s="50" t="s">
         <v>189</v>
       </c>
     </row>
@@ -2800,10 +2806,10 @@
       <c r="G29" s="39"/>
       <c r="H29" s="39"/>
       <c r="I29" s="39"/>
-      <c r="J29" s="53" t="s">
+      <c r="J29" s="54" t="s">
         <v>190</v>
       </c>
-      <c r="K29" s="18" t="s">
+      <c r="K29" s="50" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2820,10 +2826,10 @@
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
-      <c r="J30" s="53" t="s">
+      <c r="J30" s="54" t="s">
         <v>192</v>
       </c>
-      <c r="K30" s="18" t="s">
+      <c r="K30" s="50" t="s">
         <v>193</v>
       </c>
     </row>
@@ -2840,10 +2846,10 @@
       <c r="G31" s="40"/>
       <c r="H31" s="40"/>
       <c r="I31" s="40"/>
-      <c r="J31" s="53" t="s">
+      <c r="J31" s="55" t="s">
         <v>194</v>
       </c>
-      <c r="K31" s="18" t="s">
+      <c r="K31" s="51" t="s">
         <v>195</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pagination to media, copies, and sales endpoints
API list endpoints now return paginated responses with items, total, limit, and offset. Added paged response schemas and updated repository methods to support pagination. Introduced GET endpoints for single resource retrieval. Improved type safety, fixed minor bugs, and updated DB_DRAFT.xlsx.
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAE5F6A-4D04-4948-8731-28375022F735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F750DD1-F726-4CEF-8F2E-B40999E9A8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72720" yWindow="420" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="46230" yWindow="345" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="196">
   <si>
     <t>MediaID</t>
   </si>
@@ -1248,7 +1248,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1383,6 +1383,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -2429,8 +2435,8 @@
       </c>
       <c r="B11" s="37"/>
       <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="59"/>
       <c r="J11" s="3" t="s">
         <v>4</v>
       </c>
@@ -2452,27 +2458,21 @@
         <v>4</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I12" s="14" t="s">
+      <c r="G12" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="J12">
+      <c r="H12">
         <v>1</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="I12" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="L12" t="s">
+      <c r="J12" t="s">
         <v>175</v>
       </c>
-      <c r="M12">
+      <c r="K12">
         <v>50</v>
       </c>
     </row>
@@ -2484,24 +2484,18 @@
         <v>17</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13">
+      <c r="H13">
         <v>2</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="I13" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="L13" t="s">
+      <c r="J13" t="s">
         <v>175</v>
       </c>
-      <c r="M13">
+      <c r="K13">
         <v>50</v>
       </c>
     </row>
@@ -2513,20 +2507,16 @@
         <v>23</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J14">
+      <c r="H14">
         <v>3</v>
       </c>
-      <c r="K14" s="23" t="s">
+      <c r="I14" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="L14" t="s">
+      <c r="J14" t="s">
         <v>176</v>
       </c>
-      <c r="M14">
+      <c r="K14">
         <v>50</v>
       </c>
     </row>
@@ -2550,80 +2540,44 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A16" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="1"/>
-      <c r="J16">
+      <c r="A16" s="1"/>
+      <c r="F16">
         <v>5</v>
       </c>
-      <c r="K16" s="23" t="s">
+      <c r="G16" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="L16" t="s">
+      <c r="H16" t="s">
         <v>175</v>
       </c>
-      <c r="M16">
+      <c r="I16">
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="J17" t="s">
+    <row r="17" spans="1:11">
+      <c r="A17" s="1"/>
+      <c r="F17" t="s">
         <v>173</v>
       </c>
-      <c r="L17">
+      <c r="H17">
         <f>COUNTIF(L12:L16, "AVAILABLE")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
-      <c r="A18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="1"/>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="1"/>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:11">
       <c r="A21" s="48" t="s">
         <v>92</v>
       </c>
@@ -2637,7 +2591,7 @@
       <c r="H21" s="39"/>
       <c r="I21" s="39"/>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:11">
       <c r="A22" t="s">
         <v>78</v>
       </c>
@@ -2659,7 +2613,7 @@
       </c>
       <c r="K22" s="53"/>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:11">
       <c r="A23" s="18" t="s">
         <v>81</v>
       </c>
@@ -2683,7 +2637,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:11">
       <c r="A24" s="18" t="s">
         <v>84</v>
       </c>
@@ -2707,7 +2661,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:11">
       <c r="A25" s="18" t="s">
         <v>86</v>
       </c>
@@ -2731,7 +2685,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:11">
       <c r="A26" s="18" t="s">
         <v>89</v>
       </c>
@@ -2755,7 +2709,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:11">
       <c r="A27" s="18" t="s">
         <v>109</v>
       </c>
@@ -2779,7 +2733,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:11">
       <c r="C28" s="18"/>
       <c r="E28" s="39"/>
       <c r="F28" s="39"/>
@@ -2793,7 +2747,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:11">
       <c r="A29" s="43" t="s">
         <v>93</v>
       </c>
@@ -2813,7 +2767,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:11">
       <c r="A30" s="42" t="s">
         <v>91</v>
       </c>
@@ -2833,7 +2787,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:11">
       <c r="A31" s="42" t="s">
         <v>94</v>
       </c>
@@ -2853,7 +2807,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:11">
       <c r="A32" s="42" t="s">
         <v>95</v>
       </c>
@@ -3335,14 +3289,13 @@
       <c r="C72" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="85">
+  <mergeCells count="84">
     <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="E29:I29"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="E21:I21"/>
     <mergeCell ref="E22:I22"/>

</xml_diff>

<commit_message>
Refactor: remove media copies logic and update schema
Removed all code, models, and endpoints related to media copies. Updated the database schema: dropped tblMediaCopies, renamed tblMediaTitles to tblMedia with an Amount field, and changed tblSales to reference MediaID instead of CopyID. Cleaned up error handlers, schemas, enums, and project files accordingly. Sales logic now operates directly on MediaID. Updated database and Excel files to match new structure.
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F750DD1-F726-4CEF-8F2E-B40999E9A8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C75A697-3B0F-49DB-8457-D0197852357A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46230" yWindow="345" windowWidth="18480" windowHeight="15240" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="API ENDPOINTS" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="192">
   <si>
     <t>MediaID</t>
   </si>
@@ -391,30 +391,6 @@
     <t>--</t>
   </si>
   <si>
-    <t>addMedia</t>
-  </si>
-  <si>
-    <t>if title.exists(): throw err;   else: return title</t>
-  </si>
-  <si>
-    <t>operation.name</t>
-  </si>
-  <si>
-    <t>operation.function</t>
-  </si>
-  <si>
-    <t>operation.parameters</t>
-  </si>
-  <si>
-    <t>media_title, media_type, media_genre, media_date</t>
-  </si>
-  <si>
-    <t>parameters.contraints</t>
-  </si>
-  <si>
-    <t>title/type/genre not text; date not date</t>
-  </si>
-  <si>
     <t>Typ błędu</t>
   </si>
   <si>
@@ -802,51 +778,21 @@
     <t>{ "error": "MEDIA_ALREADY_EXISTS", "message": "Media with given title and type already exists"}</t>
   </si>
   <si>
-    <t>ITEMS</t>
-  </si>
-  <si>
     <t>Title</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Release</t>
-  </si>
-  <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
     <t>Wiedzmin</t>
   </si>
   <si>
-    <t>GAME</t>
-  </si>
-  <si>
     <t>CDPR</t>
   </si>
   <si>
     <t>Price</t>
   </si>
   <si>
-    <t>COUNT(*)</t>
-  </si>
-  <si>
-    <t>GET /copies</t>
-  </si>
-  <si>
-    <t>AVAILABLE</t>
-  </si>
-  <si>
-    <t>SOLD</t>
-  </si>
-  <si>
-    <t>Cyberpunk</t>
-  </si>
-  <si>
     <t>Proces dodawania endpointu od zera</t>
   </si>
   <si>
@@ -899,16 +845,55 @@
   </si>
   <si>
     <t>API endpoint invoker</t>
+  </si>
+  <si>
+    <t>Editable</t>
+  </si>
+  <si>
+    <t>Non-Editable</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Editable (+=)</t>
+  </si>
+  <si>
+    <t>Header</t>
+  </si>
+  <si>
+    <t>DataType</t>
+  </si>
+  <si>
+    <t>Info</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>BOOK</t>
+  </si>
+  <si>
+    <t>Table_name</t>
+  </si>
+  <si>
+    <t>DATETIME()</t>
+  </si>
+  <si>
+    <t>tblMedia</t>
+  </si>
+  <si>
+    <t>taken from tblMedia</t>
+  </si>
+  <si>
+    <t>ReleaseYear</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-  </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -978,13 +963,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -996,8 +974,21 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1006,16 +997,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1153,102 +1150,21 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1298,23 +1214,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="17" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="14" xfId="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="10" fillId="2" borderId="15" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1342,57 +1251,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="22" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Bad" xfId="2" builtinId="27"/>
-    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1742,19 +1651,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="32" t="s">
+      <c r="F1" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
       <c r="R1" s="2"/>
     </row>
     <row r="2" spans="1:18">
@@ -1841,7 +1750,7 @@
       </c>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="28" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="10" t="s">
@@ -1850,21 +1759,21 @@
       <c r="C6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="36" t="s">
+      <c r="F6" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="38"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="33"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="L6" s="30"/>
-      <c r="M6" s="30"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
     </row>
     <row r="7" spans="1:18">
-      <c r="A7" s="34"/>
+      <c r="A7" s="29"/>
       <c r="B7" s="11" t="s">
         <v>38</v>
       </c>
@@ -1884,12 +1793,12 @@
         <v>6</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
+      <c r="M7" s="25"/>
     </row>
     <row r="8" spans="1:18">
-      <c r="A8" s="34"/>
+      <c r="A8" s="29"/>
       <c r="B8" s="11" t="s">
         <v>39</v>
       </c>
@@ -1909,12 +1818,12 @@
         <v>21</v>
       </c>
       <c r="J8" s="4"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="25"/>
     </row>
     <row r="9" spans="1:18">
-      <c r="A9" s="35"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="12" t="s">
         <v>40</v>
       </c>
@@ -1930,23 +1839,23 @@
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25"/>
+      <c r="M9" s="25"/>
     </row>
     <row r="11" spans="1:18">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="F11" s="36" t="s">
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="F11" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="38"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="33"/>
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="5" t="s">
@@ -1975,7 +1884,7 @@
       </c>
     </row>
     <row r="13" spans="1:18">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="28" t="s">
         <v>24</v>
       </c>
       <c r="B13" s="10" t="s">
@@ -2001,7 +1910,7 @@
       </c>
     </row>
     <row r="14" spans="1:18">
-      <c r="A14" s="34"/>
+      <c r="A14" s="29"/>
       <c r="B14" s="11" t="s">
         <v>46</v>
       </c>
@@ -2021,7 +1930,7 @@
       </c>
     </row>
     <row r="15" spans="1:18">
-      <c r="A15" s="34"/>
+      <c r="A15" s="29"/>
       <c r="B15" s="11" t="s">
         <v>47</v>
       </c>
@@ -2030,22 +1939,22 @@
       </c>
     </row>
     <row r="16" spans="1:18">
-      <c r="A16" s="35"/>
+      <c r="A16" s="30"/>
       <c r="B16" s="12" t="s">
         <v>48</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="36" t="s">
+      <c r="F16" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="38"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="33"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="10" t="s">
@@ -2068,7 +1977,7 @@
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="34"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="11" t="s">
         <v>46</v>
       </c>
@@ -2089,7 +1998,7 @@
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="34"/>
+      <c r="A19" s="29"/>
       <c r="B19" s="11" t="s">
         <v>50</v>
       </c>
@@ -2104,7 +2013,7 @@
       <c r="I19" s="3"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="35"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="12" t="s">
         <v>48</v>
       </c>
@@ -2113,7 +2022,7 @@
       </c>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="33" t="s">
+      <c r="A21" s="28" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="10" t="s">
@@ -2124,7 +2033,7 @@
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="34"/>
+      <c r="A22" s="29"/>
       <c r="B22" s="11" t="s">
         <v>46</v>
       </c>
@@ -2133,7 +2042,7 @@
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="34"/>
+      <c r="A23" s="29"/>
       <c r="B23" s="11" t="s">
         <v>47</v>
       </c>
@@ -2142,7 +2051,7 @@
       </c>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="35"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="12" t="s">
         <v>48</v>
       </c>
@@ -2151,7 +2060,7 @@
       </c>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="28" t="s">
         <v>7</v>
       </c>
       <c r="B25" s="10" t="s">
@@ -2162,7 +2071,7 @@
       </c>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" s="34"/>
+      <c r="A26" s="29"/>
       <c r="B26" s="11" t="s">
         <v>46</v>
       </c>
@@ -2171,7 +2080,7 @@
       </c>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="34"/>
+      <c r="A27" s="29"/>
       <c r="B27" s="11" t="s">
         <v>68</v>
       </c>
@@ -2180,7 +2089,7 @@
       </c>
     </row>
     <row r="28" spans="1:9">
-      <c r="A28" s="35"/>
+      <c r="A28" s="30"/>
       <c r="B28" s="12" t="s">
         <v>48</v>
       </c>
@@ -2209,1171 +2118,1049 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{183FBF69-F40B-4D82-939D-3AFD7BBD6803}">
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="49.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="49.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="H1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="3" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C2" t="s">
-        <v>165</v>
-      </c>
-      <c r="D2" t="s">
-        <v>166</v>
-      </c>
-      <c r="E2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F2" s="4"/>
-      <c r="H2" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="K2" s="17" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="3" t="s">
+      <c r="C2" s="50" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>191</v>
+      </c>
+      <c r="F2" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="G2" s="50" t="s">
+        <v>180</v>
+      </c>
+      <c r="H2" s="50" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="G3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="48"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" s="51">
+        <v>1</v>
+      </c>
+      <c r="C5" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="E5" s="51">
+        <v>2003</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="50">
+        <v>67</v>
+      </c>
+      <c r="H5" s="50">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="43"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="45"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="45"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="47" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>188</v>
+      </c>
+      <c r="F10" s="45"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="51">
+        <v>1</v>
+      </c>
+      <c r="C11" s="51">
+        <v>1</v>
+      </c>
+      <c r="D11" s="50">
+        <v>420</v>
+      </c>
+      <c r="E11" s="52">
+        <v>46053.903506944444</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="B12" s="1"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="B13" s="1"/>
+      <c r="C13" s="44"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" s="1"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" s="1"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="2:12">
+      <c r="B17" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="F17" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+    </row>
+    <row r="18" spans="2:12">
+      <c r="B18" t="s">
         <v>70</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="C18" t="s">
         <v>71</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="D18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="L18" s="35"/>
+    </row>
+    <row r="19" spans="2:12">
+      <c r="B19" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="F19" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="40"/>
+      <c r="K19" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="L19" s="24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12">
+      <c r="B20" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="17" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A6" s="45" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="2"/>
-      <c r="H6" s="49" t="s">
-        <v>163</v>
-      </c>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="49"/>
-      <c r="M6" s="49"/>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="4"/>
-      <c r="H7" s="20" t="s">
-        <v>164</v>
-      </c>
-      <c r="I7" s="21" t="s">
+      <c r="F20" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="40"/>
+      <c r="K20" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="L20" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12">
+      <c r="B21" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="L21" s="19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12">
+      <c r="B22" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="F22" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="40"/>
+      <c r="K22" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="L7" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="M7" s="27" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="H8" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="I8" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="J8" s="24">
-        <v>2015</v>
-      </c>
-      <c r="K8" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="L8" s="28">
-        <v>5</v>
-      </c>
-      <c r="M8" s="29">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="H9" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="I9" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="J9" s="24">
-        <v>2020</v>
-      </c>
-      <c r="K9" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="L9" s="28">
-        <v>10</v>
-      </c>
-      <c r="M9" s="29">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="58"/>
-      <c r="E11" s="59"/>
-      <c r="J11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="J12" t="s">
-        <v>175</v>
-      </c>
-      <c r="K12">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13">
-        <v>2</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="J13" t="s">
-        <v>175</v>
-      </c>
-      <c r="K13">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A14" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="H14">
-        <v>3</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="J14" t="s">
-        <v>176</v>
-      </c>
-      <c r="K14">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="J15">
-        <v>4</v>
-      </c>
-      <c r="K15" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="L15" t="s">
-        <v>175</v>
-      </c>
-      <c r="M15">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A16" s="1"/>
-      <c r="F16">
-        <v>5</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="H16" t="s">
-        <v>175</v>
-      </c>
-      <c r="I16">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17" s="1"/>
-      <c r="F17" t="s">
-        <v>173</v>
-      </c>
-      <c r="H17">
-        <f>COUNTIF(L12:L16, "AVAILABLE")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:11">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="A21" s="48" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="E21" s="39" t="s">
-        <v>130</v>
-      </c>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="39"/>
-      <c r="I21" s="39"/>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" s="39" t="s">
-        <v>131</v>
-      </c>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="52" t="s">
-        <v>178</v>
-      </c>
-      <c r="K22" s="53"/>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="40" t="s">
-        <v>132</v>
-      </c>
-      <c r="F23" s="40"/>
+      <c r="L22" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12">
+      <c r="B23" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>128</v>
+      </c>
       <c r="G23" s="40"/>
       <c r="H23" s="40"/>
       <c r="I23" s="40"/>
-      <c r="J23" s="56" t="s">
-        <v>181</v>
-      </c>
-      <c r="K23" s="57" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C24" s="18" t="s">
+      <c r="J23" s="40"/>
+      <c r="K23" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="L23" s="19" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12">
+      <c r="D24" s="17"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="L24" s="19" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12">
+      <c r="B25" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="40" t="s">
-        <v>133</v>
-      </c>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="54" t="s">
-        <v>183</v>
-      </c>
-      <c r="K24" s="50" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="E25" s="40" t="s">
-        <v>134</v>
-      </c>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
-      <c r="J25" s="54" t="s">
-        <v>184</v>
-      </c>
-      <c r="K25" s="50" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="E26" s="40" t="s">
-        <v>135</v>
-      </c>
-      <c r="F26" s="40"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="F25" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="L25" s="19" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12">
+      <c r="B26" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="F26" s="40" t="s">
+        <v>130</v>
+      </c>
       <c r="G26" s="40"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
-      <c r="J26" s="54" t="s">
-        <v>185</v>
-      </c>
-      <c r="K26" s="50" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="18" t="s">
-        <v>109</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="E27" s="40" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27" s="40"/>
+      <c r="J26" s="40"/>
+      <c r="K26" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="L26" s="19" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12">
+      <c r="B27" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="F27" s="40" t="s">
+        <v>131</v>
+      </c>
       <c r="G27" s="40"/>
       <c r="H27" s="40"/>
       <c r="I27" s="40"/>
-      <c r="J27" s="54" t="s">
-        <v>186</v>
-      </c>
-      <c r="K27" s="50" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="C28" s="18"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="54" t="s">
-        <v>188</v>
-      </c>
-      <c r="K28" s="50" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="43" t="s">
-        <v>93</v>
-      </c>
-      <c r="B29" s="43"/>
-      <c r="C29" s="43"/>
-      <c r="E29" s="39" t="s">
-        <v>137</v>
-      </c>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39"/>
-      <c r="J29" s="54" t="s">
-        <v>190</v>
-      </c>
-      <c r="K29" s="50" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="42" t="s">
-        <v>91</v>
-      </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="42"/>
-      <c r="E30" s="40" t="s">
-        <v>138</v>
-      </c>
-      <c r="F30" s="40"/>
+      <c r="J27" s="40"/>
+      <c r="K27" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="L27" s="20" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12">
+      <c r="B28" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
+    </row>
+    <row r="29" spans="2:12">
+      <c r="B29" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="F29" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="G29" s="37"/>
+      <c r="H29" s="37"/>
+      <c r="I29" s="37"/>
+      <c r="J29" s="37"/>
+    </row>
+    <row r="30" spans="2:12">
+      <c r="F30" s="40" t="s">
+        <v>134</v>
+      </c>
       <c r="G30" s="40"/>
       <c r="H30" s="40"/>
       <c r="I30" s="40"/>
-      <c r="J30" s="54" t="s">
-        <v>192</v>
-      </c>
-      <c r="K30" s="50" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="42" t="s">
-        <v>94</v>
-      </c>
-      <c r="B31" s="42"/>
-      <c r="C31" s="42"/>
-      <c r="E31" s="40" t="s">
-        <v>139</v>
-      </c>
-      <c r="F31" s="40"/>
+      <c r="J30" s="40"/>
+    </row>
+    <row r="31" spans="2:12">
+      <c r="B31" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="F31" s="40" t="s">
+        <v>133</v>
+      </c>
       <c r="G31" s="40"/>
       <c r="H31" s="40"/>
       <c r="I31" s="40"/>
-      <c r="J31" s="55" t="s">
-        <v>194</v>
-      </c>
-      <c r="K31" s="51" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="39"/>
-      <c r="H32" s="39"/>
-      <c r="I32" s="39"/>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" s="42" t="s">
-        <v>96</v>
-      </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="42"/>
-      <c r="E33" s="39" t="s">
-        <v>140</v>
-      </c>
-      <c r="F33" s="39"/>
-      <c r="G33" s="39"/>
-      <c r="H33" s="39"/>
-      <c r="I33" s="39"/>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="E34" s="40" t="s">
-        <v>142</v>
-      </c>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40"/>
-    </row>
-    <row r="35" spans="1:9">
-      <c r="A35" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="B35" s="43"/>
-      <c r="C35" s="43"/>
-      <c r="E35" s="40" t="s">
-        <v>141</v>
-      </c>
-      <c r="F35" s="40"/>
+      <c r="J31" s="40"/>
+    </row>
+    <row r="32" spans="2:12">
+      <c r="B32" s="41" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="F32" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="G32" s="40"/>
+      <c r="H32" s="40"/>
+      <c r="I32" s="40"/>
+      <c r="J32" s="40"/>
+    </row>
+    <row r="33" spans="2:10">
+      <c r="B33" s="41" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="37"/>
+    </row>
+    <row r="34" spans="2:10">
+      <c r="B34" s="41" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="F34" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="37"/>
+    </row>
+    <row r="35" spans="2:10">
+      <c r="B35" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="F35" s="40" t="s">
+        <v>137</v>
+      </c>
       <c r="G35" s="40"/>
       <c r="H35" s="40"/>
       <c r="I35" s="40"/>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="42" t="s">
+      <c r="J35" s="40"/>
+    </row>
+    <row r="36" spans="2:10" ht="15" customHeight="1">
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="F36" s="42" t="s">
+        <v>138</v>
+      </c>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
+      <c r="I36" s="42"/>
+      <c r="J36" s="42"/>
+    </row>
+    <row r="37" spans="2:10">
+      <c r="B37" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+      <c r="H37" s="42"/>
+      <c r="I37" s="42"/>
+      <c r="J37" s="42"/>
+    </row>
+    <row r="38" spans="2:10">
+      <c r="B38" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="42"/>
+    </row>
+    <row r="39" spans="2:10">
+      <c r="B39" s="41" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+      <c r="H39" s="42"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="42"/>
+    </row>
+    <row r="40" spans="2:10">
+      <c r="B40" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="C40" s="41"/>
+      <c r="D40" s="41"/>
+      <c r="F40" s="42"/>
+      <c r="G40" s="42"/>
+      <c r="H40" s="42"/>
+      <c r="I40" s="42"/>
+      <c r="J40" s="42"/>
+    </row>
+    <row r="41" spans="2:10">
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="F41" s="37"/>
+      <c r="G41" s="37"/>
+      <c r="H41" s="37"/>
+      <c r="I41" s="37"/>
+      <c r="J41" s="37"/>
+    </row>
+    <row r="42" spans="2:10">
+      <c r="B42" s="41" t="s">
         <v>98</v>
       </c>
-      <c r="B36" s="42"/>
-      <c r="C36" s="42"/>
-      <c r="E36" s="40" t="s">
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+      <c r="F42" s="37" t="s">
+        <v>139</v>
+      </c>
+      <c r="G42" s="37"/>
+      <c r="H42" s="37"/>
+      <c r="I42" s="37"/>
+      <c r="J42" s="37"/>
+    </row>
+    <row r="43" spans="2:10">
+      <c r="B43" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" s="41"/>
+      <c r="D43" s="41"/>
+      <c r="F43" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="G43" s="40"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="40"/>
+      <c r="J43" s="40"/>
+    </row>
+    <row r="44" spans="2:10">
+      <c r="B44" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="C44" s="41"/>
+      <c r="D44" s="41"/>
+      <c r="F44" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="G44" s="40"/>
+      <c r="H44" s="40"/>
+      <c r="I44" s="40"/>
+      <c r="J44" s="40"/>
+    </row>
+    <row r="45" spans="2:10">
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="F45" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="40"/>
+      <c r="J45" s="40"/>
+    </row>
+    <row r="46" spans="2:10">
+      <c r="B46" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="C46" s="41"/>
+      <c r="D46" s="41"/>
+      <c r="F46" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="F36" s="40"/>
-      <c r="G36" s="40"/>
-      <c r="H36" s="40"/>
-      <c r="I36" s="40"/>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="42" t="s">
-        <v>99</v>
-      </c>
-      <c r="B37" s="42"/>
-      <c r="C37" s="42"/>
-      <c r="E37" s="39"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="39"/>
-      <c r="H37" s="39"/>
-      <c r="I37" s="39"/>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="42" t="s">
-        <v>100</v>
-      </c>
-      <c r="B38" s="42"/>
-      <c r="C38" s="42"/>
-      <c r="E38" s="39" t="s">
+      <c r="G46" s="40"/>
+      <c r="H46" s="40"/>
+      <c r="I46" s="40"/>
+      <c r="J46" s="40"/>
+    </row>
+    <row r="47" spans="2:10">
+      <c r="B47" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="41"/>
+      <c r="D47" s="41"/>
+      <c r="F47" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
-      <c r="H38" s="39"/>
-      <c r="I38" s="39"/>
-    </row>
-    <row r="39" spans="1:9">
-      <c r="A39" s="42" t="s">
-        <v>101</v>
-      </c>
-      <c r="B39" s="42"/>
-      <c r="C39" s="42"/>
-      <c r="E39" s="40" t="s">
-        <v>145</v>
-      </c>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="40"/>
-      <c r="I39" s="40"/>
-    </row>
-    <row r="40" spans="1:9" ht="15" customHeight="1">
-      <c r="A40" s="19"/>
-      <c r="B40" s="19"/>
-      <c r="C40" s="19"/>
-      <c r="E40" s="41" t="s">
-        <v>146</v>
-      </c>
-      <c r="F40" s="41"/>
-      <c r="G40" s="41"/>
-      <c r="H40" s="41"/>
-      <c r="I40" s="41"/>
-    </row>
-    <row r="41" spans="1:9">
-      <c r="A41" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="42"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="41"/>
-    </row>
-    <row r="42" spans="1:9">
-      <c r="A42" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B42" s="42"/>
-      <c r="C42" s="42"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
-      <c r="G42" s="41"/>
-      <c r="H42" s="41"/>
-      <c r="I42" s="41"/>
-    </row>
-    <row r="43" spans="1:9">
-      <c r="A43" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B43" s="42"/>
-      <c r="C43" s="42"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="41"/>
-      <c r="H43" s="41"/>
-      <c r="I43" s="41"/>
-    </row>
-    <row r="44" spans="1:9">
-      <c r="A44" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="42"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="41"/>
-      <c r="I44" s="41"/>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" s="19"/>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
-      <c r="I45" s="39"/>
-    </row>
-    <row r="46" spans="1:9">
-      <c r="A46" s="42" t="s">
-        <v>106</v>
-      </c>
-      <c r="B46" s="42"/>
-      <c r="C46" s="42"/>
-      <c r="E46" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39"/>
-    </row>
-    <row r="47" spans="1:9">
-      <c r="A47" s="42" t="s">
-        <v>107</v>
-      </c>
-      <c r="B47" s="42"/>
-      <c r="C47" s="42"/>
-      <c r="E47" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="F47" s="40"/>
       <c r="G47" s="40"/>
       <c r="H47" s="40"/>
       <c r="I47" s="40"/>
-    </row>
-    <row r="48" spans="1:9">
-      <c r="A48" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="B48" s="42"/>
-      <c r="C48" s="42"/>
-      <c r="E48" s="40" t="s">
-        <v>149</v>
-      </c>
-      <c r="F48" s="40"/>
-      <c r="G48" s="40"/>
-      <c r="H48" s="40"/>
-      <c r="I48" s="40"/>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" s="19"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="E49" s="40" t="s">
-        <v>150</v>
-      </c>
-      <c r="F49" s="40"/>
-      <c r="G49" s="40"/>
-      <c r="H49" s="40"/>
-      <c r="I49" s="40"/>
-    </row>
-    <row r="50" spans="1:9">
-      <c r="A50" s="42" t="s">
-        <v>120</v>
-      </c>
-      <c r="B50" s="42"/>
-      <c r="C50" s="42"/>
-      <c r="E50" s="40" t="s">
-        <v>151</v>
-      </c>
-      <c r="F50" s="40"/>
+      <c r="J47" s="40"/>
+    </row>
+    <row r="48" spans="2:10">
+      <c r="B48" s="41" t="s">
+        <v>114</v>
+      </c>
+      <c r="C48" s="41"/>
+      <c r="D48" s="41"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="37"/>
+      <c r="H48" s="37"/>
+      <c r="I48" s="37"/>
+      <c r="J48" s="37"/>
+    </row>
+    <row r="49" spans="2:10">
+      <c r="B49" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="C49" s="41"/>
+      <c r="D49" s="41"/>
+      <c r="F49" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="G49" s="37"/>
+      <c r="H49" s="37"/>
+      <c r="I49" s="37"/>
+      <c r="J49" s="37"/>
+    </row>
+    <row r="50" spans="2:10">
+      <c r="B50" s="41"/>
+      <c r="C50" s="41"/>
+      <c r="D50" s="41"/>
+      <c r="F50" s="40" t="s">
+        <v>146</v>
+      </c>
       <c r="G50" s="40"/>
       <c r="H50" s="40"/>
       <c r="I50" s="40"/>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" s="42" t="s">
-        <v>121</v>
-      </c>
-      <c r="B51" s="42"/>
-      <c r="C51" s="42"/>
-      <c r="E51" s="40" t="s">
-        <v>152</v>
-      </c>
-      <c r="F51" s="40"/>
+      <c r="J50" s="40"/>
+    </row>
+    <row r="51" spans="2:10">
+      <c r="B51" s="41" t="s">
+        <v>116</v>
+      </c>
+      <c r="C51" s="41"/>
+      <c r="D51" s="41"/>
+      <c r="F51" s="40" t="s">
+        <v>147</v>
+      </c>
       <c r="G51" s="40"/>
       <c r="H51" s="40"/>
       <c r="I51" s="40"/>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="B52" s="42"/>
-      <c r="C52" s="42"/>
-      <c r="E52" s="39"/>
-      <c r="F52" s="39"/>
-      <c r="G52" s="39"/>
-      <c r="H52" s="39"/>
-      <c r="I52" s="39"/>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" s="42" t="s">
-        <v>123</v>
-      </c>
-      <c r="B53" s="42"/>
-      <c r="C53" s="42"/>
-      <c r="E53" s="39" t="s">
-        <v>153</v>
-      </c>
-      <c r="F53" s="39"/>
-      <c r="G53" s="39"/>
-      <c r="H53" s="39"/>
-      <c r="I53" s="39"/>
-    </row>
-    <row r="54" spans="1:9">
-      <c r="A54" s="42"/>
-      <c r="B54" s="42"/>
-      <c r="C54" s="42"/>
-      <c r="E54" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="F54" s="40"/>
+      <c r="J51" s="40"/>
+    </row>
+    <row r="52" spans="2:10">
+      <c r="B52" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="C52" s="41"/>
+      <c r="D52" s="41"/>
+      <c r="F52" s="37"/>
+      <c r="G52" s="37"/>
+      <c r="H52" s="37"/>
+      <c r="I52" s="37"/>
+      <c r="J52" s="37"/>
+    </row>
+    <row r="53" spans="2:10">
+      <c r="B53" s="41" t="s">
+        <v>118</v>
+      </c>
+      <c r="C53" s="41"/>
+      <c r="D53" s="41"/>
+      <c r="F53" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="G53" s="37"/>
+      <c r="H53" s="37"/>
+      <c r="I53" s="37"/>
+      <c r="J53" s="37"/>
+    </row>
+    <row r="54" spans="2:10">
+      <c r="B54" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="F54" s="40" t="s">
+        <v>149</v>
+      </c>
       <c r="G54" s="40"/>
       <c r="H54" s="40"/>
       <c r="I54" s="40"/>
-    </row>
-    <row r="55" spans="1:9">
-      <c r="A55" s="42" t="s">
-        <v>124</v>
-      </c>
-      <c r="B55" s="42"/>
-      <c r="C55" s="42"/>
-      <c r="E55" s="40" t="s">
-        <v>155</v>
-      </c>
-      <c r="F55" s="40"/>
-      <c r="G55" s="40"/>
-      <c r="H55" s="40"/>
-      <c r="I55" s="40"/>
-    </row>
-    <row r="56" spans="1:9">
-      <c r="A56" s="42" t="s">
-        <v>125</v>
-      </c>
-      <c r="B56" s="42"/>
-      <c r="C56" s="42"/>
-      <c r="E56" s="39"/>
-      <c r="F56" s="39"/>
-      <c r="G56" s="39"/>
-      <c r="H56" s="39"/>
-      <c r="I56" s="39"/>
-    </row>
-    <row r="57" spans="1:9">
-      <c r="A57" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="B57" s="42"/>
-      <c r="C57" s="42"/>
-      <c r="E57" s="39" t="s">
-        <v>156</v>
-      </c>
-      <c r="F57" s="39"/>
-      <c r="G57" s="39"/>
-      <c r="H57" s="39"/>
-      <c r="I57" s="39"/>
-    </row>
-    <row r="58" spans="1:9">
-      <c r="A58" s="42" t="s">
-        <v>88</v>
-      </c>
-      <c r="B58" s="42"/>
-      <c r="C58" s="42"/>
-      <c r="E58" s="40" t="s">
-        <v>157</v>
-      </c>
-      <c r="F58" s="40"/>
-      <c r="G58" s="40"/>
-      <c r="H58" s="40"/>
-      <c r="I58" s="40"/>
-    </row>
-    <row r="59" spans="1:9" ht="15" customHeight="1">
-      <c r="A59" s="42" t="s">
-        <v>127</v>
-      </c>
-      <c r="B59" s="42"/>
-      <c r="C59" s="42"/>
-      <c r="E59" s="41" t="s">
-        <v>158</v>
-      </c>
-      <c r="F59" s="41"/>
-      <c r="G59" s="41"/>
-      <c r="H59" s="41"/>
-      <c r="I59" s="41"/>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60" s="42"/>
-      <c r="B60" s="42"/>
-      <c r="C60" s="42"/>
-      <c r="E60" s="41"/>
-      <c r="F60" s="41"/>
-      <c r="G60" s="41"/>
-      <c r="H60" s="41"/>
-      <c r="I60" s="41"/>
-    </row>
-    <row r="61" spans="1:9">
-      <c r="A61" s="42" t="s">
-        <v>128</v>
-      </c>
-      <c r="B61" s="42"/>
-      <c r="C61" s="42"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="39"/>
-      <c r="G61" s="39"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="39"/>
-    </row>
-    <row r="62" spans="1:9">
-      <c r="A62" s="42" t="s">
-        <v>129</v>
-      </c>
-      <c r="B62" s="42"/>
-      <c r="C62" s="42"/>
-      <c r="E62" s="39" t="s">
-        <v>160</v>
-      </c>
-      <c r="F62" s="39"/>
-      <c r="G62" s="39"/>
-      <c r="H62" s="39"/>
-      <c r="I62" s="39"/>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="E63" s="40" t="s">
-        <v>159</v>
-      </c>
-      <c r="F63" s="40"/>
-      <c r="G63" s="40"/>
-      <c r="H63" s="40"/>
-      <c r="I63" s="40"/>
-    </row>
-    <row r="64" spans="1:9">
-      <c r="A64" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="B64" s="43"/>
-      <c r="C64" s="43"/>
-      <c r="E64" s="40" t="s">
-        <v>161</v>
-      </c>
-      <c r="F64" s="40"/>
-      <c r="G64" s="40"/>
-      <c r="H64" s="40"/>
-      <c r="I64" s="40"/>
-    </row>
-    <row r="65" spans="1:9">
-      <c r="A65" s="42" t="s">
-        <v>113</v>
-      </c>
-      <c r="B65" s="42"/>
-      <c r="C65" s="42"/>
-      <c r="E65" s="40" t="s">
-        <v>162</v>
-      </c>
-      <c r="F65" s="40"/>
-      <c r="G65" s="40"/>
-      <c r="H65" s="40"/>
-      <c r="I65" s="40"/>
-    </row>
-    <row r="66" spans="1:9">
-      <c r="A66" s="42" t="s">
-        <v>114</v>
-      </c>
-      <c r="B66" s="42"/>
-      <c r="C66" s="42"/>
-    </row>
-    <row r="67" spans="1:9">
-      <c r="A67" s="19"/>
-      <c r="B67" s="19"/>
-      <c r="C67" s="19"/>
-    </row>
-    <row r="68" spans="1:9">
-      <c r="A68" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="B68" s="42"/>
-      <c r="C68" s="42"/>
-    </row>
-    <row r="69" spans="1:9">
-      <c r="A69" s="42" t="s">
-        <v>116</v>
-      </c>
-      <c r="B69" s="42"/>
-      <c r="C69" s="42"/>
-    </row>
-    <row r="70" spans="1:9">
-      <c r="A70" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="B70" s="42"/>
-      <c r="C70" s="42"/>
-    </row>
-    <row r="71" spans="1:9">
-      <c r="A71" s="42" t="s">
-        <v>118</v>
-      </c>
-      <c r="B71" s="42"/>
-      <c r="C71" s="42"/>
-    </row>
-    <row r="72" spans="1:9">
-      <c r="A72" s="42" t="s">
+      <c r="J54" s="40"/>
+    </row>
+    <row r="55" spans="2:10" ht="15" customHeight="1">
+      <c r="B55" s="41" t="s">
         <v>119</v>
       </c>
-      <c r="B72" s="42"/>
-      <c r="C72" s="42"/>
+      <c r="C55" s="41"/>
+      <c r="D55" s="41"/>
+      <c r="F55" s="42" t="s">
+        <v>150</v>
+      </c>
+      <c r="G55" s="42"/>
+      <c r="H55" s="42"/>
+      <c r="I55" s="42"/>
+      <c r="J55" s="42"/>
+    </row>
+    <row r="56" spans="2:10">
+      <c r="B56" s="41"/>
+      <c r="C56" s="41"/>
+      <c r="D56" s="41"/>
+      <c r="F56" s="42"/>
+      <c r="G56" s="42"/>
+      <c r="H56" s="42"/>
+      <c r="I56" s="42"/>
+      <c r="J56" s="42"/>
+    </row>
+    <row r="57" spans="2:10">
+      <c r="B57" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="C57" s="41"/>
+      <c r="D57" s="41"/>
+      <c r="F57" s="37"/>
+      <c r="G57" s="37"/>
+      <c r="H57" s="37"/>
+      <c r="I57" s="37"/>
+      <c r="J57" s="37"/>
+    </row>
+    <row r="58" spans="2:10">
+      <c r="B58" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="C58" s="41"/>
+      <c r="D58" s="41"/>
+      <c r="F58" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="G58" s="37"/>
+      <c r="H58" s="37"/>
+      <c r="I58" s="37"/>
+      <c r="J58" s="37"/>
+    </row>
+    <row r="59" spans="2:10">
+      <c r="F59" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="G59" s="40"/>
+      <c r="H59" s="40"/>
+      <c r="I59" s="40"/>
+      <c r="J59" s="40"/>
+    </row>
+    <row r="60" spans="2:10">
+      <c r="B60" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="C60" s="36"/>
+      <c r="D60" s="36"/>
+      <c r="F60" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="G60" s="40"/>
+      <c r="H60" s="40"/>
+      <c r="I60" s="40"/>
+      <c r="J60" s="40"/>
+    </row>
+    <row r="61" spans="2:10">
+      <c r="B61" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="C61" s="41"/>
+      <c r="D61" s="41"/>
+      <c r="F61" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="G61" s="40"/>
+      <c r="H61" s="40"/>
+      <c r="I61" s="40"/>
+      <c r="J61" s="40"/>
+    </row>
+    <row r="62" spans="2:10">
+      <c r="B62" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="C62" s="41"/>
+      <c r="D62" s="41"/>
+    </row>
+    <row r="63" spans="2:10">
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+    </row>
+    <row r="64" spans="2:10">
+      <c r="B64" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="C64" s="41"/>
+      <c r="D64" s="41"/>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+    </row>
+    <row r="66" spans="2:4">
+      <c r="B66" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+    </row>
+    <row r="67" spans="2:4">
+      <c r="B67" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+    </row>
+    <row r="68" spans="2:4">
+      <c r="B68" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="C68" s="41"/>
+      <c r="D68" s="41"/>
     </row>
   </sheetData>
-  <mergeCells count="84">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="E29:I29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="E21:I21"/>
-    <mergeCell ref="E22:I22"/>
-    <mergeCell ref="E23:I23"/>
-    <mergeCell ref="E24:I24"/>
-    <mergeCell ref="E25:I25"/>
-    <mergeCell ref="E26:I26"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="H6:M6"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="E35:I35"/>
-    <mergeCell ref="E40:I44"/>
-    <mergeCell ref="E55:I55"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="E38:I38"/>
-    <mergeCell ref="E39:I39"/>
-    <mergeCell ref="E45:I45"/>
-    <mergeCell ref="E46:I46"/>
-    <mergeCell ref="E47:I47"/>
-    <mergeCell ref="E48:I48"/>
-    <mergeCell ref="E49:I49"/>
-    <mergeCell ref="E30:I30"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="E32:I32"/>
-    <mergeCell ref="E33:I33"/>
-    <mergeCell ref="E34:I34"/>
-    <mergeCell ref="E50:I50"/>
-    <mergeCell ref="E51:I51"/>
-    <mergeCell ref="E52:I52"/>
-    <mergeCell ref="E53:I53"/>
-    <mergeCell ref="E54:I54"/>
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="E63:I63"/>
-    <mergeCell ref="E64:I64"/>
-    <mergeCell ref="E65:I65"/>
-    <mergeCell ref="E56:I56"/>
-    <mergeCell ref="E57:I57"/>
-    <mergeCell ref="E58:I58"/>
-    <mergeCell ref="E61:I61"/>
-    <mergeCell ref="E59:I60"/>
+  <mergeCells count="82">
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="F58:J58"/>
+    <mergeCell ref="F59:J59"/>
+    <mergeCell ref="F60:J60"/>
+    <mergeCell ref="F61:J61"/>
+    <mergeCell ref="F52:J52"/>
+    <mergeCell ref="F53:J53"/>
+    <mergeCell ref="F54:J54"/>
+    <mergeCell ref="F57:J57"/>
+    <mergeCell ref="F55:J56"/>
+    <mergeCell ref="F46:J46"/>
+    <mergeCell ref="F47:J47"/>
+    <mergeCell ref="F48:J48"/>
+    <mergeCell ref="F49:J49"/>
+    <mergeCell ref="F50:J50"/>
+    <mergeCell ref="F26:J26"/>
+    <mergeCell ref="F27:J27"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="F36:J40"/>
+    <mergeCell ref="F51:J51"/>
+    <mergeCell ref="F32:J32"/>
+    <mergeCell ref="F33:J33"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="F42:J42"/>
+    <mergeCell ref="F43:J43"/>
+    <mergeCell ref="F44:J44"/>
+    <mergeCell ref="F45:J45"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="F25:J25"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F18:J18"/>
+    <mergeCell ref="F19:J19"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="F21:J21"/>
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="F23:J23"/>
+    <mergeCell ref="F24:J24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor enums, expand models, add sold out error handling
- Move MediaSortField and SalesSortField enums to enums_repo.py for better organization; update imports accordingly.
- Add MediaAlreadySoldOut exception and handler (406 error).
- Rename MediaTitle to Media; add amount and price fields.
- Add date field to Sale model and schema.
- Update schemas to include new fields and adjust SaleCreateSchema to use media_id.
- Add placeholders for update/delete schemas.
- Update DB_DRAFT.xlsx (details not shown).
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7536DA14-C186-4FDE-B9CD-F0FFCDCA7E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BB1D67-10D7-4D45-963D-9389F484100B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3330" yWindow="4440" windowWidth="21615" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="42855" yWindow="1080" windowWidth="21615" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="OPERATIONS" sheetId="3" r:id="rId1"/>
@@ -636,9 +636,6 @@
     <t>REAL</t>
   </si>
   <si>
-    <t>DECIMAL</t>
-  </si>
-  <si>
     <t>DATETIME</t>
   </si>
   <si>
@@ -675,6 +672,9 @@
   </si>
   <si>
     <t>List all sales records with included tblMedia records, based on MediaID, can be filtered by date range</t>
+  </si>
+  <si>
+    <t>DATE</t>
   </si>
 </sst>
 </file>
@@ -1462,7 +1462,7 @@
         <v>150</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>150</v>
@@ -1508,7 +1508,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>99</v>
@@ -1574,10 +1574,10 @@
         <v>151</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E9" s="41" t="s">
         <v>153</v>
-      </c>
-      <c r="E9" s="41" t="s">
-        <v>154</v>
       </c>
       <c r="F9" s="30"/>
     </row>
@@ -1625,7 +1625,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
@@ -1680,7 +1680,7 @@
         <v>10</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="67.5">
@@ -1689,10 +1689,10 @@
         <v>142</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="33.75">
@@ -1718,7 +1718,7 @@
         <v>144</v>
       </c>
       <c r="D21" s="39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="33.75">
@@ -1730,7 +1730,7 @@
         <v>137</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="33.75">

</xml_diff>

<commit_message>
**API /docs readibility fix**: Refactor MediaListQuerySchema to plain class with __init__
Refactored MediaListQuerySchema from a Pydantic BaseModel to a plain Python class with an explicit __init__ method, retaining all FastAPI Query parameter metadata. Updated list_media to use **query.__dict__ for cleaner argument passing. No changes to query logic or available parameters. Also updated DB_DRAFT.xlsx (details not shown).
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BB1D67-10D7-4D45-963D-9389F484100B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60939C94-5074-486E-9EF3-8A39C0BFDE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42855" yWindow="1080" windowWidth="21615" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="OPERATIONS" sheetId="3" r:id="rId1"/>
@@ -792,7 +792,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -812,6 +812,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8585"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -928,7 +946,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -941,21 +959,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -967,9 +970,45 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -977,83 +1016,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1063,6 +1065,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF8585"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1397,7 +1404,7 @@
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.42578125" customWidth="1"/>
     <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="99" customWidth="1"/>
     <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" customWidth="1"/>
@@ -1409,47 +1416,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="13" t="s">
         <v>123</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="F2" s="41" t="s">
+      <c r="F2" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="G2" s="41" t="s">
+      <c r="G2" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="41" t="s">
+      <c r="H2" s="14" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="13" t="s">
         <v>124</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1475,7 +1482,7 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="13" t="s">
         <v>125</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1501,28 +1508,28 @@
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="47">
+      <c r="B5" s="16">
         <v>1</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C5" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="D5" s="47" t="s">
+      <c r="D5" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="E5" s="47">
+      <c r="E5" s="16">
         <v>2015</v>
       </c>
-      <c r="F5" s="47" t="s">
+      <c r="F5" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="G5" s="48">
+      <c r="G5" s="17">
         <v>67</v>
       </c>
-      <c r="H5" s="42">
+      <c r="H5" s="15">
         <v>420</v>
       </c>
     </row>
@@ -1534,19 +1541,19 @@
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="28"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="13" t="s">
         <v>123</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -1558,13 +1565,12 @@
       <c r="D8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F8" s="30"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="13" t="s">
         <v>124</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1576,13 +1582,12 @@
       <c r="D9" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="F9" s="30"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="13" t="s">
         <v>125</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1594,25 +1599,24 @@
       <c r="D10" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="F10" s="30"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="47">
+      <c r="B11" s="16">
         <v>1</v>
       </c>
-      <c r="C11" s="47">
+      <c r="C11" s="16">
         <v>1</v>
       </c>
-      <c r="D11" s="48">
+      <c r="D11" s="17">
         <v>420</v>
       </c>
-      <c r="E11" s="49">
+      <c r="E11" s="18">
         <v>46053.903506944444</v>
       </c>
       <c r="F11" s="1"/>
@@ -1624,142 +1628,142 @@
       <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="43" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="101.25">
-      <c r="A16" s="43" t="s">
+    <row r="16" spans="1:8" ht="90">
+      <c r="A16" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="33" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="22.5">
-      <c r="A17" s="43"/>
-      <c r="B17" s="45" t="s">
+    <row r="17" spans="1:12">
+      <c r="A17" s="19"/>
+      <c r="B17" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="32" t="s">
         <v>134</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="33" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="101.25">
-      <c r="A18" s="43"/>
-      <c r="B18" s="45" t="s">
+    <row r="18" spans="1:12" ht="78.75">
+      <c r="A18" s="19"/>
+      <c r="B18" s="34" t="s">
         <v>140</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="38" t="s">
+      <c r="D18" s="36" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="67.5">
-      <c r="A19" s="43"/>
-      <c r="B19" s="45" t="s">
+    <row r="19" spans="1:12" ht="45">
+      <c r="A19" s="19"/>
+      <c r="B19" s="34" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="D19" s="38" t="s">
+      <c r="D19" s="36" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="33.75">
-      <c r="A20" s="43"/>
-      <c r="B20" s="46" t="s">
+    <row r="20" spans="1:12">
+      <c r="A20" s="19"/>
+      <c r="B20" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="37" t="s">
+      <c r="C20" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="39" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="90">
-      <c r="A21" s="43" t="s">
+    <row r="21" spans="1:12" ht="78.75">
+      <c r="A21" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="40" t="s">
         <v>135</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="36" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="33.75">
-      <c r="A22" s="43"/>
-      <c r="B22" s="6" t="s">
+    <row r="22" spans="1:12">
+      <c r="A22" s="19"/>
+      <c r="B22" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="35" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="D22" s="36" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="33.75">
-      <c r="A23" s="43"/>
-      <c r="B23" s="35" t="s">
+    <row r="23" spans="1:12">
+      <c r="A23" s="19"/>
+      <c r="B23" s="41" t="s">
         <v>139</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="40" t="s">
+      <c r="D23" s="39" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="33.75">
-      <c r="A24" s="43"/>
-      <c r="B24" s="34" t="s">
+    <row r="24" spans="1:12">
+      <c r="A24" s="19"/>
+      <c r="B24" s="41" t="s">
         <v>138</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="40" t="s">
+      <c r="D24" s="39" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="25" spans="1:12">
       <c r="B25" s="1"/>
-      <c r="C25" s="29"/>
+      <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:12">
       <c r="B26" s="1"/>
@@ -1775,18 +1779,18 @@
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="F29" s="22" t="s">
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="F29" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
     </row>
     <row r="30" spans="1:12">
       <c r="B30" t="s">
@@ -1798,163 +1802,163 @@
       <c r="D30" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="22" t="s">
+      <c r="F30" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
     </row>
     <row r="31" spans="1:12">
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="25" t="s">
+      <c r="F31" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="G31" s="25"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="25"/>
-      <c r="J31" s="25"/>
-      <c r="K31" s="19" t="s">
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="L31" s="20"/>
+      <c r="L31" s="29"/>
     </row>
     <row r="32" spans="1:12">
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="25" t="s">
+      <c r="F32" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25"/>
-      <c r="J32" s="25"/>
-      <c r="K32" s="16" t="s">
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="L32" s="17" t="s">
+      <c r="L32" s="12" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="33" spans="2:12">
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="25" t="s">
+      <c r="F33" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="14" t="s">
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="L33" s="12" t="s">
+      <c r="L33" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="2:12">
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F34" s="25" t="s">
+      <c r="F34" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="25"/>
-      <c r="J34" s="25"/>
-      <c r="K34" s="14" t="s">
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="L34" s="12" t="s">
+      <c r="L34" s="7" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="35" spans="2:12">
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F35" s="25" t="s">
+      <c r="F35" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="G35" s="25"/>
-      <c r="H35" s="25"/>
-      <c r="I35" s="25"/>
-      <c r="J35" s="25"/>
-      <c r="K35" s="14" t="s">
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="L35" s="12" t="s">
+      <c r="L35" s="7" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="36" spans="2:12">
-      <c r="D36" s="10"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
-      <c r="K36" s="14" t="s">
+      <c r="D36" s="5"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="L36" s="12" t="s">
+      <c r="L36" s="7" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="37" spans="2:12">
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="F37" s="22" t="s">
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="F37" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
-      <c r="K37" s="14" t="s">
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="L37" s="12" t="s">
+      <c r="L37" s="7" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1964,17 +1968,17 @@
       </c>
       <c r="C38" s="26"/>
       <c r="D38" s="26"/>
-      <c r="F38" s="25" t="s">
+      <c r="F38" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="G38" s="25"/>
-      <c r="H38" s="25"/>
-      <c r="I38" s="25"/>
-      <c r="J38" s="25"/>
-      <c r="K38" s="14" t="s">
+      <c r="G38" s="24"/>
+      <c r="H38" s="24"/>
+      <c r="I38" s="24"/>
+      <c r="J38" s="24"/>
+      <c r="K38" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="L38" s="12" t="s">
+      <c r="L38" s="7" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1984,17 +1988,17 @@
       </c>
       <c r="C39" s="26"/>
       <c r="D39" s="26"/>
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="25"/>
-      <c r="K39" s="14" t="s">
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="24"/>
+      <c r="J39" s="24"/>
+      <c r="K39" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="L39" s="12" t="s">
+      <c r="L39" s="7" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2004,15 +2008,15 @@
       </c>
       <c r="C40" s="26"/>
       <c r="D40" s="26"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="15" t="s">
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="L40" s="13" t="s">
+      <c r="L40" s="8" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2022,36 +2026,36 @@
       </c>
       <c r="C41" s="26"/>
       <c r="D41" s="26"/>
-      <c r="F41" s="22" t="s">
+      <c r="F41" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
     </row>
     <row r="42" spans="2:12">
-      <c r="F42" s="25" t="s">
+      <c r="F42" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="G42" s="25"/>
-      <c r="H42" s="25"/>
-      <c r="I42" s="25"/>
-      <c r="J42" s="25"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="24"/>
+      <c r="I42" s="24"/>
+      <c r="J42" s="24"/>
     </row>
     <row r="43" spans="2:12">
-      <c r="B43" s="21" t="s">
+      <c r="B43" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C43" s="21"/>
-      <c r="D43" s="21"/>
-      <c r="F43" s="25" t="s">
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
+      <c r="F43" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="G43" s="25"/>
-      <c r="H43" s="25"/>
-      <c r="I43" s="25"/>
-      <c r="J43" s="25"/>
+      <c r="G43" s="24"/>
+      <c r="H43" s="24"/>
+      <c r="I43" s="24"/>
+      <c r="J43" s="24"/>
     </row>
     <row r="44" spans="2:12">
       <c r="B44" s="26" t="s">
@@ -2059,13 +2063,13 @@
       </c>
       <c r="C44" s="26"/>
       <c r="D44" s="26"/>
-      <c r="F44" s="25" t="s">
+      <c r="F44" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="G44" s="25"/>
-      <c r="H44" s="25"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="25"/>
+      <c r="G44" s="24"/>
+      <c r="H44" s="24"/>
+      <c r="I44" s="24"/>
+      <c r="J44" s="24"/>
     </row>
     <row r="45" spans="2:12">
       <c r="B45" s="26" t="s">
@@ -2073,11 +2077,11 @@
       </c>
       <c r="C45" s="26"/>
       <c r="D45" s="26"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23"/>
     </row>
     <row r="46" spans="2:12">
       <c r="B46" s="26" t="s">
@@ -2085,13 +2089,13 @@
       </c>
       <c r="C46" s="26"/>
       <c r="D46" s="26"/>
-      <c r="F46" s="22" t="s">
+      <c r="F46" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
     </row>
     <row r="47" spans="2:12">
       <c r="B47" s="26" t="s">
@@ -2099,25 +2103,25 @@
       </c>
       <c r="C47" s="26"/>
       <c r="D47" s="26"/>
-      <c r="F47" s="25" t="s">
+      <c r="F47" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="G47" s="25"/>
-      <c r="H47" s="25"/>
-      <c r="I47" s="25"/>
-      <c r="J47" s="25"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="24"/>
+      <c r="I47" s="24"/>
+      <c r="J47" s="24"/>
     </row>
     <row r="48" spans="2:12" ht="15" customHeight="1">
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="F48" s="27" t="s">
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
+      <c r="F48" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="27"/>
-      <c r="J48" s="27"/>
+      <c r="G48" s="25"/>
+      <c r="H48" s="25"/>
+      <c r="I48" s="25"/>
+      <c r="J48" s="25"/>
     </row>
     <row r="49" spans="2:10">
       <c r="B49" s="26" t="s">
@@ -2125,11 +2129,11 @@
       </c>
       <c r="C49" s="26"/>
       <c r="D49" s="26"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="27"/>
-      <c r="I49" s="27"/>
-      <c r="J49" s="27"/>
+      <c r="F49" s="25"/>
+      <c r="G49" s="25"/>
+      <c r="H49" s="25"/>
+      <c r="I49" s="25"/>
+      <c r="J49" s="25"/>
     </row>
     <row r="50" spans="2:10">
       <c r="B50" s="26" t="s">
@@ -2137,11 +2141,11 @@
       </c>
       <c r="C50" s="26"/>
       <c r="D50" s="26"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="H50" s="27"/>
-      <c r="I50" s="27"/>
-      <c r="J50" s="27"/>
+      <c r="F50" s="25"/>
+      <c r="G50" s="25"/>
+      <c r="H50" s="25"/>
+      <c r="I50" s="25"/>
+      <c r="J50" s="25"/>
     </row>
     <row r="51" spans="2:10">
       <c r="B51" s="26" t="s">
@@ -2149,11 +2153,11 @@
       </c>
       <c r="C51" s="26"/>
       <c r="D51" s="26"/>
-      <c r="F51" s="27"/>
-      <c r="G51" s="27"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="27"/>
-      <c r="J51" s="27"/>
+      <c r="F51" s="25"/>
+      <c r="G51" s="25"/>
+      <c r="H51" s="25"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="25"/>
     </row>
     <row r="52" spans="2:10">
       <c r="B52" s="26" t="s">
@@ -2161,21 +2165,21 @@
       </c>
       <c r="C52" s="26"/>
       <c r="D52" s="26"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
-      <c r="I52" s="27"/>
-      <c r="J52" s="27"/>
+      <c r="F52" s="25"/>
+      <c r="G52" s="25"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25"/>
     </row>
     <row r="53" spans="2:10">
-      <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="23"/>
+      <c r="J53" s="23"/>
     </row>
     <row r="54" spans="2:10">
       <c r="B54" s="26" t="s">
@@ -2183,13 +2187,13 @@
       </c>
       <c r="C54" s="26"/>
       <c r="D54" s="26"/>
-      <c r="F54" s="22" t="s">
+      <c r="F54" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="G54" s="22"/>
-      <c r="H54" s="22"/>
-      <c r="I54" s="22"/>
-      <c r="J54" s="22"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="23"/>
     </row>
     <row r="55" spans="2:10">
       <c r="B55" s="26" t="s">
@@ -2197,13 +2201,13 @@
       </c>
       <c r="C55" s="26"/>
       <c r="D55" s="26"/>
-      <c r="F55" s="25" t="s">
+      <c r="F55" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="G55" s="25"/>
-      <c r="H55" s="25"/>
-      <c r="I55" s="25"/>
-      <c r="J55" s="25"/>
+      <c r="G55" s="24"/>
+      <c r="H55" s="24"/>
+      <c r="I55" s="24"/>
+      <c r="J55" s="24"/>
     </row>
     <row r="56" spans="2:10">
       <c r="B56" s="26" t="s">
@@ -2211,25 +2215,25 @@
       </c>
       <c r="C56" s="26"/>
       <c r="D56" s="26"/>
-      <c r="F56" s="25" t="s">
+      <c r="F56" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="G56" s="25"/>
-      <c r="H56" s="25"/>
-      <c r="I56" s="25"/>
-      <c r="J56" s="25"/>
+      <c r="G56" s="24"/>
+      <c r="H56" s="24"/>
+      <c r="I56" s="24"/>
+      <c r="J56" s="24"/>
     </row>
     <row r="57" spans="2:10">
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="F57" s="25" t="s">
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="F57" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="G57" s="25"/>
-      <c r="H57" s="25"/>
-      <c r="I57" s="25"/>
-      <c r="J57" s="25"/>
+      <c r="G57" s="24"/>
+      <c r="H57" s="24"/>
+      <c r="I57" s="24"/>
+      <c r="J57" s="24"/>
     </row>
     <row r="58" spans="2:10">
       <c r="B58" s="26" t="s">
@@ -2237,13 +2241,13 @@
       </c>
       <c r="C58" s="26"/>
       <c r="D58" s="26"/>
-      <c r="F58" s="25" t="s">
+      <c r="F58" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="G58" s="25"/>
-      <c r="H58" s="25"/>
-      <c r="I58" s="25"/>
-      <c r="J58" s="25"/>
+      <c r="G58" s="24"/>
+      <c r="H58" s="24"/>
+      <c r="I58" s="24"/>
+      <c r="J58" s="24"/>
     </row>
     <row r="59" spans="2:10">
       <c r="B59" s="26" t="s">
@@ -2251,13 +2255,13 @@
       </c>
       <c r="C59" s="26"/>
       <c r="D59" s="26"/>
-      <c r="F59" s="25" t="s">
+      <c r="F59" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="G59" s="25"/>
-      <c r="H59" s="25"/>
-      <c r="I59" s="25"/>
-      <c r="J59" s="25"/>
+      <c r="G59" s="24"/>
+      <c r="H59" s="24"/>
+      <c r="I59" s="24"/>
+      <c r="J59" s="24"/>
     </row>
     <row r="60" spans="2:10">
       <c r="B60" s="26" t="s">
@@ -2265,11 +2269,11 @@
       </c>
       <c r="C60" s="26"/>
       <c r="D60" s="26"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="23"/>
+      <c r="H60" s="23"/>
+      <c r="I60" s="23"/>
+      <c r="J60" s="23"/>
     </row>
     <row r="61" spans="2:10">
       <c r="B61" s="26" t="s">
@@ -2277,25 +2281,25 @@
       </c>
       <c r="C61" s="26"/>
       <c r="D61" s="26"/>
-      <c r="F61" s="22" t="s">
+      <c r="F61" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="G61" s="22"/>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
+      <c r="G61" s="23"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="23"/>
     </row>
     <row r="62" spans="2:10">
       <c r="B62" s="26"/>
       <c r="C62" s="26"/>
       <c r="D62" s="26"/>
-      <c r="F62" s="25" t="s">
+      <c r="F62" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="G62" s="25"/>
-      <c r="H62" s="25"/>
-      <c r="I62" s="25"/>
-      <c r="J62" s="25"/>
+      <c r="G62" s="24"/>
+      <c r="H62" s="24"/>
+      <c r="I62" s="24"/>
+      <c r="J62" s="24"/>
     </row>
     <row r="63" spans="2:10">
       <c r="B63" s="26" t="s">
@@ -2303,13 +2307,13 @@
       </c>
       <c r="C63" s="26"/>
       <c r="D63" s="26"/>
-      <c r="F63" s="25" t="s">
+      <c r="F63" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="25"/>
-      <c r="J63" s="25"/>
+      <c r="G63" s="24"/>
+      <c r="H63" s="24"/>
+      <c r="I63" s="24"/>
+      <c r="J63" s="24"/>
     </row>
     <row r="64" spans="2:10">
       <c r="B64" s="26" t="s">
@@ -2317,11 +2321,11 @@
       </c>
       <c r="C64" s="26"/>
       <c r="D64" s="26"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="22"/>
+      <c r="F64" s="23"/>
+      <c r="G64" s="23"/>
+      <c r="H64" s="23"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="23"/>
     </row>
     <row r="65" spans="2:10">
       <c r="B65" s="26" t="s">
@@ -2329,13 +2333,13 @@
       </c>
       <c r="C65" s="26"/>
       <c r="D65" s="26"/>
-      <c r="F65" s="22" t="s">
+      <c r="F65" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="G65" s="22"/>
-      <c r="H65" s="22"/>
-      <c r="I65" s="22"/>
-      <c r="J65" s="22"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="23"/>
+      <c r="I65" s="23"/>
+      <c r="J65" s="23"/>
     </row>
     <row r="66" spans="2:10">
       <c r="B66" s="26" t="s">
@@ -2343,13 +2347,13 @@
       </c>
       <c r="C66" s="26"/>
       <c r="D66" s="26"/>
-      <c r="F66" s="25" t="s">
+      <c r="F66" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="G66" s="25"/>
-      <c r="H66" s="25"/>
-      <c r="I66" s="25"/>
-      <c r="J66" s="25"/>
+      <c r="G66" s="24"/>
+      <c r="H66" s="24"/>
+      <c r="I66" s="24"/>
+      <c r="J66" s="24"/>
     </row>
     <row r="67" spans="2:10" ht="15" customHeight="1">
       <c r="B67" s="26" t="s">
@@ -2357,23 +2361,23 @@
       </c>
       <c r="C67" s="26"/>
       <c r="D67" s="26"/>
-      <c r="F67" s="27" t="s">
+      <c r="F67" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="G67" s="27"/>
-      <c r="H67" s="27"/>
-      <c r="I67" s="27"/>
-      <c r="J67" s="27"/>
+      <c r="G67" s="25"/>
+      <c r="H67" s="25"/>
+      <c r="I67" s="25"/>
+      <c r="J67" s="25"/>
     </row>
     <row r="68" spans="2:10">
       <c r="B68" s="26"/>
       <c r="C68" s="26"/>
       <c r="D68" s="26"/>
-      <c r="F68" s="27"/>
-      <c r="G68" s="27"/>
-      <c r="H68" s="27"/>
-      <c r="I68" s="27"/>
-      <c r="J68" s="27"/>
+      <c r="F68" s="25"/>
+      <c r="G68" s="25"/>
+      <c r="H68" s="25"/>
+      <c r="I68" s="25"/>
+      <c r="J68" s="25"/>
     </row>
     <row r="69" spans="2:10">
       <c r="B69" s="26" t="s">
@@ -2381,11 +2385,11 @@
       </c>
       <c r="C69" s="26"/>
       <c r="D69" s="26"/>
-      <c r="F69" s="22"/>
-      <c r="G69" s="22"/>
-      <c r="H69" s="22"/>
-      <c r="I69" s="22"/>
-      <c r="J69" s="22"/>
+      <c r="F69" s="23"/>
+      <c r="G69" s="23"/>
+      <c r="H69" s="23"/>
+      <c r="I69" s="23"/>
+      <c r="J69" s="23"/>
     </row>
     <row r="70" spans="2:10">
       <c r="B70" s="26" t="s">
@@ -2393,36 +2397,36 @@
       </c>
       <c r="C70" s="26"/>
       <c r="D70" s="26"/>
-      <c r="F70" s="22" t="s">
+      <c r="F70" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="22"/>
+      <c r="G70" s="23"/>
+      <c r="H70" s="23"/>
+      <c r="I70" s="23"/>
+      <c r="J70" s="23"/>
     </row>
     <row r="71" spans="2:10">
-      <c r="F71" s="25" t="s">
+      <c r="F71" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="G71" s="25"/>
-      <c r="H71" s="25"/>
-      <c r="I71" s="25"/>
-      <c r="J71" s="25"/>
+      <c r="G71" s="24"/>
+      <c r="H71" s="24"/>
+      <c r="I71" s="24"/>
+      <c r="J71" s="24"/>
     </row>
     <row r="72" spans="2:10">
-      <c r="B72" s="21" t="s">
+      <c r="B72" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C72" s="21"/>
-      <c r="D72" s="21"/>
-      <c r="F72" s="25" t="s">
+      <c r="C72" s="27"/>
+      <c r="D72" s="27"/>
+      <c r="F72" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="G72" s="25"/>
-      <c r="H72" s="25"/>
-      <c r="I72" s="25"/>
-      <c r="J72" s="25"/>
+      <c r="G72" s="24"/>
+      <c r="H72" s="24"/>
+      <c r="I72" s="24"/>
+      <c r="J72" s="24"/>
     </row>
     <row r="73" spans="2:10">
       <c r="B73" s="26" t="s">
@@ -2430,13 +2434,13 @@
       </c>
       <c r="C73" s="26"/>
       <c r="D73" s="26"/>
-      <c r="F73" s="25" t="s">
+      <c r="F73" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="G73" s="25"/>
-      <c r="H73" s="25"/>
-      <c r="I73" s="25"/>
-      <c r="J73" s="25"/>
+      <c r="G73" s="24"/>
+      <c r="H73" s="24"/>
+      <c r="I73" s="24"/>
+      <c r="J73" s="24"/>
     </row>
     <row r="74" spans="2:10">
       <c r="B74" s="26" t="s">
@@ -2446,9 +2450,9 @@
       <c r="D74" s="26"/>
     </row>
     <row r="75" spans="2:10">
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="11"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6"/>
+      <c r="D75" s="6"/>
     </row>
     <row r="76" spans="2:10">
       <c r="B76" s="26" t="s">
@@ -2487,30 +2491,51 @@
     </row>
   </sheetData>
   <mergeCells count="85">
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A16:A20"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="F70:J70"/>
-    <mergeCell ref="F71:J71"/>
-    <mergeCell ref="F72:J72"/>
-    <mergeCell ref="F73:J73"/>
-    <mergeCell ref="F64:J64"/>
-    <mergeCell ref="F65:J65"/>
-    <mergeCell ref="F66:J66"/>
-    <mergeCell ref="F69:J69"/>
-    <mergeCell ref="F67:J68"/>
-    <mergeCell ref="F58:J58"/>
-    <mergeCell ref="F59:J59"/>
-    <mergeCell ref="F60:J60"/>
-    <mergeCell ref="F61:J61"/>
-    <mergeCell ref="F62:J62"/>
-    <mergeCell ref="F38:J38"/>
-    <mergeCell ref="F39:J39"/>
-    <mergeCell ref="F40:J40"/>
-    <mergeCell ref="F41:J41"/>
-    <mergeCell ref="F42:J42"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="F37:J37"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="F32:J32"/>
+    <mergeCell ref="F33:J33"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="F36:J36"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B65:D65"/>
     <mergeCell ref="B66:D66"/>
     <mergeCell ref="B67:D67"/>
     <mergeCell ref="B68:D68"/>
@@ -2527,51 +2552,30 @@
     <mergeCell ref="F55:J55"/>
     <mergeCell ref="F56:J56"/>
     <mergeCell ref="F57:J57"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B74:D74"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="B79:D79"/>
-    <mergeCell ref="B78:D78"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="F37:J37"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="F32:J32"/>
-    <mergeCell ref="F33:J33"/>
-    <mergeCell ref="F34:J34"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="F36:J36"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="F39:J39"/>
+    <mergeCell ref="F40:J40"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="F42:J42"/>
+    <mergeCell ref="F58:J58"/>
+    <mergeCell ref="F59:J59"/>
+    <mergeCell ref="F60:J60"/>
+    <mergeCell ref="F61:J61"/>
+    <mergeCell ref="F62:J62"/>
+    <mergeCell ref="F70:J70"/>
+    <mergeCell ref="F71:J71"/>
+    <mergeCell ref="F72:J72"/>
+    <mergeCell ref="F73:J73"/>
+    <mergeCell ref="F64:J64"/>
+    <mergeCell ref="F65:J65"/>
+    <mergeCell ref="F66:J66"/>
+    <mergeCell ref="F69:J69"/>
+    <mergeCell ref="F67:J68"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor media update logic, add validation & error handling
Expanded error handling with InvalidValueError and InvalidKeyError, including FastAPI handlers for 403 responses. Refactored media creation and update endpoints to use schema objects and enforce validation (e.g., quantity and price >= 0, Title+MediaType uniqueness). Updated MediaUpdateSchema to forbid extra fields and require minimum lengths. Rewrote media_repo.update to update all fields at once and return the updated object. Updated binary files to support new logic. API now returns updated media record on PUT.
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60939C94-5074-486E-9EF3-8A39C0BFDE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9014823B-8156-48B9-A6CE-39750B21B7FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="4785" yWindow="4185" windowWidth="31755" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="OPERATIONS" sheetId="3" r:id="rId1"/>
@@ -986,6 +986,65 @@
     <xf numFmtId="22" fontId="15" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -996,65 +1055,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1419,15 +1419,15 @@
       <c r="A1" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="13" t="s">
@@ -1544,12 +1544,12 @@
       <c r="A7" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:8">
@@ -1628,136 +1628,136 @@
       <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="41" t="s">
         <v>155</v>
       </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="43" t="s">
+      <c r="C15" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="31" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="90">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="40" t="s">
         <v>129</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="33" t="s">
+      <c r="D16" s="21" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:12">
-      <c r="A17" s="19"/>
-      <c r="B17" s="31" t="s">
+      <c r="A17" s="40"/>
+      <c r="B17" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="D17" s="33" t="s">
+      <c r="D17" s="21" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="78.75">
-      <c r="A18" s="19"/>
-      <c r="B18" s="34" t="s">
+      <c r="A18" s="40"/>
+      <c r="B18" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="36" t="s">
+      <c r="D18" s="24" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="45">
-      <c r="A19" s="19"/>
-      <c r="B19" s="34" t="s">
+      <c r="A19" s="40"/>
+      <c r="B19" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="D19" s="36" t="s">
+      <c r="D19" s="24" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:12">
-      <c r="A20" s="19"/>
-      <c r="B20" s="37" t="s">
+      <c r="A20" s="40"/>
+      <c r="B20" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="27" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="78.75">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="24" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:12">
-      <c r="A22" s="19"/>
-      <c r="B22" s="40" t="s">
+      <c r="A22" s="40"/>
+      <c r="B22" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="24" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:12">
-      <c r="A23" s="19"/>
-      <c r="B23" s="41" t="s">
+      <c r="A23" s="40"/>
+      <c r="B23" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="C23" s="42" t="s">
+      <c r="C23" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="27" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="19"/>
-      <c r="B24" s="41" t="s">
+      <c r="A24" s="40"/>
+      <c r="B24" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C24" s="42" t="s">
+      <c r="C24" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="27" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1779,18 +1779,18 @@
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="B29" s="30" t="s">
+      <c r="B29" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="F29" s="23" t="s">
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="F29" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
     </row>
     <row r="30" spans="1:12">
       <c r="B30" t="s">
@@ -1802,13 +1802,13 @@
       <c r="D30" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
     </row>
     <row r="31" spans="1:12">
       <c r="B31" s="5" t="s">
@@ -1820,17 +1820,17 @@
       <c r="D31" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="24" t="s">
+      <c r="F31" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="24"/>
-      <c r="J31" s="24"/>
-      <c r="K31" s="28" t="s">
+      <c r="G31" s="37"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="37"/>
+      <c r="K31" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="L31" s="29"/>
+      <c r="L31" s="33"/>
     </row>
     <row r="32" spans="1:12">
       <c r="B32" s="5" t="s">
@@ -1842,13 +1842,13 @@
       <c r="D32" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="24" t="s">
+      <c r="F32" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="37"/>
       <c r="K32" s="11" t="s">
         <v>105</v>
       </c>
@@ -1866,13 +1866,13 @@
       <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="24" t="s">
+      <c r="F33" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="9" t="s">
         <v>107</v>
       </c>
@@ -1890,13 +1890,13 @@
       <c r="D34" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F34" s="24" t="s">
+      <c r="F34" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="37"/>
       <c r="K34" s="9" t="s">
         <v>108</v>
       </c>
@@ -1914,13 +1914,13 @@
       <c r="D35" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F35" s="24" t="s">
+      <c r="F35" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
-      <c r="J35" s="24"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="37"/>
       <c r="K35" s="9" t="s">
         <v>109</v>
       </c>
@@ -1930,11 +1930,11 @@
     </row>
     <row r="36" spans="2:12">
       <c r="D36" s="5"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
+      <c r="F36" s="35"/>
+      <c r="G36" s="35"/>
+      <c r="H36" s="35"/>
+      <c r="I36" s="35"/>
+      <c r="J36" s="35"/>
       <c r="K36" s="9" t="s">
         <v>110</v>
       </c>
@@ -1943,18 +1943,18 @@
       </c>
     </row>
     <row r="37" spans="2:12">
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="F37" s="23" t="s">
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="F37" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="23"/>
+      <c r="G37" s="35"/>
+      <c r="H37" s="35"/>
+      <c r="I37" s="35"/>
+      <c r="J37" s="35"/>
       <c r="K37" s="9" t="s">
         <v>112</v>
       </c>
@@ -1963,18 +1963,18 @@
       </c>
     </row>
     <row r="38" spans="2:12">
-      <c r="B38" s="26" t="s">
+      <c r="B38" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="F38" s="24" t="s">
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="F38" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="24"/>
-      <c r="J38" s="24"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="37"/>
+      <c r="I38" s="37"/>
+      <c r="J38" s="37"/>
       <c r="K38" s="9" t="s">
         <v>114</v>
       </c>
@@ -1983,18 +1983,18 @@
       </c>
     </row>
     <row r="39" spans="2:12">
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="F39" s="24" t="s">
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="F39" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="G39" s="24"/>
-      <c r="H39" s="24"/>
-      <c r="I39" s="24"/>
-      <c r="J39" s="24"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="37"/>
+      <c r="I39" s="37"/>
+      <c r="J39" s="37"/>
       <c r="K39" s="9" t="s">
         <v>116</v>
       </c>
@@ -2003,16 +2003,16 @@
       </c>
     </row>
     <row r="40" spans="2:12">
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="F40" s="35"/>
+      <c r="G40" s="35"/>
+      <c r="H40" s="35"/>
+      <c r="I40" s="35"/>
+      <c r="J40" s="35"/>
       <c r="K40" s="10" t="s">
         <v>118</v>
       </c>
@@ -2021,433 +2021,433 @@
       </c>
     </row>
     <row r="41" spans="2:12">
-      <c r="B41" s="26" t="s">
+      <c r="B41" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="F41" s="23" t="s">
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="F41" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="G41" s="23"/>
-      <c r="H41" s="23"/>
-      <c r="I41" s="23"/>
-      <c r="J41" s="23"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
     </row>
     <row r="42" spans="2:12">
-      <c r="F42" s="24" t="s">
+      <c r="F42" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="G42" s="24"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="24"/>
-      <c r="J42" s="24"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="37"/>
+      <c r="I42" s="37"/>
+      <c r="J42" s="37"/>
     </row>
     <row r="43" spans="2:12">
-      <c r="B43" s="27" t="s">
+      <c r="B43" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
-      <c r="F43" s="24" t="s">
+      <c r="C43" s="34"/>
+      <c r="D43" s="34"/>
+      <c r="F43" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="G43" s="24"/>
-      <c r="H43" s="24"/>
-      <c r="I43" s="24"/>
-      <c r="J43" s="24"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="37"/>
+      <c r="I43" s="37"/>
+      <c r="J43" s="37"/>
     </row>
     <row r="44" spans="2:12">
-      <c r="B44" s="26" t="s">
+      <c r="B44" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="26"/>
-      <c r="D44" s="26"/>
-      <c r="F44" s="24" t="s">
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="F44" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="G44" s="24"/>
-      <c r="H44" s="24"/>
-      <c r="I44" s="24"/>
-      <c r="J44" s="24"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="37"/>
+      <c r="I44" s="37"/>
+      <c r="J44" s="37"/>
     </row>
     <row r="45" spans="2:12">
-      <c r="B45" s="26" t="s">
+      <c r="B45" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="23"/>
-      <c r="I45" s="23"/>
-      <c r="J45" s="23"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="F45" s="35"/>
+      <c r="G45" s="35"/>
+      <c r="H45" s="35"/>
+      <c r="I45" s="35"/>
+      <c r="J45" s="35"/>
     </row>
     <row r="46" spans="2:12">
-      <c r="B46" s="26" t="s">
+      <c r="B46" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="26"/>
-      <c r="D46" s="26"/>
-      <c r="F46" s="23" t="s">
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
+      <c r="F46" s="35" t="s">
         <v>78</v>
       </c>
-      <c r="G46" s="23"/>
-      <c r="H46" s="23"/>
-      <c r="I46" s="23"/>
-      <c r="J46" s="23"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="35"/>
+      <c r="J46" s="35"/>
     </row>
     <row r="47" spans="2:12">
-      <c r="B47" s="26" t="s">
+      <c r="B47" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="F47" s="24" t="s">
+      <c r="C47" s="38"/>
+      <c r="D47" s="38"/>
+      <c r="F47" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="G47" s="24"/>
-      <c r="H47" s="24"/>
-      <c r="I47" s="24"/>
-      <c r="J47" s="24"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37"/>
+      <c r="I47" s="37"/>
+      <c r="J47" s="37"/>
     </row>
     <row r="48" spans="2:12" ht="15" customHeight="1">
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
-      <c r="F48" s="25" t="s">
+      <c r="F48" s="39" t="s">
         <v>80</v>
       </c>
-      <c r="G48" s="25"/>
-      <c r="H48" s="25"/>
-      <c r="I48" s="25"/>
-      <c r="J48" s="25"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="39"/>
+      <c r="I48" s="39"/>
+      <c r="J48" s="39"/>
     </row>
     <row r="49" spans="2:10">
-      <c r="B49" s="26" t="s">
+      <c r="B49" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="26"/>
-      <c r="D49" s="26"/>
-      <c r="F49" s="25"/>
-      <c r="G49" s="25"/>
-      <c r="H49" s="25"/>
-      <c r="I49" s="25"/>
-      <c r="J49" s="25"/>
+      <c r="C49" s="38"/>
+      <c r="D49" s="38"/>
+      <c r="F49" s="39"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="39"/>
+      <c r="I49" s="39"/>
+      <c r="J49" s="39"/>
     </row>
     <row r="50" spans="2:10">
-      <c r="B50" s="26" t="s">
+      <c r="B50" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="F50" s="25"/>
-      <c r="G50" s="25"/>
-      <c r="H50" s="25"/>
-      <c r="I50" s="25"/>
-      <c r="J50" s="25"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="38"/>
+      <c r="F50" s="39"/>
+      <c r="G50" s="39"/>
+      <c r="H50" s="39"/>
+      <c r="I50" s="39"/>
+      <c r="J50" s="39"/>
     </row>
     <row r="51" spans="2:10">
-      <c r="B51" s="26" t="s">
+      <c r="B51" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="F51" s="25"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="25"/>
-      <c r="I51" s="25"/>
-      <c r="J51" s="25"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="38"/>
+      <c r="F51" s="39"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="39"/>
+      <c r="I51" s="39"/>
+      <c r="J51" s="39"/>
     </row>
     <row r="52" spans="2:10">
-      <c r="B52" s="26" t="s">
+      <c r="B52" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="F52" s="25"/>
-      <c r="G52" s="25"/>
-      <c r="H52" s="25"/>
-      <c r="I52" s="25"/>
-      <c r="J52" s="25"/>
+      <c r="C52" s="38"/>
+      <c r="D52" s="38"/>
+      <c r="F52" s="39"/>
+      <c r="G52" s="39"/>
+      <c r="H52" s="39"/>
+      <c r="I52" s="39"/>
+      <c r="J52" s="39"/>
     </row>
     <row r="53" spans="2:10">
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
       <c r="D53" s="6"/>
-      <c r="F53" s="23"/>
-      <c r="G53" s="23"/>
-      <c r="H53" s="23"/>
-      <c r="I53" s="23"/>
-      <c r="J53" s="23"/>
+      <c r="F53" s="35"/>
+      <c r="G53" s="35"/>
+      <c r="H53" s="35"/>
+      <c r="I53" s="35"/>
+      <c r="J53" s="35"/>
     </row>
     <row r="54" spans="2:10">
-      <c r="B54" s="26" t="s">
+      <c r="B54" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="C54" s="26"/>
-      <c r="D54" s="26"/>
-      <c r="F54" s="23" t="s">
+      <c r="C54" s="38"/>
+      <c r="D54" s="38"/>
+      <c r="F54" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="J54" s="23"/>
+      <c r="G54" s="35"/>
+      <c r="H54" s="35"/>
+      <c r="I54" s="35"/>
+      <c r="J54" s="35"/>
     </row>
     <row r="55" spans="2:10">
-      <c r="B55" s="26" t="s">
+      <c r="B55" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="F55" s="24" t="s">
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="F55" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="G55" s="24"/>
-      <c r="H55" s="24"/>
-      <c r="I55" s="24"/>
-      <c r="J55" s="24"/>
+      <c r="G55" s="37"/>
+      <c r="H55" s="37"/>
+      <c r="I55" s="37"/>
+      <c r="J55" s="37"/>
     </row>
     <row r="56" spans="2:10">
-      <c r="B56" s="26" t="s">
+      <c r="B56" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="F56" s="24" t="s">
+      <c r="C56" s="38"/>
+      <c r="D56" s="38"/>
+      <c r="F56" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="G56" s="24"/>
-      <c r="H56" s="24"/>
-      <c r="I56" s="24"/>
-      <c r="J56" s="24"/>
+      <c r="G56" s="37"/>
+      <c r="H56" s="37"/>
+      <c r="I56" s="37"/>
+      <c r="J56" s="37"/>
     </row>
     <row r="57" spans="2:10">
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
       <c r="D57" s="6"/>
-      <c r="F57" s="24" t="s">
+      <c r="F57" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="G57" s="24"/>
-      <c r="H57" s="24"/>
-      <c r="I57" s="24"/>
-      <c r="J57" s="24"/>
+      <c r="G57" s="37"/>
+      <c r="H57" s="37"/>
+      <c r="I57" s="37"/>
+      <c r="J57" s="37"/>
     </row>
     <row r="58" spans="2:10">
-      <c r="B58" s="26" t="s">
+      <c r="B58" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="26"/>
-      <c r="D58" s="26"/>
-      <c r="F58" s="24" t="s">
+      <c r="C58" s="38"/>
+      <c r="D58" s="38"/>
+      <c r="F58" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="G58" s="24"/>
-      <c r="H58" s="24"/>
-      <c r="I58" s="24"/>
-      <c r="J58" s="24"/>
+      <c r="G58" s="37"/>
+      <c r="H58" s="37"/>
+      <c r="I58" s="37"/>
+      <c r="J58" s="37"/>
     </row>
     <row r="59" spans="2:10">
-      <c r="B59" s="26" t="s">
+      <c r="B59" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="26"/>
-      <c r="D59" s="26"/>
-      <c r="F59" s="24" t="s">
+      <c r="C59" s="38"/>
+      <c r="D59" s="38"/>
+      <c r="F59" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="G59" s="24"/>
-      <c r="H59" s="24"/>
-      <c r="I59" s="24"/>
-      <c r="J59" s="24"/>
+      <c r="G59" s="37"/>
+      <c r="H59" s="37"/>
+      <c r="I59" s="37"/>
+      <c r="J59" s="37"/>
     </row>
     <row r="60" spans="2:10">
-      <c r="B60" s="26" t="s">
+      <c r="B60" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="26"/>
-      <c r="D60" s="26"/>
-      <c r="F60" s="23"/>
-      <c r="G60" s="23"/>
-      <c r="H60" s="23"/>
-      <c r="I60" s="23"/>
-      <c r="J60" s="23"/>
+      <c r="C60" s="38"/>
+      <c r="D60" s="38"/>
+      <c r="F60" s="35"/>
+      <c r="G60" s="35"/>
+      <c r="H60" s="35"/>
+      <c r="I60" s="35"/>
+      <c r="J60" s="35"/>
     </row>
     <row r="61" spans="2:10">
-      <c r="B61" s="26" t="s">
+      <c r="B61" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="26"/>
-      <c r="D61" s="26"/>
-      <c r="F61" s="23" t="s">
+      <c r="C61" s="38"/>
+      <c r="D61" s="38"/>
+      <c r="F61" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="G61" s="23"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="23"/>
-      <c r="J61" s="23"/>
+      <c r="G61" s="35"/>
+      <c r="H61" s="35"/>
+      <c r="I61" s="35"/>
+      <c r="J61" s="35"/>
     </row>
     <row r="62" spans="2:10">
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="26"/>
-      <c r="F62" s="24" t="s">
+      <c r="B62" s="38"/>
+      <c r="C62" s="38"/>
+      <c r="D62" s="38"/>
+      <c r="F62" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="G62" s="24"/>
-      <c r="H62" s="24"/>
-      <c r="I62" s="24"/>
-      <c r="J62" s="24"/>
+      <c r="G62" s="37"/>
+      <c r="H62" s="37"/>
+      <c r="I62" s="37"/>
+      <c r="J62" s="37"/>
     </row>
     <row r="63" spans="2:10">
-      <c r="B63" s="26" t="s">
+      <c r="B63" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="26"/>
-      <c r="D63" s="26"/>
-      <c r="F63" s="24" t="s">
+      <c r="C63" s="38"/>
+      <c r="D63" s="38"/>
+      <c r="F63" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="G63" s="24"/>
-      <c r="H63" s="24"/>
-      <c r="I63" s="24"/>
-      <c r="J63" s="24"/>
+      <c r="G63" s="37"/>
+      <c r="H63" s="37"/>
+      <c r="I63" s="37"/>
+      <c r="J63" s="37"/>
     </row>
     <row r="64" spans="2:10">
-      <c r="B64" s="26" t="s">
+      <c r="B64" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="26"/>
-      <c r="D64" s="26"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="23"/>
+      <c r="C64" s="38"/>
+      <c r="D64" s="38"/>
+      <c r="F64" s="35"/>
+      <c r="G64" s="35"/>
+      <c r="H64" s="35"/>
+      <c r="I64" s="35"/>
+      <c r="J64" s="35"/>
     </row>
     <row r="65" spans="2:10">
-      <c r="B65" s="26" t="s">
+      <c r="B65" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="26"/>
-      <c r="D65" s="26"/>
-      <c r="F65" s="23" t="s">
+      <c r="C65" s="38"/>
+      <c r="D65" s="38"/>
+      <c r="F65" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="G65" s="23"/>
-      <c r="H65" s="23"/>
-      <c r="I65" s="23"/>
-      <c r="J65" s="23"/>
+      <c r="G65" s="35"/>
+      <c r="H65" s="35"/>
+      <c r="I65" s="35"/>
+      <c r="J65" s="35"/>
     </row>
     <row r="66" spans="2:10">
-      <c r="B66" s="26" t="s">
+      <c r="B66" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="26"/>
-      <c r="D66" s="26"/>
-      <c r="F66" s="24" t="s">
+      <c r="C66" s="38"/>
+      <c r="D66" s="38"/>
+      <c r="F66" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="G66" s="24"/>
-      <c r="H66" s="24"/>
-      <c r="I66" s="24"/>
-      <c r="J66" s="24"/>
+      <c r="G66" s="37"/>
+      <c r="H66" s="37"/>
+      <c r="I66" s="37"/>
+      <c r="J66" s="37"/>
     </row>
     <row r="67" spans="2:10" ht="15" customHeight="1">
-      <c r="B67" s="26" t="s">
+      <c r="B67" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="C67" s="26"/>
-      <c r="D67" s="26"/>
-      <c r="F67" s="25" t="s">
+      <c r="C67" s="38"/>
+      <c r="D67" s="38"/>
+      <c r="F67" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="G67" s="25"/>
-      <c r="H67" s="25"/>
-      <c r="I67" s="25"/>
-      <c r="J67" s="25"/>
+      <c r="G67" s="39"/>
+      <c r="H67" s="39"/>
+      <c r="I67" s="39"/>
+      <c r="J67" s="39"/>
     </row>
     <row r="68" spans="2:10">
-      <c r="B68" s="26"/>
-      <c r="C68" s="26"/>
-      <c r="D68" s="26"/>
-      <c r="F68" s="25"/>
-      <c r="G68" s="25"/>
-      <c r="H68" s="25"/>
-      <c r="I68" s="25"/>
-      <c r="J68" s="25"/>
+      <c r="B68" s="38"/>
+      <c r="C68" s="38"/>
+      <c r="D68" s="38"/>
+      <c r="F68" s="39"/>
+      <c r="G68" s="39"/>
+      <c r="H68" s="39"/>
+      <c r="I68" s="39"/>
+      <c r="J68" s="39"/>
     </row>
     <row r="69" spans="2:10">
-      <c r="B69" s="26" t="s">
+      <c r="B69" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="C69" s="26"/>
-      <c r="D69" s="26"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="23"/>
-      <c r="H69" s="23"/>
-      <c r="I69" s="23"/>
-      <c r="J69" s="23"/>
+      <c r="C69" s="38"/>
+      <c r="D69" s="38"/>
+      <c r="F69" s="35"/>
+      <c r="G69" s="35"/>
+      <c r="H69" s="35"/>
+      <c r="I69" s="35"/>
+      <c r="J69" s="35"/>
     </row>
     <row r="70" spans="2:10">
-      <c r="B70" s="26" t="s">
+      <c r="B70" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="C70" s="26"/>
-      <c r="D70" s="26"/>
-      <c r="F70" s="23" t="s">
+      <c r="C70" s="38"/>
+      <c r="D70" s="38"/>
+      <c r="F70" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23"/>
-      <c r="I70" s="23"/>
-      <c r="J70" s="23"/>
+      <c r="G70" s="35"/>
+      <c r="H70" s="35"/>
+      <c r="I70" s="35"/>
+      <c r="J70" s="35"/>
     </row>
     <row r="71" spans="2:10">
-      <c r="F71" s="24" t="s">
+      <c r="F71" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="G71" s="24"/>
-      <c r="H71" s="24"/>
-      <c r="I71" s="24"/>
-      <c r="J71" s="24"/>
+      <c r="G71" s="37"/>
+      <c r="H71" s="37"/>
+      <c r="I71" s="37"/>
+      <c r="J71" s="37"/>
     </row>
     <row r="72" spans="2:10">
-      <c r="B72" s="27" t="s">
+      <c r="B72" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="C72" s="27"/>
-      <c r="D72" s="27"/>
-      <c r="F72" s="24" t="s">
+      <c r="C72" s="34"/>
+      <c r="D72" s="34"/>
+      <c r="F72" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="G72" s="24"/>
-      <c r="H72" s="24"/>
-      <c r="I72" s="24"/>
-      <c r="J72" s="24"/>
+      <c r="G72" s="37"/>
+      <c r="H72" s="37"/>
+      <c r="I72" s="37"/>
+      <c r="J72" s="37"/>
     </row>
     <row r="73" spans="2:10">
-      <c r="B73" s="26" t="s">
+      <c r="B73" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="C73" s="26"/>
-      <c r="D73" s="26"/>
-      <c r="F73" s="24" t="s">
+      <c r="C73" s="38"/>
+      <c r="D73" s="38"/>
+      <c r="F73" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="G73" s="24"/>
-      <c r="H73" s="24"/>
-      <c r="I73" s="24"/>
-      <c r="J73" s="24"/>
+      <c r="G73" s="37"/>
+      <c r="H73" s="37"/>
+      <c r="I73" s="37"/>
+      <c r="J73" s="37"/>
     </row>
     <row r="74" spans="2:10">
-      <c r="B74" s="26" t="s">
+      <c r="B74" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="C74" s="26"/>
-      <c r="D74" s="26"/>
+      <c r="C74" s="38"/>
+      <c r="D74" s="38"/>
     </row>
     <row r="75" spans="2:10">
       <c r="B75" s="6"/>
@@ -2455,71 +2455,82 @@
       <c r="D75" s="6"/>
     </row>
     <row r="76" spans="2:10">
-      <c r="B76" s="26" t="s">
+      <c r="B76" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="C76" s="26"/>
-      <c r="D76" s="26"/>
+      <c r="C76" s="38"/>
+      <c r="D76" s="38"/>
     </row>
     <row r="77" spans="2:10">
-      <c r="B77" s="26" t="s">
+      <c r="B77" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="C77" s="26"/>
-      <c r="D77" s="26"/>
+      <c r="C77" s="38"/>
+      <c r="D77" s="38"/>
     </row>
     <row r="78" spans="2:10">
-      <c r="B78" s="26" t="s">
+      <c r="B78" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
+      <c r="C78" s="38"/>
+      <c r="D78" s="38"/>
     </row>
     <row r="79" spans="2:10">
-      <c r="B79" s="26" t="s">
+      <c r="B79" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C79" s="26"/>
-      <c r="D79" s="26"/>
+      <c r="C79" s="38"/>
+      <c r="D79" s="38"/>
     </row>
     <row r="80" spans="2:10">
-      <c r="B80" s="26" t="s">
+      <c r="B80" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="C80" s="26"/>
-      <c r="D80" s="26"/>
+      <c r="C80" s="38"/>
+      <c r="D80" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="85">
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="F37:J37"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="F32:J32"/>
-    <mergeCell ref="F33:J33"/>
-    <mergeCell ref="F34:J34"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="F36:J36"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="B79:D79"/>
-    <mergeCell ref="B78:D78"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="F70:J70"/>
+    <mergeCell ref="F71:J71"/>
+    <mergeCell ref="F72:J72"/>
+    <mergeCell ref="F73:J73"/>
+    <mergeCell ref="F64:J64"/>
+    <mergeCell ref="F65:J65"/>
+    <mergeCell ref="F66:J66"/>
+    <mergeCell ref="F69:J69"/>
+    <mergeCell ref="F67:J68"/>
+    <mergeCell ref="F58:J58"/>
+    <mergeCell ref="F59:J59"/>
+    <mergeCell ref="F60:J60"/>
+    <mergeCell ref="F61:J61"/>
+    <mergeCell ref="F62:J62"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="F39:J39"/>
+    <mergeCell ref="F40:J40"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="F42:J42"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="F43:J43"/>
+    <mergeCell ref="F48:J52"/>
+    <mergeCell ref="F63:J63"/>
+    <mergeCell ref="F44:J44"/>
+    <mergeCell ref="F45:J45"/>
+    <mergeCell ref="F46:J46"/>
+    <mergeCell ref="F47:J47"/>
+    <mergeCell ref="F53:J53"/>
+    <mergeCell ref="F54:J54"/>
+    <mergeCell ref="F55:J55"/>
+    <mergeCell ref="F56:J56"/>
+    <mergeCell ref="F57:J57"/>
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B74:D74"/>
@@ -2536,46 +2547,35 @@
     <mergeCell ref="B63:D63"/>
     <mergeCell ref="B64:D64"/>
     <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="B67:D67"/>
-    <mergeCell ref="B68:D68"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="F43:J43"/>
-    <mergeCell ref="F48:J52"/>
-    <mergeCell ref="F63:J63"/>
-    <mergeCell ref="F44:J44"/>
-    <mergeCell ref="F45:J45"/>
-    <mergeCell ref="F46:J46"/>
-    <mergeCell ref="F47:J47"/>
-    <mergeCell ref="F53:J53"/>
-    <mergeCell ref="F54:J54"/>
-    <mergeCell ref="F55:J55"/>
-    <mergeCell ref="F56:J56"/>
-    <mergeCell ref="F57:J57"/>
-    <mergeCell ref="F38:J38"/>
-    <mergeCell ref="F39:J39"/>
-    <mergeCell ref="F40:J40"/>
-    <mergeCell ref="F41:J41"/>
-    <mergeCell ref="F42:J42"/>
-    <mergeCell ref="F58:J58"/>
-    <mergeCell ref="F59:J59"/>
-    <mergeCell ref="F60:J60"/>
-    <mergeCell ref="F61:J61"/>
-    <mergeCell ref="F62:J62"/>
-    <mergeCell ref="F70:J70"/>
-    <mergeCell ref="F71:J71"/>
-    <mergeCell ref="F72:J72"/>
-    <mergeCell ref="F73:J73"/>
-    <mergeCell ref="F64:J64"/>
-    <mergeCell ref="F65:J65"/>
-    <mergeCell ref="F66:J66"/>
-    <mergeCell ref="F69:J69"/>
-    <mergeCell ref="F67:J68"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A16:A20"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="B77:D77"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="F37:J37"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="F32:J32"/>
+    <mergeCell ref="F33:J33"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="F36:J36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge Front and Back
</commit_message>
<xml_diff>
--- a/backend/DB_DRAFT.xlsx
+++ b/backend/DB_DRAFT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gero2\source\repos\StoreFlow\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9014823B-8156-48B9-A6CE-39750B21B7FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979A7D55-9E11-4A24-BB25-D119D1D23169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4785" yWindow="4185" windowWidth="31755" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
+    <workbookView xWindow="40800" yWindow="690" windowWidth="24435" windowHeight="14010" xr2:uid="{291862C8-D710-4EB8-8BED-80BBEE43BFDA}"/>
   </bookViews>
   <sheets>
     <sheet name="OPERATIONS" sheetId="3" r:id="rId1"/>
@@ -792,7 +792,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -824,12 +824,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1" tint="0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF8585"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -946,7 +940,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -995,15 +989,6 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1012,9 +997,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1056,6 +1038,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1419,15 +1404,15 @@
       <c r="A1" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="B1" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="13" t="s">
@@ -1544,12 +1529,12 @@
       <c r="A7" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:8">
@@ -1628,29 +1613,29 @@
       <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="41" t="s">
+      <c r="A14" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="27" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="90">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="36" t="s">
         <v>129</v>
       </c>
       <c r="B16" s="19" t="s">
@@ -1664,7 +1649,7 @@
       </c>
     </row>
     <row r="17" spans="1:12">
-      <c r="A17" s="40"/>
+      <c r="A17" s="36"/>
       <c r="B17" s="19" t="s">
         <v>133</v>
       </c>
@@ -1676,88 +1661,88 @@
       </c>
     </row>
     <row r="18" spans="1:12" ht="78.75">
-      <c r="A18" s="40"/>
-      <c r="B18" s="22" t="s">
+      <c r="A18" s="36"/>
+      <c r="B18" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="21" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="45">
-      <c r="A19" s="40"/>
-      <c r="B19" s="22" t="s">
+      <c r="A19" s="36"/>
+      <c r="B19" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="21" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:12">
-      <c r="A20" s="40"/>
-      <c r="B20" s="25" t="s">
+      <c r="A20" s="36"/>
+      <c r="B20" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="C20" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="24" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="78.75">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="40" t="s">
         <v>135</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="21" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:12">
-      <c r="A22" s="40"/>
-      <c r="B22" s="28" t="s">
+      <c r="A22" s="36"/>
+      <c r="B22" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="21" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:12">
-      <c r="A23" s="40"/>
-      <c r="B23" s="29" t="s">
+      <c r="A23" s="36"/>
+      <c r="B23" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="C23" s="30" t="s">
+      <c r="C23" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="D23" s="24" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="40"/>
-      <c r="B24" s="29" t="s">
+      <c r="A24" s="36"/>
+      <c r="B24" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="C24" s="30" t="s">
+      <c r="C24" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="24" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1779,18 +1764,18 @@
       <c r="F28" s="1"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="F29" s="35" t="s">
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="F29" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
     </row>
     <row r="30" spans="1:12">
       <c r="B30" t="s">
@@ -1802,13 +1787,13 @@
       <c r="D30" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="35" t="s">
+      <c r="F30" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="G30" s="35"/>
-      <c r="H30" s="35"/>
-      <c r="I30" s="35"/>
-      <c r="J30" s="35"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
     </row>
     <row r="31" spans="1:12">
       <c r="B31" s="5" t="s">
@@ -1820,17 +1805,17 @@
       <c r="D31" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="37" t="s">
+      <c r="F31" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="G31" s="37"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="37"/>
-      <c r="J31" s="37"/>
-      <c r="K31" s="32" t="s">
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="L31" s="33"/>
+      <c r="L31" s="29"/>
     </row>
     <row r="32" spans="1:12">
       <c r="B32" s="5" t="s">
@@ -1842,13 +1827,13 @@
       <c r="D32" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="37" t="s">
+      <c r="F32" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="G32" s="37"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="37"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
+      <c r="I32" s="33"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="11" t="s">
         <v>105</v>
       </c>
@@ -1866,13 +1851,13 @@
       <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="37" t="s">
+      <c r="F33" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="37"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="33"/>
+      <c r="I33" s="33"/>
+      <c r="J33" s="33"/>
       <c r="K33" s="9" t="s">
         <v>107</v>
       </c>
@@ -1890,13 +1875,13 @@
       <c r="D34" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F34" s="37" t="s">
+      <c r="F34" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="G34" s="37"/>
-      <c r="H34" s="37"/>
-      <c r="I34" s="37"/>
-      <c r="J34" s="37"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
+      <c r="I34" s="33"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="9" t="s">
         <v>108</v>
       </c>
@@ -1914,13 +1899,13 @@
       <c r="D35" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F35" s="37" t="s">
+      <c r="F35" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="37"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="33"/>
+      <c r="J35" s="33"/>
       <c r="K35" s="9" t="s">
         <v>109</v>
       </c>
@@ -1930,11 +1915,11 @@
     </row>
     <row r="36" spans="2:12">
       <c r="D36" s="5"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="35"/>
-      <c r="I36" s="35"/>
-      <c r="J36" s="35"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="31"/>
       <c r="K36" s="9" t="s">
         <v>110</v>
       </c>
@@ -1943,18 +1928,18 @@
       </c>
     </row>
     <row r="37" spans="2:12">
-      <c r="B37" s="34" t="s">
+      <c r="B37" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="34"/>
-      <c r="D37" s="34"/>
-      <c r="F37" s="35" t="s">
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
+      <c r="F37" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="35"/>
-      <c r="J37" s="35"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="31"/>
       <c r="K37" s="9" t="s">
         <v>112</v>
       </c>
@@ -1963,18 +1948,18 @@
       </c>
     </row>
     <row r="38" spans="2:12">
-      <c r="B38" s="38" t="s">
+      <c r="B38" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="38"/>
-      <c r="D38" s="38"/>
-      <c r="F38" s="37" t="s">
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="F38" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="G38" s="37"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="37"/>
-      <c r="J38" s="37"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="33"/>
+      <c r="I38" s="33"/>
+      <c r="J38" s="33"/>
       <c r="K38" s="9" t="s">
         <v>114</v>
       </c>
@@ -1983,18 +1968,18 @@
       </c>
     </row>
     <row r="39" spans="2:12">
-      <c r="B39" s="38" t="s">
+      <c r="B39" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="38"/>
-      <c r="D39" s="38"/>
-      <c r="F39" s="37" t="s">
+      <c r="C39" s="34"/>
+      <c r="D39" s="34"/>
+      <c r="F39" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37"/>
-      <c r="I39" s="37"/>
-      <c r="J39" s="37"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
       <c r="K39" s="9" t="s">
         <v>116</v>
       </c>
@@ -2003,16 +1988,16 @@
       </c>
     </row>
     <row r="40" spans="2:12">
-      <c r="B40" s="38" t="s">
+      <c r="B40" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="35"/>
-      <c r="J40" s="35"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="34"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="31"/>
+      <c r="J40" s="31"/>
       <c r="K40" s="10" t="s">
         <v>118</v>
       </c>
@@ -2021,433 +2006,433 @@
       </c>
     </row>
     <row r="41" spans="2:12">
-      <c r="B41" s="38" t="s">
+      <c r="B41" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="F41" s="35" t="s">
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+      <c r="F41" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="G41" s="35"/>
-      <c r="H41" s="35"/>
-      <c r="I41" s="35"/>
-      <c r="J41" s="35"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="31"/>
+      <c r="J41" s="31"/>
     </row>
     <row r="42" spans="2:12">
-      <c r="F42" s="37" t="s">
+      <c r="F42" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="G42" s="37"/>
-      <c r="H42" s="37"/>
-      <c r="I42" s="37"/>
-      <c r="J42" s="37"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="33"/>
     </row>
     <row r="43" spans="2:12">
-      <c r="B43" s="34" t="s">
+      <c r="B43" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C43" s="34"/>
-      <c r="D43" s="34"/>
-      <c r="F43" s="37" t="s">
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="F43" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="G43" s="37"/>
-      <c r="H43" s="37"/>
-      <c r="I43" s="37"/>
-      <c r="J43" s="37"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="33"/>
     </row>
     <row r="44" spans="2:12">
-      <c r="B44" s="38" t="s">
+      <c r="B44" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="38"/>
-      <c r="D44" s="38"/>
-      <c r="F44" s="37" t="s">
+      <c r="C44" s="34"/>
+      <c r="D44" s="34"/>
+      <c r="F44" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="G44" s="37"/>
-      <c r="H44" s="37"/>
-      <c r="I44" s="37"/>
-      <c r="J44" s="37"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="33"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
     </row>
     <row r="45" spans="2:12">
-      <c r="B45" s="38" t="s">
+      <c r="B45" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="38"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="H45" s="35"/>
-      <c r="I45" s="35"/>
-      <c r="J45" s="35"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="F45" s="31"/>
+      <c r="G45" s="31"/>
+      <c r="H45" s="31"/>
+      <c r="I45" s="31"/>
+      <c r="J45" s="31"/>
     </row>
     <row r="46" spans="2:12">
-      <c r="B46" s="38" t="s">
+      <c r="B46" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C46" s="38"/>
-      <c r="D46" s="38"/>
-      <c r="F46" s="35" t="s">
+      <c r="C46" s="34"/>
+      <c r="D46" s="34"/>
+      <c r="F46" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
-      <c r="J46" s="35"/>
+      <c r="G46" s="31"/>
+      <c r="H46" s="31"/>
+      <c r="I46" s="31"/>
+      <c r="J46" s="31"/>
     </row>
     <row r="47" spans="2:12">
-      <c r="B47" s="38" t="s">
+      <c r="B47" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="C47" s="38"/>
-      <c r="D47" s="38"/>
-      <c r="F47" s="37" t="s">
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+      <c r="F47" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="37"/>
-      <c r="J47" s="37"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
     </row>
     <row r="48" spans="2:12" ht="15" customHeight="1">
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
-      <c r="F48" s="39" t="s">
+      <c r="F48" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="G48" s="39"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="39"/>
-      <c r="J48" s="39"/>
+      <c r="G48" s="35"/>
+      <c r="H48" s="35"/>
+      <c r="I48" s="35"/>
+      <c r="J48" s="35"/>
     </row>
     <row r="49" spans="2:10">
-      <c r="B49" s="38" t="s">
+      <c r="B49" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="38"/>
-      <c r="D49" s="38"/>
-      <c r="F49" s="39"/>
-      <c r="G49" s="39"/>
-      <c r="H49" s="39"/>
-      <c r="I49" s="39"/>
-      <c r="J49" s="39"/>
+      <c r="C49" s="34"/>
+      <c r="D49" s="34"/>
+      <c r="F49" s="35"/>
+      <c r="G49" s="35"/>
+      <c r="H49" s="35"/>
+      <c r="I49" s="35"/>
+      <c r="J49" s="35"/>
     </row>
     <row r="50" spans="2:10">
-      <c r="B50" s="38" t="s">
+      <c r="B50" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="C50" s="38"/>
-      <c r="D50" s="38"/>
-      <c r="F50" s="39"/>
-      <c r="G50" s="39"/>
-      <c r="H50" s="39"/>
-      <c r="I50" s="39"/>
-      <c r="J50" s="39"/>
+      <c r="C50" s="34"/>
+      <c r="D50" s="34"/>
+      <c r="F50" s="35"/>
+      <c r="G50" s="35"/>
+      <c r="H50" s="35"/>
+      <c r="I50" s="35"/>
+      <c r="J50" s="35"/>
     </row>
     <row r="51" spans="2:10">
-      <c r="B51" s="38" t="s">
+      <c r="B51" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="C51" s="38"/>
-      <c r="D51" s="38"/>
-      <c r="F51" s="39"/>
-      <c r="G51" s="39"/>
-      <c r="H51" s="39"/>
-      <c r="I51" s="39"/>
-      <c r="J51" s="39"/>
+      <c r="C51" s="34"/>
+      <c r="D51" s="34"/>
+      <c r="F51" s="35"/>
+      <c r="G51" s="35"/>
+      <c r="H51" s="35"/>
+      <c r="I51" s="35"/>
+      <c r="J51" s="35"/>
     </row>
     <row r="52" spans="2:10">
-      <c r="B52" s="38" t="s">
+      <c r="B52" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C52" s="38"/>
-      <c r="D52" s="38"/>
-      <c r="F52" s="39"/>
-      <c r="G52" s="39"/>
-      <c r="H52" s="39"/>
-      <c r="I52" s="39"/>
-      <c r="J52" s="39"/>
+      <c r="C52" s="34"/>
+      <c r="D52" s="34"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="35"/>
+      <c r="I52" s="35"/>
+      <c r="J52" s="35"/>
     </row>
     <row r="53" spans="2:10">
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
       <c r="D53" s="6"/>
-      <c r="F53" s="35"/>
-      <c r="G53" s="35"/>
-      <c r="H53" s="35"/>
-      <c r="I53" s="35"/>
-      <c r="J53" s="35"/>
+      <c r="F53" s="31"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="31"/>
+      <c r="I53" s="31"/>
+      <c r="J53" s="31"/>
     </row>
     <row r="54" spans="2:10">
-      <c r="B54" s="38" t="s">
+      <c r="B54" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C54" s="38"/>
-      <c r="D54" s="38"/>
-      <c r="F54" s="35" t="s">
+      <c r="C54" s="34"/>
+      <c r="D54" s="34"/>
+      <c r="F54" s="31" t="s">
         <v>81</v>
       </c>
-      <c r="G54" s="35"/>
-      <c r="H54" s="35"/>
-      <c r="I54" s="35"/>
-      <c r="J54" s="35"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="31"/>
+      <c r="J54" s="31"/>
     </row>
     <row r="55" spans="2:10">
-      <c r="B55" s="38" t="s">
+      <c r="B55" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="F55" s="37" t="s">
+      <c r="C55" s="34"/>
+      <c r="D55" s="34"/>
+      <c r="F55" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="G55" s="37"/>
-      <c r="H55" s="37"/>
-      <c r="I55" s="37"/>
-      <c r="J55" s="37"/>
+      <c r="G55" s="33"/>
+      <c r="H55" s="33"/>
+      <c r="I55" s="33"/>
+      <c r="J55" s="33"/>
     </row>
     <row r="56" spans="2:10">
-      <c r="B56" s="38" t="s">
+      <c r="B56" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="C56" s="38"/>
-      <c r="D56" s="38"/>
-      <c r="F56" s="37" t="s">
+      <c r="C56" s="34"/>
+      <c r="D56" s="34"/>
+      <c r="F56" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="G56" s="37"/>
-      <c r="H56" s="37"/>
-      <c r="I56" s="37"/>
-      <c r="J56" s="37"/>
+      <c r="G56" s="33"/>
+      <c r="H56" s="33"/>
+      <c r="I56" s="33"/>
+      <c r="J56" s="33"/>
     </row>
     <row r="57" spans="2:10">
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
       <c r="D57" s="6"/>
-      <c r="F57" s="37" t="s">
+      <c r="F57" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="G57" s="37"/>
-      <c r="H57" s="37"/>
-      <c r="I57" s="37"/>
-      <c r="J57" s="37"/>
+      <c r="G57" s="33"/>
+      <c r="H57" s="33"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
     </row>
     <row r="58" spans="2:10">
-      <c r="B58" s="38" t="s">
+      <c r="B58" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="C58" s="38"/>
-      <c r="D58" s="38"/>
-      <c r="F58" s="37" t="s">
+      <c r="C58" s="34"/>
+      <c r="D58" s="34"/>
+      <c r="F58" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="G58" s="37"/>
-      <c r="H58" s="37"/>
-      <c r="I58" s="37"/>
-      <c r="J58" s="37"/>
+      <c r="G58" s="33"/>
+      <c r="H58" s="33"/>
+      <c r="I58" s="33"/>
+      <c r="J58" s="33"/>
     </row>
     <row r="59" spans="2:10">
-      <c r="B59" s="38" t="s">
+      <c r="B59" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="C59" s="38"/>
-      <c r="D59" s="38"/>
-      <c r="F59" s="37" t="s">
+      <c r="C59" s="34"/>
+      <c r="D59" s="34"/>
+      <c r="F59" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="G59" s="37"/>
-      <c r="H59" s="37"/>
-      <c r="I59" s="37"/>
-      <c r="J59" s="37"/>
+      <c r="G59" s="33"/>
+      <c r="H59" s="33"/>
+      <c r="I59" s="33"/>
+      <c r="J59" s="33"/>
     </row>
     <row r="60" spans="2:10">
-      <c r="B60" s="38" t="s">
+      <c r="B60" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="C60" s="38"/>
-      <c r="D60" s="38"/>
-      <c r="F60" s="35"/>
-      <c r="G60" s="35"/>
-      <c r="H60" s="35"/>
-      <c r="I60" s="35"/>
-      <c r="J60" s="35"/>
+      <c r="C60" s="34"/>
+      <c r="D60" s="34"/>
+      <c r="F60" s="31"/>
+      <c r="G60" s="31"/>
+      <c r="H60" s="31"/>
+      <c r="I60" s="31"/>
+      <c r="J60" s="31"/>
     </row>
     <row r="61" spans="2:10">
-      <c r="B61" s="38" t="s">
+      <c r="B61" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C61" s="38"/>
-      <c r="D61" s="38"/>
-      <c r="F61" s="35" t="s">
+      <c r="C61" s="34"/>
+      <c r="D61" s="34"/>
+      <c r="F61" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="G61" s="35"/>
-      <c r="H61" s="35"/>
-      <c r="I61" s="35"/>
-      <c r="J61" s="35"/>
+      <c r="G61" s="31"/>
+      <c r="H61" s="31"/>
+      <c r="I61" s="31"/>
+      <c r="J61" s="31"/>
     </row>
     <row r="62" spans="2:10">
-      <c r="B62" s="38"/>
-      <c r="C62" s="38"/>
-      <c r="D62" s="38"/>
-      <c r="F62" s="37" t="s">
+      <c r="B62" s="34"/>
+      <c r="C62" s="34"/>
+      <c r="D62" s="34"/>
+      <c r="F62" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="G62" s="37"/>
-      <c r="H62" s="37"/>
-      <c r="I62" s="37"/>
-      <c r="J62" s="37"/>
+      <c r="G62" s="33"/>
+      <c r="H62" s="33"/>
+      <c r="I62" s="33"/>
+      <c r="J62" s="33"/>
     </row>
     <row r="63" spans="2:10">
-      <c r="B63" s="38" t="s">
+      <c r="B63" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="38"/>
-      <c r="D63" s="38"/>
-      <c r="F63" s="37" t="s">
+      <c r="C63" s="34"/>
+      <c r="D63" s="34"/>
+      <c r="F63" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="G63" s="37"/>
-      <c r="H63" s="37"/>
-      <c r="I63" s="37"/>
-      <c r="J63" s="37"/>
+      <c r="G63" s="33"/>
+      <c r="H63" s="33"/>
+      <c r="I63" s="33"/>
+      <c r="J63" s="33"/>
     </row>
     <row r="64" spans="2:10">
-      <c r="B64" s="38" t="s">
+      <c r="B64" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="C64" s="38"/>
-      <c r="D64" s="38"/>
-      <c r="F64" s="35"/>
-      <c r="G64" s="35"/>
-      <c r="H64" s="35"/>
-      <c r="I64" s="35"/>
-      <c r="J64" s="35"/>
+      <c r="C64" s="34"/>
+      <c r="D64" s="34"/>
+      <c r="F64" s="31"/>
+      <c r="G64" s="31"/>
+      <c r="H64" s="31"/>
+      <c r="I64" s="31"/>
+      <c r="J64" s="31"/>
     </row>
     <row r="65" spans="2:10">
-      <c r="B65" s="38" t="s">
+      <c r="B65" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="38"/>
-      <c r="D65" s="38"/>
-      <c r="F65" s="35" t="s">
+      <c r="C65" s="34"/>
+      <c r="D65" s="34"/>
+      <c r="F65" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="G65" s="35"/>
-      <c r="H65" s="35"/>
-      <c r="I65" s="35"/>
-      <c r="J65" s="35"/>
+      <c r="G65" s="31"/>
+      <c r="H65" s="31"/>
+      <c r="I65" s="31"/>
+      <c r="J65" s="31"/>
     </row>
     <row r="66" spans="2:10">
-      <c r="B66" s="38" t="s">
+      <c r="B66" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="38"/>
-      <c r="D66" s="38"/>
-      <c r="F66" s="37" t="s">
+      <c r="C66" s="34"/>
+      <c r="D66" s="34"/>
+      <c r="F66" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="G66" s="37"/>
-      <c r="H66" s="37"/>
-      <c r="I66" s="37"/>
-      <c r="J66" s="37"/>
+      <c r="G66" s="33"/>
+      <c r="H66" s="33"/>
+      <c r="I66" s="33"/>
+      <c r="J66" s="33"/>
     </row>
     <row r="67" spans="2:10" ht="15" customHeight="1">
-      <c r="B67" s="38" t="s">
+      <c r="B67" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="C67" s="38"/>
-      <c r="D67" s="38"/>
-      <c r="F67" s="39" t="s">
+      <c r="C67" s="34"/>
+      <c r="D67" s="34"/>
+      <c r="F67" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="G67" s="39"/>
-      <c r="H67" s="39"/>
-      <c r="I67" s="39"/>
-      <c r="J67" s="39"/>
+      <c r="G67" s="35"/>
+      <c r="H67" s="35"/>
+      <c r="I67" s="35"/>
+      <c r="J67" s="35"/>
     </row>
     <row r="68" spans="2:10">
-      <c r="B68" s="38"/>
-      <c r="C68" s="38"/>
-      <c r="D68" s="38"/>
-      <c r="F68" s="39"/>
-      <c r="G68" s="39"/>
-      <c r="H68" s="39"/>
-      <c r="I68" s="39"/>
-      <c r="J68" s="39"/>
+      <c r="B68" s="34"/>
+      <c r="C68" s="34"/>
+      <c r="D68" s="34"/>
+      <c r="F68" s="35"/>
+      <c r="G68" s="35"/>
+      <c r="H68" s="35"/>
+      <c r="I68" s="35"/>
+      <c r="J68" s="35"/>
     </row>
     <row r="69" spans="2:10">
-      <c r="B69" s="38" t="s">
+      <c r="B69" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="C69" s="38"/>
-      <c r="D69" s="38"/>
-      <c r="F69" s="35"/>
-      <c r="G69" s="35"/>
-      <c r="H69" s="35"/>
-      <c r="I69" s="35"/>
-      <c r="J69" s="35"/>
+      <c r="C69" s="34"/>
+      <c r="D69" s="34"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+      <c r="I69" s="31"/>
+      <c r="J69" s="31"/>
     </row>
     <row r="70" spans="2:10">
-      <c r="B70" s="38" t="s">
+      <c r="B70" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="C70" s="38"/>
-      <c r="D70" s="38"/>
-      <c r="F70" s="35" t="s">
+      <c r="C70" s="34"/>
+      <c r="D70" s="34"/>
+      <c r="F70" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="G70" s="35"/>
-      <c r="H70" s="35"/>
-      <c r="I70" s="35"/>
-      <c r="J70" s="35"/>
+      <c r="G70" s="31"/>
+      <c r="H70" s="31"/>
+      <c r="I70" s="31"/>
+      <c r="J70" s="31"/>
     </row>
     <row r="71" spans="2:10">
-      <c r="F71" s="37" t="s">
+      <c r="F71" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="G71" s="37"/>
-      <c r="H71" s="37"/>
-      <c r="I71" s="37"/>
-      <c r="J71" s="37"/>
+      <c r="G71" s="33"/>
+      <c r="H71" s="33"/>
+      <c r="I71" s="33"/>
+      <c r="J71" s="33"/>
     </row>
     <row r="72" spans="2:10">
-      <c r="B72" s="34" t="s">
+      <c r="B72" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="C72" s="34"/>
-      <c r="D72" s="34"/>
-      <c r="F72" s="37" t="s">
+      <c r="C72" s="30"/>
+      <c r="D72" s="30"/>
+      <c r="F72" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="G72" s="37"/>
-      <c r="H72" s="37"/>
-      <c r="I72" s="37"/>
-      <c r="J72" s="37"/>
+      <c r="G72" s="33"/>
+      <c r="H72" s="33"/>
+      <c r="I72" s="33"/>
+      <c r="J72" s="33"/>
     </row>
     <row r="73" spans="2:10">
-      <c r="B73" s="38" t="s">
+      <c r="B73" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="C73" s="38"/>
-      <c r="D73" s="38"/>
-      <c r="F73" s="37" t="s">
+      <c r="C73" s="34"/>
+      <c r="D73" s="34"/>
+      <c r="F73" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="G73" s="37"/>
-      <c r="H73" s="37"/>
-      <c r="I73" s="37"/>
-      <c r="J73" s="37"/>
+      <c r="G73" s="33"/>
+      <c r="H73" s="33"/>
+      <c r="I73" s="33"/>
+      <c r="J73" s="33"/>
     </row>
     <row r="74" spans="2:10">
-      <c r="B74" s="38" t="s">
+      <c r="B74" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="C74" s="38"/>
-      <c r="D74" s="38"/>
+      <c r="C74" s="34"/>
+      <c r="D74" s="34"/>
     </row>
     <row r="75" spans="2:10">
       <c r="B75" s="6"/>
@@ -2455,39 +2440,39 @@
       <c r="D75" s="6"/>
     </row>
     <row r="76" spans="2:10">
-      <c r="B76" s="38" t="s">
+      <c r="B76" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="C76" s="38"/>
-      <c r="D76" s="38"/>
+      <c r="C76" s="34"/>
+      <c r="D76" s="34"/>
     </row>
     <row r="77" spans="2:10">
-      <c r="B77" s="38" t="s">
+      <c r="B77" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="C77" s="38"/>
-      <c r="D77" s="38"/>
+      <c r="C77" s="34"/>
+      <c r="D77" s="34"/>
     </row>
     <row r="78" spans="2:10">
-      <c r="B78" s="38" t="s">
+      <c r="B78" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="C78" s="38"/>
-      <c r="D78" s="38"/>
+      <c r="C78" s="34"/>
+      <c r="D78" s="34"/>
     </row>
     <row r="79" spans="2:10">
-      <c r="B79" s="38" t="s">
+      <c r="B79" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="C79" s="38"/>
-      <c r="D79" s="38"/>
+      <c r="C79" s="34"/>
+      <c r="D79" s="34"/>
     </row>
     <row r="80" spans="2:10">
-      <c r="B80" s="38" t="s">
+      <c r="B80" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="C80" s="38"/>
-      <c r="D80" s="38"/>
+      <c r="C80" s="34"/>
+      <c r="D80" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="85">

</xml_diff>